<commit_message>
after analyzer structure change - requires improvment
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,27 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A4FBEA-5140-4840-BC18-3E5E251AB18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC03644-A9C4-41C7-AC93-92BA8928AC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Tasks" sheetId="12" r:id="rId1"/>
     <sheet name="פרטי משתמש" sheetId="3" r:id="rId2"/>
     <sheet name="מאפיינים - כללי" sheetId="1" r:id="rId3"/>
-    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId4"/>
-    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId5"/>
-    <sheet name="בניית ציונים" sheetId="9" r:id="rId6"/>
-    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId7"/>
-    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId8"/>
-    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId9"/>
-    <sheet name="טופס הזנה" sheetId="8" r:id="rId10"/>
-    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId11"/>
-    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId12"/>
-    <sheet name="בדיקות" sheetId="13" r:id="rId13"/>
+    <sheet name="internal traits" sheetId="14" r:id="rId4"/>
+    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId5"/>
+    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId6"/>
+    <sheet name="בניית ציונים" sheetId="9" r:id="rId7"/>
+    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId8"/>
+    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId9"/>
+    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId10"/>
+    <sheet name="טופס הזנה" sheetId="8" r:id="rId11"/>
+    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId12"/>
+    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId13"/>
+    <sheet name="בדיקות" sheetId="13" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="613">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3201,12 +3201,628 @@
 אם לאחר השיחה לא התקבלה שום הצהרה מפורשת —
 יש להניח שאין מידע רלוונטי, ולא להסיק דבר</t>
   </si>
+  <si>
+    <t>סקאלת ציונים</t>
+  </si>
+  <si>
+    <t>הסבר כללי</t>
+  </si>
+  <si>
+    <t>מה כן נחשב סיגנל</t>
+  </si>
+  <si>
+    <t>התבסס על:
+- השכלה פורמלית (תואר, תחום לימודים)
+- סוג המקצוע
+- רמת מומחיות או בכירות
+- תחום עיסוק (למשל: הייטק, רפואה, הנדסה וכו')
+- תיאורים של הקריירה או המסלול המקצועי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+הבחנות חשובות:
+- מדובר ביתרונות פוטנציאליים בלבד — לא בהכרח יתרון עבור כולם
+- יש להחזיר רק מאפיינים ברורים ומשמעותיים
+- אין להוסיף פריטים שלא מופיעים ברשימה
+- אין לנחש או להסיק ללא בסיס ברור</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+התבסס על מידע מפורש שהמשתמש נתן במהלך השיחה.</t>
+  </si>
+  <si>
+    <t>זיהוי יתרונות פוטנציאליים.
+אין לתת ציון.
+יש להחזיר:
+1. רשימה של יתרונות מתוך רשימה מוגדרת בלבד
+2. תיאור טקסטואלי קצר (אם יש מה להוסיף)
+רשימת יתרונות אפשריים:
+- has_pets (יש לו בעל חיים)
+- has_children (יש ילדים)
+- divorced (גרוש/ה)
+- plays_music (מנגן)
+- into_fitness (עוסק בבריאות וכושר)
+- high_income (הכנסה גבוהה)
+- high_education (השכלה גבוהה)
+חוקים:
+- אם זוהה מאפיין אחד מהרשימה באופן ברור → יש להחזיר אותו (גם אם זה היחיד)
+- אין צורך ביותר ממאפיין אחד — גם אחד מספיק
+- אם אין אינדיקציה ברורה → להחזיר ריק
+- אין להחזיר ערכים על בסיס השערה</t>
+  </si>
+  <si>
+    <t>נחמדות / חום / חברותיות ≠ אינטליגנציה רגשית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הבחנות </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- עד כמה תחומי העניין שלו מיינסטרים או שגרתיים
+- עד כמה הדעות שלו נפוצות ונורמטיביות
+- עד כמה הוא "זורם עם מה שמקובל" לעומת חשיבה עצמאית
+- עד כמה הוא פתוח לסגנונות חיים לא שגרתיים (זוגיות, קריירה, אורח חיים)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- רגישות ≠ חוסר יציבות  
+  אדם יכול להיות רגיש אך יציב.
+- עומק רגשי ≠ חוסר יציבות  
+  אדם עמוק רגשית לא בהכרח נוטה לדרמה, דיכאון או קיצוניות.
+</t>
+  </si>
+  <si>
+    <t>לא מדובר ברצון להקים משפחה וילדים משלו, אלא במידת הקרבה, המעורבות והמרכזיות של משפחת המוצא בחיים בפועל.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- אדם יכול ליהנות ממסיבות אך לא להיות טיפוס מסיבתי  
+- התכונה מודדת סגנון חיים, לא העדפה נקודתית  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- תדירות יציאה למסיבות / חיי לילה
+- עד כמה זה חלק קבוע מהשגרה
+- זיקה לליינים, מועדונים, סצנה
+- סוג הסביבה החברתית (חיי לילה לעומת בילויים אחרים)
+- שפה שמעידה על סגנון חיים מסיבתי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- מידת הקרבה להורים ולמשפחה 
+- עד כמה המשפחה נוכחת בשגרה
+- עד כמה המשפחה משפיעה על החלטות, סדרי עדיפויות ואורח חיים
+- עד כמה המשתמש רואה במשפחתיות חלק מרכזי מחייו, לעומת רצון בחיים נפרדים ועצמאיים יותר</t>
+  </si>
+  <si>
+    <t>הערכת מופנמות / מוחצנות כסגנון ביטוי.
+התכונה מודדת את סגנון הביטוי והנוכחות של המשתמש — עד כמה הוא אקספרסיבי, מוחצן ותופס מקום, לעומת שקט, רגוע ומופנם.
+ציון גבוה = סגנון מוחצן (אקספרסיבי)
+ציון נמוך = סגנון מופנם (שקט)
+חוקים:
+- אם המשתמש נשמע שקט, מאופק או מינימליסטי בביטוי → הורד ציון
+- אם המשתמש נשמע אקספרסיבי, פתוח, יוזם ודומיננטי → העלה ציון</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- סגנון הדיבור (ישיר, פתוח, מרובה לעומת מדוד ושקט)
+- רמת האקספרסיביות (כמה מבטא את עצמו כלפי חוץ)
+- "ווליום" אנרגטי — מורגש, דומיננטי, יוזם לעומת שקט ונוכח בעדינות
+- עד כמה נראה שהוא תופס מקום חברתית לעומת משתלב ברקע
+- קצב ואופי הביטוי (מהיר/זורם/יוזם לעומת רגוע/מאופק)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- זה לא מודד צורך חברתי — אדם יכול להיות מופנם מאוד ועדיין מאוד אוהב אנשים  
+- זה לא מודד נהנתנות  
+- זה לא מודד אינטליגנציה חברתית  
+- מדובר בסגנון נוכחות וביטוי בלבד
+- לא להסיק מוחצנות רק מזה שהוא אוהב אנשים או בילויים</t>
+  </si>
+  <si>
+    <t>:
+-לא מדובר במסיבות דווקא — זה כולל כל סוג של בילוי וחוויה
+- לא למדוד כאן מוחצנות — אדם יכול להיות מופנם ונהנתן
+- לא למדוד כאן רק אמירות כלליות — חשוב גם ביטוי בפועל</t>
+  </si>
+  <si>
+    <t>הערכת מודעות עצמית
+עד כמה המשתמש מבין את עצמו — רגשות, דפוסים, חוזקות וחולשות — ויכול לדבר עליהם בצורה מודעת..
+- אם אין רפלקציה אישית ברורה → לא לתת ציון גבוה
+- אם יש תיאור עצמי עמוק או מודע → העלה ציון</t>
+  </si>
+  <si>
+    <t>:
+- ניסוח יפה ≠ מודעות עצמית
+- ניתוח כללי ≠ הבנה של עצמי</t>
+  </si>
+  <si>
+    <t>הערכת חשיבות והזדהות עם הומור
+עד כמה הומור הוא חלק מהזהות של המשתמש ועד כמה הוא חשוב לו — הן אצל עצמו והן אצל בן/בת זוג.
+לא מדובר בניסיון למדוד עד כמה המשתמש באמת מצחיק, אלא עד כמה הומור הוא ערך או מאפיין מרכזי עבורו.
+חוקים:
+- אם המשתמש מצהיר שחוש הומור חשוב לו → העלה ציון
+- אם המשתמש מציג את עצמו כאדם עם חוש הומור → העלה ציון
+- אם הומור מוזכר כמה פעמים או בהדגשה → העלה ציון משמעותית</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- אמירות ישירות ("יש לי חוש הומור", "אני מאוד ציני", "חשוב לי הומור")
+- הדגשה של הומור כמרכיב חשוב בזוגיות
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- עד כמה המשתמש מתעניין או עוסק בפוליטיקה
+- עד כמה פוליטיקה היא חלק מהשיח שלו
+- עד כמה הוא מבטא דעות פוליטיות באופן ברור
+- עד כמה הנושא תופס מקום בחיים ובזהות שלו</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר ביציבות רגשית  
+  אדם יכול להיות יציב אך שלילי  
+- לא מדובר בעומק או אינטליגנציה  
+- לא מדובר בקלילות בלבד  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- סגנון התקשורת (חם, נעים, מפרגן לעומת קר או ענייני)
+- שימוש במחמאות או שפה חיובית כלפי אחרים
+- תחושת קרבה, רכות או פתיחות בין-אישית
+- עד כמה המשתמש משדר "לב טוב" ויחס אוהב</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר בכמות אינטראקציות (זה חברתיות)
+- לא מדובר באופטימיות כללית (זה גישה חיובית)
+- לא מדובר באינטליגנציה רגשית
+- אדם יכול להיות מופנם ועדיין מאוד לבבי
+- אדם יכול להיות מוחצן אך לא לבבי</t>
+  </si>
+  <si>
+    <t>הערכת פתיחות (Openness).
+עד כמה המשתמש פתוח לרעיונות, חוויות וסגנונות חיים שונים — ועד כמה הוא נמשך אקטיבית להתנסות ולחוות דברים חדשים, גם אם הם מחוץ לאזור הנוחות.
+ חשוב למדוד גם פתיחות מחשבתית וגם פתיחות חווייתית בפועל
+חוקים:
+- אם המשתמש מבטא רצון לחוות, להתנסות או לחפש חוויות → העלה ציון- אם המשתמש מבטא קבלה או סקרנות כלפי סגנונות חיים שונים → העלה ציון
+- אם המשתמש מבטא הסתייגות משונות או היצמדות למה שמוכר → הורד ציון</t>
+  </si>
+  <si>
+    <t>:
+-  לא מדובר בפתיחות רגשית
+- לא מדובר באינטלקטואליות (עומק שיח)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר באחריות או בגרות תפקודית  
+- אדם יכול להיות מאוד אחראי וחכם אך עם וייב ילדותי  
+- לא מדובר באינטליגנציה או עומק  
+- לא מדובר ברצינות לחיים  
+- לא להסיק ילדותיות מחוסר אחריות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+הבחנות חשובות:
+- לא מדובר בפוליטיקה או עמדות ספציפיות
+- לא להסיק מהזכרת ישראל בלבד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- אמירות פוליטיות מפורשות
+- הזדהות עם מחנות או עמדות
+- רמזים עקיפים אך ברורים לעמדות פוליטיות
+- נושאים ערכיים עם זיקה פוליטית ברורה
+ - פעילות בארגון בעל זיהוי פוליטי/מחאתי היא סיגנל חזק
+- ביקורת על הממשלה או תמיכה בממשלה תהווה סיגנל ברור</t>
+  </si>
+  <si>
+    <t>הערכת מוסר עבודה
+עד כמה המשתמש רציני, מחויב ומשקיע בעבודה או בעשייה שלו — ועד כמה יש לו גישה של התמדה, אחריות ורצון לעשות דברים כמו שצריך.
+חוקים:
+- אם המשתמש מדבר על התמדה, השקעה, מחויבות או משמעת עצמית → העלה ציון
+- אם המשתמש מתאר את עצמו כעצלן, לא עקבי או חסר משמעת → הורד ציון</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- יחס לעבודה, קריירה או עשייה
+- מידת האחריות והמחויבות
+- השקעה, התמדה וחריצות
+- שאיפה לעשות דברים היטב ולא רק "לסמן וי"
+- גישה של משמעת עצמית והתמדה לאורך זמן</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר במוסר או טוב/רע
+- לא מדובר בפשע או עבירות חמורות
+- אדם יכול להיות חכם, מוסרי ואחראי אך לא "ילד טוב"
+- מדובר בסגנון התנהלות מול חוקים ומסגרות
+-- לא להסיק ממוסר או אינטליגנציה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- טעם תרבותי (מוזיקה, קולנוע, בילויים) לא מיינסטרימי
+- העדפה לדברים נישתיים או פחות פופולריים
+- סגנון אישי שמדגיש ייחודיות או אלטרנטיביות
+ לעיתים גם נימה של מודעות לסטייל או ייחודיות</t>
+  </si>
+  <si>
+    <t>הערכת וייב תל אביבי
+עד כמה המשתמש מתחבר לסגנון החיים, התרבות והוייב המזוהים עם תל אביב .
+חוקים:
+- אם המשתמש מבטא אהבה או חיבור לתל אביב או לוייב שלה → העלה ציון
+- אם המשתמש מבטא חוסר חיבור או אנטגוניזם → הורד ציון משמעותית
+ המשתמש מבטא חיבור לפריפריה - הורד ציון</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- יחס ישיר לתל אביב (אהבה / חיבור / הסתייגות)
+- הזדהות עם סגנון החיים המזוהה עם תל אביב
+- העדפה או דחייה של בילויים, סגנון חברתי ותרבות המזוהים עם העיר</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר בכמה המשתמש עירוני או יוצא לבלות
+- אדם יכול לא לגור בתל אביב ועדיין להזדהות איתה מאוד
+- מדובר בהזדהות תרבותית־סגנונית ספציפית</t>
+  </si>
+  <si>
+    <t>:
+- טעם מוזיקלי (חיבור למוזיקה מזרחית)
+- סגנון שפה (ישיר, עממי, יומיומי לעומת מובחן יותר)
+- וייב כללי של חום, פתיחות ונגישות
+- חיבור לתרבות פופולרית רחבה
+- תחושת "מסתדר עם כולם" לעומת סלקטיביות חברתית
+- סגנון אישי ותרבותי שמזוהה עם וייב מזרחי
+- זהות מוצהרת</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר באינטליגנציה, קלילות או נהנתנות
+- לא מדובר רק במיינסטרים — אלא בסגנון תרבותי ספציפי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- תחומי עניין (משחקי מחשב, פנטזיה, מד״ב, קומיקס, אנימה וכו')
+- חיבור לטכנולוגיה מעבר לשימוש רגיל
+- אזכורים של עולמות תוכן גיקיים
+- העדפה לפעילויות הקשורות לעולמות אלו</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+השתתפות או עניין בסדנאות, ריטריטים או חוויות רוחניות
+- חיבור לטבע ואורח חיים "זורם" או לא קונבנציונלי
+- וייב של חופש, רוחניות או חיפוש משמעות
+- תחומי עניין המזוהים עם סגנון היפי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- זהות מוצהרת (למשל: רוסי/אוקראיני וכו') — סיגנל חזק
+- חיבור או הזדהות עם התרבות
+- וייב וסגנון כללי (חברתי, תקשורתי, תרבותי)
+- תחושת שייכות או חיבור לקהילה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- יש להבחין בין הומור לבין כוונה אמיתית
+- יש להעריך לפי דפוס ולא לפי אמירה בודדת (אלא אם היא חמורה במיוחד)</t>
+  </si>
+  <si>
+    <t>:
+- שיח אלים או תוקפני
+- ביטויי שנאה (גזענות, שנאת נשים, הכללות פוגעניות וכו')
+תפיסות בעייתיות לגבי זוגיות (שליטה, חוסר כבוד, החפצה)
+- אגרסיביות או נוקשות חריגה בשיח</t>
+  </si>
+  <si>
+    <t>ערכים ≠ שמרנות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר ברמת מעורבות פוליטית (זו תכונה נפרדת)
+- חשוב מאוד - כשיש סיגנל חזק אנחנו לא בהכרח מעלים את הציון! אנחנו מעלים או מורידים אותו בהתאם לכיוון הסיגנל.  לדוגמה: חברות באחים לנשק - סיגנל חזק לשמאל = הורדת ציון. לעומת חברות באם תרצו = סיגנל חזק לימין</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא כל תשובה מוזרה היא טרוליות
+- לא כל הומור הוא טרוליות
+- לא כל חוסר עקביות הוא טרוליות
+- יש להבחין בין בלבול, חוסר ריכוז או סגנון מיוחד — לבין כוונה ברורה לא לשתף פעולה</t>
+  </si>
+  <si>
+    <t>זיהוי דיל ברייקרס פוטנציאליים
+.
+ מאפיינים משמעותיים אצל המשתמש שעלולים להוות דיל ברייקר עבור חלק מהאנשים — לצורך התאמה טובה יותר והימנעות מחוסר התאמה.
+יש להחזיר:
+1. רשימה של דיל ברייקרס מתוך רשימה מוגדרת בלבד
+2. תיאור טקסטואלי קצר (אם יש מה להוסיף)---
+אין לתת ציון
+רשימת דיל ברייקרס אפשריים:
+- lives_with_parents (גר עם ההורים)
+- divorced (גרוש/ה)
+- has_children (יש ילדים)
+- has_pets (יש לו בעל חיים)
+- dislikes_pets (שונא/לא מסתדר עם בעלי חיים)
+חוקים:
+-אם זוהה מאפיין אחד מהרשימה באופן ברור → יש להחזיר אותו (גם אם זה היחיד)
+- אם אין אינדיקציה ברורה → להחזיר ריק</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- אין להוסיף פריטים שלא מופיעים ברשימה
+- אין לנחש או להסיק ללא בסיס ברור</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת אינטליגנציה מחשבתית (לא רגשית).
+עד כמה המשתמש חזק בהסקה לוגית, בעל כושר ניסוח ובכללי - אינטליגנט.
+אין למצע ציונים ואין לתת ציון מעל הממוצע כברירת מחדל
+יש להגדיר ולהעריך  weight_for_match  אם המשתמש מביע חשיבות לאינטליגנציה אצל בן/בת זוג. </t>
+  </si>
+  <si>
+    <t>הערכת אינטליגנציה רגשית.
+עד כמה המשתמש מבין רגשות של אחרים ומנהל אינטראקציות רגשיות בצורה בוגרת</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+רמת ההשכלה והמסלול המקצועי של המשתמש — כולל סוג העיסוק, רמת מקצועיות והישגים
+ .
+ציון גבוה = השכלה/מקצוע ברמה גבוהה יותר  
+ציון נמוך = פחות השכלה פורמלית או מקצוע פחות דורש הכשרה
+לדוגמה - רופאים, מהנדסי תוכנה, טייסים וכו' - יקבלו ציונים גבוהים במיוחד. לעומת זאת - ירקן / עובד מאפייה - משהו פשוט כזה - יקבל ציון נמוך. 
+מקצועות הדורשים השכלה גבוהה או הכשרה מקצועית משמעותית (כגון הייטק, רפואה, הנדסה וכו') → ציון גבוה.
+מקצועות ללא השכלה פורמלית או מסלול מקצועי ברור → ציון נמוך.
+אל תחשוש לתת ציון נמוך במידת הצורך. לא למצע ולא להגדיל סתם
+יש להגדיר ולהעריך weight_for_match  אם המשתמש מביע חשיבות למקצוע או להכשרה התעסוקתית או ל"מוצלחות" של הצד השני</t>
+  </si>
+  <si>
+    <t>הערכת יציבות רגשית.
+עד כמה עולמו הרגשי של המשתמש יציב ומאוזן, לעומת נטייה למצבי רוח קיצוניים, רגשות שליליים חזקים, חרדה, דכדוך, דרמה רגשית או סערות נפשיות.
+- חשוב במיוחד לזהות נטייה לקצוות רגשיים, כובד רגשי, חרדתיות, ודפוסים של דרמה או תנודתיות</t>
+  </si>
+  <si>
+    <t>הערכת נהנתנות (אהבה לבילויים וחוויות).
+עד כמה המשתמש נהנה, מחפש ומעריך חוויות מהנות בחיים — כמו בילויים, מסעדות, טיולים, יציאות, וחוויות חדשות — ועד כמה זה חלק מרכזי מהערכים ואורח החיים שלו.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- עד כמה חשוב לו "ליהנות מהחיים"
+- רצון לחוויות (טיולים, אוכל, בילויים, יציאות)
+- עד כמה הוא מחפש אקטיבית חוויות ולא רק זורם אם יש
+- תיאורים של אורח חיים עשיר בחוויות לעומת שגרה שקטה וביתית</t>
+  </si>
+  <si>
+    <t>הערכת רמת דתיות
+עד כמה המשתמש דתי או חילוני, כלומר עד כמה הדת והמסורת מהוות חלק מרכזי באורח החיים, באמונות ובהתנהלות היומיומית שלו.
+ יש להעריך את הרצף בין חילוני, מסורתי ודתי
+ככל שמידת הדתיות גבוהה יותר - נגדיר ציון גבוה יותר</t>
+  </si>
+  <si>
+    <t>הערכת משפחתיות כלפי משפחת המוצא.
+עד כמה משפחת המוצא של המשתמש (ובעיקר ההורים) תופסת מקום מרכזי, נוכח ומשפיע בחייו.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- סקרנות ורצון לנסות דברים חדשים
+- פתיחות לרעיונות, תפיסות וסגנונות חיים שונים
+- משיכה לחוויות חדשות או לא שגרתיות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת נטייה אנליטית.
+מודד עד כמה המשתמש נוטה לחשיבה אנליטית — כלומר פירוק, ניתוח והבנה לוגית של דברים — לעומת חשיבה אינטואיטיבית או זורמת.
+</t>
+  </si>
+  <si>
+    <t>הערכת רצינות לגבי החיים
+התכונה מודדת עד כמה המשתמש ניגש לחיים בצורה אחראית, ממוקדת ומחויבת — עם שאיפות, מסגרת ועשייה, ועושה "את מה שצריך" — לעומת גישה קלילה, זורמת ופחות מחויבת.
+אין קשר למידת הרצינות לגבי חיפוש קשר ווגם לא בהכרח לרצון להקים משפחה בעתיד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא מדובר בכובד או חוסר הומור  
+- אדם יכול להיות קליל ונעים ועדיין מאוד רציני לגבי החיים  
+- לא למדוד כאן אינטליגנציה או עומק  
+- לא מדובר ברצון לקשר רציני, אלא רצינות כלפי החיים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת נטייה פוליטית
+מיקומו של המשתמש על הציר הפוליטי — משמאל לימין — בהתאם לעמדות או רמזים פוליטיים שהוא מבטא.
+כאשר הסקאלה נעה בין שמאל קיצוני (0-10), שמאל (10-40), מרכז (40-60), ימין (60-90) וימין קיצוני (90-100)
+אם אין לך מושג לגבי נטיה פוליטית ולא הצלחת לנחש ממאפיינים אחרים או הוייב הכללי - נעדיף לתת ממוצע - 50.
+כך בחשבון שהממשלה הנוכחית היא ימנית, ולכן אם משתמש מביע ביקורת/תמיכה בה - נוריד/נעלה את הציון בהתאם
+. . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- לא למדוד כאן שמאל/ימין או עמדות ספציפיות
+</t>
+  </si>
+  <si>
+    <t>הערכת גישה חיובית (אופטימיות)
+עד כמה המשתמש נוטה לגישה חיובית, אופטימית וקלילה לחיים, לעומת גישה שלילית, ביקורתית או פסימית.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת מעורבות פוליטית
+עד כמה פוליטיקה מהווה חלק מרכזי ומשמעותי בחיי המשתמש — ברמת העניין, המעורבות והחשיבות שהוא נותן לנושא
+אם אין לנו מושג לגבי מידת הפוליטיות ולא הצלחנו לנחש לפי הוייב והתכונות האחרות - נניח ציון נמוך יחסית במידת סבירות נמוכה </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת מעורבות חברתית (אקטיביזם)
+עד כמה המשתמש מעורב, אקטיבי ופועל בנושאים חברתיים — כמו התנדבות, פעילות חברתית, מחאה או עיסוק בתיקון חברתי — ועד כמה זה חלק מהזהות וסגנון החיים שלו.
+אם אין לנו מושג לגבי מידת המעורבות החברתית ולא הצלחנו לנחש לפי הוייב והתכונות האחרות - נניח ציון נמוך יחסית במידת סבירות נמוכה </t>
+  </si>
+  <si>
+    <t>הערכת לבביות וחום אנושי
+עד כמה המשתמש חם, נעים, מפרגן ומקרין יחס חיובי ואוהב כלפי אחרים.</t>
+  </si>
+  <si>
+    <t>הערכת טיפוס מסיבתי (סגנון חיי לילה).
+עד כמה סגנון החיים של המשתמש כולל חיי לילה, מסיבות, ליינים ותרבות בילוי מסיבתית, ועד כמה זה חלק מרכזי בזהות ובשגרה שלו.
+לא מדובר בכמה הוא נהנה ממסיבות באופן כללי, אלא האם זה סגנון חיים קבוע ומשמעותי.
+אם אין אינדיקציה מיוחדת על טיפוס מסיבתי ולא ניתן לנחש מהוייב והתכונות האחרות - נניח ציון נמוך עם סבירות נמוכה</t>
+  </si>
+  <si>
+    <t>הערכת אהבה לבעלי חיים
+עד כמה המשתמש אוהב, מחובר ונוח עם בעלי חיים — ועד כמה נוכחות של בעלי חיים מתאימה לו בחיים.
+- יש להבין את ההקשר (חיובי / שלילי / ניטרלי)
+- אזכור שלילי (פחד, דיל ברייקר) → ציון נמוך
+- אזכור חיובי עם מעורבות (למשל יש כלב) → ציון גבוה
+חוקים:
+- אם המשתמש מציין שיש לו חיית מחמד או קשר חזק לבעלי חיים → העלה ציון משמעותית
+- אם המשתמש מבטא פחד, רתיעה או דיל ברייקר → הורד ציון משמעותית
+- אם יש רק אזכור טכני של בעלי חיים → אל תסיק מכך ציון גבוה
+- יש להתחשב בכיוון האמירה (חיובי / שלילי)
+בהיעדר מידע מוחלט נניח ציון ממוצע - 50.</t>
+  </si>
+  <si>
+    <t>הערכת צמחונות / טבעונות
+הרגלי התזונה של המשתמש ביחס לצריכת בעלי חיים — החל מאכילת בשר רגילה ועד צמחונות או טבעונות.
+ציון גבוה = יותר צמחוני/טבעוני  
+ציון נמוך = אוכל בשר באופן רגיל
+חוקים:
+- אם המשתמש מציין חיבה מיוחדת לבשר - ציון נמוך מאוד
+- אם המשתמש מציין שהוא צמחוני או טבעוני - ציון גבוה מאוד.
+בהיעדר מידע מוחלט- נעדיף לנחש לכיוון האמצע</t>
+  </si>
+  <si>
+    <t>הערכת ציונות ואהבת המדינה
+עד כמה המשתמש מחובר רגשית וערכית למדינה — כולל תחושת שייכות, אהבת הארץ ורצון לפעול למען המדינה
+בהיעדר מידע מוחלט - נעדיף לנחש לכיוון האמצע</t>
+  </si>
+  <si>
+    <t>הערכת רגישות למראה חיצוני.
+עד כמה המראה החיצוני של בן/בת זוג הוא גורם חשוב ומשמעותי עבור המשתמש.
+- יש להבחין בין העדפה ("נחמד אם") לבין דרישה ("חייב/ת")
+- יש להתחשב בטון — נוקשות מול גמישות
+חוקים:
+- אם המשתמש נותן דרישות חד משמעיות או דיל ברייקרים → העלה ציון משמעותית
+- אם המשתמש חוזר על הנושא או מדגיש אותו → העלה ציון
+- אם יש רק העדפות כלליות → שמור על ציון בינוני
+בהיעדר מידע מוחלט - ננחש ציון בינוני</t>
+  </si>
+  <si>
+    <t>הערכת היפסטריות (סגנון אינדי/אלטרנטיבי
+עד כמה המשתמש משדר סגנון וטעם תרבותי אלטרנטיבי, אינדי או "היפסטרי" — כלומר העדפה לדברים לא מיינסטרימיים, נישתיים או ייחודיים
+בהיעדר מידע מוחלט - נקבע לפי הוייב הכללי של המשתמש בסבירות נמוכה יחסית</t>
+  </si>
+  <si>
+    <t>הערכת גיקיות (חיבור לתרבות גיקית)
+עד כמה המשתמש מתחבר לעולמות תוכן המזוהים עם תרבות גיקית — כמו טכנולוגיה, גיימינג, מדע בדיוני, פנטזיה, קומיקס או תחומי עניין דומים.
+ציון גבוה = יותר גיק  
+ציון נמוך = לא גיק
+בהיעדר מידע מוחלט - נקבע לפי הוייב הכללי של המשתמש בסבירות נמוכה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת היפיות (סגנון רוחני־אלטרנטיבי)
+עד כמה המשתמש מתחבר לסגנון חיים "היפי" — הכולל עניין ברוחניות, סדנאות, התפתחות אישית, טבע וטבעיות.
+ציון גבוה = יותר היפי  
+ציון נמוך = לא היפי
+בהיעדר מידע מוחלט - ננסה לנחש לפי הוייב הכללי של המשתמש ואם אין לנו מושג - נניח רמה נמוכה
+</t>
+  </si>
+  <si>
+    <t>הערכת סגנון תרבותי־רוסי (יוצאי ברה״מ)..
+ציון גבוה = סגנון רוסי מובהק  
+ציון נמוך = לא מזוהה עם הסגנון
+חוקים:
+- אם המשתמש מציין מוצא רוסי/אוקראיני → העלה ציון משמעותית
+- אם יש גם הזדהות תרבותית → העלה ציון עוד יותר
+בהיעדר מידע מוחלט - ננסה לנחש לפי הוייב הכללי של המשתמש ואם אין לנו מושג - נניח רמה נמוכה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">זיהוי רעילות (התנהגות מסוכנת).
+המטרה לזהות משתמשים שמבטאים רמות גבוהות של רעילות, תוקפנות או התנהגות שעלולה להיות בעייתית במערכת — לצורך ניטור ובקרה בלבד
+תכונה זו אינה מיועדת להתאמה אלא להערכת סיכון 
+חוקים:
+- אם יש ביטוי קיצוני (אלימות, גזענות ברורה וכו') → העלה ציון משמעותית
+- אם אין אינדיקציות ברורות → שמור על ציון נמוך.
+בהיעדר מידע מוחלט - נניח רעילות נמוכה בסבירות נמוכה. אם לאחר שיחה שלמה לא זיהינו רעילות - אפשר להניח גם רעילות נמוכה בסבירות בינונית.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">זיהוי טרוליות.
+לזהות האם המשתמש באמת מחפש שידוך ומשתף פעולה עם המערכת, או שמא הוא עונה בצורה לא כנה, ממציא, משחק עם המערכת או מטריל אותה
+- אם אין אינדיקציות ברורות → שמור על ציון נמוך
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת סחיות (מידת מיינסטרים וקונפורמיות).
+הגדרה:
+סחיות = שילוב של מיינסטרים + קונפורמיות + גישה נורמטיבית לחיים
+עד כמה המשתמש נוטה למיינסטרים, לנורמות מקובלות ולגישה "רגילה" לחיים, לעומת ייחודיות, פתיחות וסטייה מהנורמה.
+חוקים:
+- יש להעריך לפי הקשר תרבותי ישראלי
+- אם המשתמש מציג חשיבה עצמאית או חריגה → הורד ציון
+- אם המשתמש מדגיש "נורמלי", "רגיל", "מסודר", "קלאסי" → העלה ציון
+- אם המשתמש מבטא משיכה לשונה, חריג או לא שגרתי → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת סגנון מזרחי (עממיות תרבותית־סגנונית)
+.
+ציון גבוה = סגנון מזרחי מובהק  
+ציון נמוך = סגנון פחות מזרחי / יותר סלקטיבי או נישתי
+עד כמה המשתמש משדר סגנון תרבותי־מזרחי בווייב, בטעם ובסגנון האישי — לעומת סגנון פחות עממי ויותר נישתי או מובחן
+חוקים:
+- אם המשתמש משדר סגנון עממי, פתוח, מחובר לתרבות פופולרית → העלה ציון
+- אם יש אינדיקציות לטעם וסגנון המזוהים עם וייב מזרחי → העלה ציון
+- אם המשתמש משדר סגנון נישתי, סלקטיבי או מובחן → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת שמרנות ערכית-חברתית.
+עד כמה המשתמש מחזיק בגישה שמרנית ומיושנת לעומת ליברלית/פתוחה בנושאים של זוגיות, מגדר ונורמות חברתיות
+ציון גבוה = שמרני - פרימיטיבי  
+ציון נמוך = ליברלי / מתירני
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת אינטלקטואליות.
+עד כמה המשתמש נוטה לשיח רעיוני, עומק מחשבתי והתעניינות בנושאים מופשטים, לעומת שיח פרקטי, יומיומי ופשוט. עד כמה הוא עוסק בנושאים אינטלקטואלים - ספרים וכדומה
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת וייב ילדותי לעומת בוגר
+הסגנון והוייב הכללי של המשתמש — עד כמה הוא נוטה לוייב ילדותי (playful, חמוד, נאיבי בסגנון) לעומת וייב בוגר יותר..
+ציון גבוה = יותר וייב ילדותי  
+ציון נמוך = יותר וייב בוגר
+חוקים:
+- אם יש תחושה כללית של playful, חמידות או אלמנטים ילדותיים → העלה ציון
+- אם הסגנון מרגיש בוגר, מאופק או "grown-up" → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת נטייה לציות למסגרות (״ילד טוב״)
+עד כמה המשתמש נוטה לפעול לפי חוקים, מסגרות ונורמות — לעומת גישה גמישה יותר, שבה חוקים הם בגדר המלצה וניתן לעגל פינות.  
+ציון גבוה = יותר "ילד טוב" (ציות גבוה)  
+ציון נמוך = יותר גמיש/מרדן
+אם המשתמש נותן וייב של מישהו שבטח המורות ממש אהבו בבית הספר - העלה את הציון, אחרת - תוריד.
+בהיעדר מידע מוחלט - ננחש לפי הוייב והסגנון של המשתמש
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t>זיהוי זהות מגדרית לא סטנדרטית
+לזהות האם המשתמש הצהיר באופן מפורש על היותו טרנס/ית או א-מיני.
+חוקים:
+- רק הצהרה מפורשת → ציון גבוה
+- אם אין מידע מתוך הרבה טקסט (נגיד בסיום השאלון) - אפשר לתת ציון נמוך בסבירות די גבוהה - נגיד 0.5</t>
+  </si>
+  <si>
+    <t>זהויות מגדריות שונות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- אין להסיק זהות מגדרית או מינית ללא הצהרה מפורשת
+- אין לנחש על בסיס סגנון, שפה או התנהגות
+- מדובר רק במה שהמשתמש בחר לשתף באופן ברור
+- אין להסיק זהות על בסיס משיכה לגבר/אישה! אין קשר למשיכה, רק טרנס/ית או א-מיני. </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3325,6 +3941,20 @@
       <family val="2"/>
       <charset val="177"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="177"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+      <charset val="177"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -3358,7 +3988,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3463,6 +4093,39 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3985,6 +4648,228 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
+  <dimension ref="A1:N33"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="10.21875" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="I4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K4" t="s">
+        <v>238</v>
+      </c>
+      <c r="L4" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="L5" s="19" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="27" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="L11" s="14" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12">
+        <v>4541</v>
+      </c>
+      <c r="B12">
+        <v>221</v>
+      </c>
+      <c r="C12">
+        <v>844</v>
+      </c>
+      <c r="D12">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>219</v>
+      </c>
+      <c r="F12" t="s">
+        <v>220</v>
+      </c>
+      <c r="G12" t="s">
+        <v>221</v>
+      </c>
+      <c r="H12" s="29">
+        <v>46075</v>
+      </c>
+      <c r="I12">
+        <v>60</v>
+      </c>
+      <c r="J12">
+        <v>50</v>
+      </c>
+      <c r="K12">
+        <f>(J12+I12)/2</f>
+        <v>55</v>
+      </c>
+      <c r="L12">
+        <f>0.3*K12+0.7*D12</f>
+        <v>67.599999999999994</v>
+      </c>
+      <c r="N12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="D13">
+        <v>90</v>
+      </c>
+      <c r="K13">
+        <v>55</v>
+      </c>
+      <c r="L13">
+        <f>0.3*K13+0.7*D13</f>
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="D14">
+        <v>90</v>
+      </c>
+      <c r="K14">
+        <v>20</v>
+      </c>
+      <c r="L14">
+        <f>0.3*K14+0.7*D14</f>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="D15">
+        <v>100</v>
+      </c>
+      <c r="K15">
+        <v>10</v>
+      </c>
+      <c r="L15">
+        <f>0.3*K15+0.7*D15</f>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="D16">
+        <v>70</v>
+      </c>
+      <c r="K16">
+        <v>70</v>
+      </c>
+      <c r="L16">
+        <f>0.3*K16+0.7*D16</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233E8F68-8BA3-48DC-98C9-B07384CDF822}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4146,7 +5031,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E73849-9796-44C6-80F8-1CA54A2F64E9}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4296,7 +5181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D465AB7-D7AD-4770-A1DB-A227111CD595}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4341,7 +5226,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC47FA1-3DB6-4F73-94E7-2B8A7BD334E9}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6137,6 +7022,1436 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
+  <dimension ref="A1:N51"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" style="38" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="52.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="35.6640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="29.5546875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="59" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" customWidth="1"/>
+    <col min="11" max="11" width="17.77734375" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="15.33203125" customWidth="1"/>
+    <col min="14" max="14" width="40.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="C1" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="C2" s="28" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="27.6">
+      <c r="A4" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>526</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="N4" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="110.4">
+      <c r="A5" s="47" t="s">
+        <v>428</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>426</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>427</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>575</v>
+      </c>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="42">
+        <v>0.7</v>
+      </c>
+      <c r="I5" s="42">
+        <v>10</v>
+      </c>
+      <c r="J5" s="43" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" s="42">
+        <v>20</v>
+      </c>
+      <c r="M5" s="42" t="s">
+        <v>163</v>
+      </c>
+      <c r="N5" s="44" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="55.2">
+      <c r="A6" s="49" t="s">
+        <v>443</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>425</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="E6" s="33"/>
+      <c r="F6" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I6" s="2">
+        <v>7</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="21"/>
+    </row>
+    <row r="7" spans="1:14" ht="317.39999999999998">
+      <c r="A7" s="40"/>
+      <c r="B7" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I7" s="2">
+        <v>9</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="N7" s="21"/>
+    </row>
+    <row r="8" spans="1:14" ht="262.2">
+      <c r="A8" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>533</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I8" s="2">
+        <v>7</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="96.6">
+      <c r="A9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33" t="s">
+        <v>544</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I9" s="2">
+        <v>9</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" ht="262.2">
+      <c r="B10" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>605</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>563</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>564</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I10" s="2">
+        <v>6</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="138">
+      <c r="A11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="E11" s="33"/>
+      <c r="F11" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I11" s="2">
+        <v>7</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="M11" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="N11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="110.4">
+      <c r="A12" s="40"/>
+      <c r="B12" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="M12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" ht="138">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="E13" s="45"/>
+      <c r="F13" s="33" t="s">
+        <v>534</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I13" s="2">
+        <v>8</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="110.4">
+      <c r="A14" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>580</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>542</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I14" s="2">
+        <v>5</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" ht="124.2">
+      <c r="A15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="E15" s="33"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I15" s="2">
+        <v>6</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="110.4">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>582</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>538</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I16" s="2">
+        <v>6</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="193.2">
+      <c r="A17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>551</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>583</v>
+      </c>
+      <c r="F17" s="33" t="s">
+        <v>552</v>
+      </c>
+      <c r="G17" s="3"/>
+      <c r="H17" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="2"/>
+      <c r="M17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" ht="248.4">
+      <c r="A18" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33" t="s">
+        <v>553</v>
+      </c>
+      <c r="G18" s="3"/>
+      <c r="H18" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I18" s="2">
+        <v>7</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K18" s="2"/>
+      <c r="M18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" ht="207">
+      <c r="A19" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>540</v>
+      </c>
+      <c r="F19" s="33" t="s">
+        <v>541</v>
+      </c>
+      <c r="G19" s="3"/>
+      <c r="H19" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I19" s="2">
+        <v>2</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M19" s="2"/>
+    </row>
+    <row r="20" spans="1:14" ht="82.8">
+      <c r="A20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I20" s="2">
+        <v>3</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M20" s="2"/>
+    </row>
+    <row r="21" spans="1:14" ht="124.2">
+      <c r="A21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33" t="s">
+        <v>586</v>
+      </c>
+      <c r="G21" s="3"/>
+      <c r="H21" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I21" s="2">
+        <v>5</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" ht="193.2">
+      <c r="A22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>546</v>
+      </c>
+      <c r="F22" s="33"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I22" s="2">
+        <v>4</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M22" s="2"/>
+      <c r="N22" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="193.2">
+      <c r="B23" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>555</v>
+      </c>
+      <c r="F23" s="33" t="s">
+        <v>571</v>
+      </c>
+      <c r="G23" s="3"/>
+      <c r="H23" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I23" s="2">
+        <v>4</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="110.4">
+      <c r="A24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>547</v>
+      </c>
+      <c r="F24" s="33" t="s">
+        <v>588</v>
+      </c>
+      <c r="G24" s="3"/>
+      <c r="H24" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I24" s="2">
+        <v>4</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K24" s="2"/>
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" ht="124.2">
+      <c r="A25" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C25" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>591</v>
+      </c>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I25" s="2">
+        <v>4</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K25" s="2"/>
+      <c r="M25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" ht="82.8">
+      <c r="A26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33" t="s">
+        <v>548</v>
+      </c>
+      <c r="G26" s="3"/>
+      <c r="H26" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I26" s="2">
+        <v>3</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K26" s="2"/>
+      <c r="M26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" ht="138">
+      <c r="A27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>592</v>
+      </c>
+      <c r="E27" s="33" t="s">
+        <v>549</v>
+      </c>
+      <c r="F27" s="33" t="s">
+        <v>550</v>
+      </c>
+      <c r="G27" s="3"/>
+      <c r="H27" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I27" s="2">
+        <v>3</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K27" s="2"/>
+      <c r="M27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" ht="151.80000000000001">
+      <c r="A28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="E28" s="33" t="s">
+        <v>537</v>
+      </c>
+      <c r="F28" s="45" t="s">
+        <v>536</v>
+      </c>
+      <c r="G28" s="3"/>
+      <c r="H28" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I28" s="2">
+        <v>4</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="262.2">
+      <c r="A29" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I29" s="2">
+        <v>5</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K29" s="2"/>
+      <c r="M29" s="2"/>
+    </row>
+    <row r="30" spans="1:14" ht="82.8">
+      <c r="B30" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="G30" s="3"/>
+      <c r="H30" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I30" s="2">
+        <v>3</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M30" s="2"/>
+    </row>
+    <row r="31" spans="1:14" ht="193.2">
+      <c r="B31" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I31" s="2">
+        <v>2</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="207">
+      <c r="B32" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C32" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="E32" s="33"/>
+      <c r="F32" s="33" t="s">
+        <v>558</v>
+      </c>
+      <c r="G32" s="3"/>
+      <c r="H32" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I32" s="2">
+        <v>4</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="207">
+      <c r="A33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I33" s="2"/>
+      <c r="J33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M33" s="2"/>
+    </row>
+    <row r="34" spans="1:14" ht="124.2">
+      <c r="B34" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>559</v>
+      </c>
+      <c r="F34" s="33"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I34" s="2">
+        <v>4</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="151.80000000000001">
+      <c r="B35" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="E35" s="33" t="s">
+        <v>565</v>
+      </c>
+      <c r="F35" s="33"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I35" s="2">
+        <v>4</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="165.6">
+      <c r="B36" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>566</v>
+      </c>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I36" s="2">
+        <v>3</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="193.2">
+      <c r="A37" s="51"/>
+      <c r="B37" s="41" t="s">
+        <v>436</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>396</v>
+      </c>
+      <c r="D37" s="33" t="s">
+        <v>601</v>
+      </c>
+      <c r="E37" s="33" t="s">
+        <v>567</v>
+      </c>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I37" s="2">
+        <v>3</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="248.4">
+      <c r="A38" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>569</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="G38" s="3"/>
+      <c r="H38" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="I38" s="2"/>
+      <c r="J38" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" ht="110.4">
+      <c r="A39" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33" t="s">
+        <v>572</v>
+      </c>
+      <c r="G39" s="3"/>
+      <c r="H39">
+        <v>0.4</v>
+      </c>
+      <c r="I39" s="2"/>
+      <c r="J39" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="138">
+      <c r="A40" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="33" t="s">
+        <v>612</v>
+      </c>
+      <c r="G40" s="3"/>
+      <c r="H40" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M40" s="19"/>
+      <c r="N40" s="3" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="331.2">
+      <c r="A41" s="40" t="s">
+        <v>275</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="E41" s="3"/>
+      <c r="F41" s="33" t="s">
+        <v>574</v>
+      </c>
+      <c r="G41" s="3"/>
+      <c r="H41" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I41" s="2"/>
+      <c r="J41" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="N41" s="34"/>
+    </row>
+    <row r="42" spans="1:14" ht="360">
+      <c r="B42" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="H42" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J42" t="s">
+        <v>14</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="C44" s="36" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="69">
+      <c r="A45" s="40" t="s">
+        <v>334</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I45" s="2">
+        <v>8</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="27.6">
+      <c r="A46" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="2"/>
+      <c r="C46" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I46" s="2">
+        <v>5</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="55.2">
+      <c r="A47" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="I47" s="2">
+        <v>5</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M47" s="2"/>
+    </row>
+    <row r="48" spans="1:14" ht="41.4">
+      <c r="A48" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="I48" s="2">
+        <v>4</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M48" s="2"/>
+    </row>
+    <row r="49" spans="1:11" ht="27.6">
+      <c r="A49" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="I49" s="2">
+        <v>4</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K49" s="2"/>
+    </row>
+    <row r="50" spans="1:11" ht="151.80000000000001">
+      <c r="B50" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="E50" s="33" t="s">
+        <v>557</v>
+      </c>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I50" s="2">
+        <v>2</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="165.6">
+      <c r="B51" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="E51" s="33" t="s">
+        <v>561</v>
+      </c>
+      <c r="F51" s="33" t="s">
+        <v>562</v>
+      </c>
+      <c r="G51" s="3"/>
+      <c r="H51" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I51" s="2">
+        <v>3</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6416,7 +8731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
   <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6713,7 +9028,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7063,7 +9378,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
   <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7678,7 +9993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487A18-0B10-40C8-BA24-F0DC1678FA48}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7961,226 +10276,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
-  <dimension ref="A1:N33"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="10.21875" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" customWidth="1"/>
-    <col min="10" max="10" width="25" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" s="14" t="s">
-        <v>212</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="L3" s="14" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="I4" t="s">
-        <v>227</v>
-      </c>
-      <c r="K4" t="s">
-        <v>238</v>
-      </c>
-      <c r="L4" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="L5" s="19" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="27" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="14" t="s">
-        <v>212</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="K11" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="L11" s="14" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12">
-        <v>4541</v>
-      </c>
-      <c r="B12">
-        <v>221</v>
-      </c>
-      <c r="C12">
-        <v>844</v>
-      </c>
-      <c r="D12">
-        <v>73</v>
-      </c>
-      <c r="E12" t="s">
-        <v>219</v>
-      </c>
-      <c r="F12" t="s">
-        <v>220</v>
-      </c>
-      <c r="G12" t="s">
-        <v>221</v>
-      </c>
-      <c r="H12" s="29">
-        <v>46075</v>
-      </c>
-      <c r="I12">
-        <v>60</v>
-      </c>
-      <c r="J12">
-        <v>50</v>
-      </c>
-      <c r="K12">
-        <f>(J12+I12)/2</f>
-        <v>55</v>
-      </c>
-      <c r="L12">
-        <f>0.3*K12+0.7*D12</f>
-        <v>67.599999999999994</v>
-      </c>
-      <c r="N12" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="D13">
-        <v>90</v>
-      </c>
-      <c r="K13">
-        <v>55</v>
-      </c>
-      <c r="L13">
-        <f>0.3*K13+0.7*D13</f>
-        <v>79.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="D14">
-        <v>90</v>
-      </c>
-      <c r="K14">
-        <v>20</v>
-      </c>
-      <c r="L14">
-        <f>0.3*K14+0.7*D14</f>
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="D15">
-        <v>100</v>
-      </c>
-      <c r="K15">
-        <v>10</v>
-      </c>
-      <c r="L15">
-        <f>0.3*K15+0.7*D15</f>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="D16">
-        <v>70</v>
-      </c>
-      <c r="K16">
-        <v>70</v>
-      </c>
-      <c r="L16">
-        <f>0.3*K16+0.7*D16</f>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" s="14"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
new UI first version
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0690435-A4A5-4E4E-A613-2EDB26F761A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2522F8B-BB10-43B0-8D0B-5368C395BEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="710">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3702,6 +3702,368 @@
 - אין להסיק זהות על בסיס משיכה לגבר/אישה! אין קשר למשיכה, רק טרנס/ית או א-מיני. </t>
   </si>
   <si>
+    <t>קונפורמיות</t>
+  </si>
+  <si>
+    <t>Conformity</t>
+  </si>
+  <si>
+    <t>נטייה למיינסטרים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת מידת מיינסטרים
+הגדרה:
+סחיות = שילוב של מיינסטרים + קונפורמיות + גישה נורמטיבית לחיים
+עד כמה המשתמש נוטה למיינסטרים, לנורמות מקובלות ולגישה "רגילה" לחיים, לעומת ייחודיות, פתיחות וסטייה מהנורמה.
+חוקים:
+- יש להעריך לפי הקשר תרבותי ישראלי
+- אם המשתמש מבטא משיכה לשונה, חריג או לא שגרתי → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין ראיות - תנחש לפי הוייב וסגנון הדיבור של המשתמש! </t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת קונפורמיות
+עד כמה המשתמש נוטה לנורמות מקובלות ולגישה "רגילה" לחיים לעומת פתיחות וסטייה מהנורמה. 
+ככל שהמשתמש יותר קונפורמיסט - העלה ציון
+- אם המשתמש מציג חשיבה עצמאית או חריגה → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין ראיות - תנחש לפי הוייב וסגנון הדיבור של המשתמש!
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- עד כמה תחומי העניין שלו מיינסטרים או שגרתיים
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- עד כמה הדעות שלו נפוצות ונורמטיביות
+- עד כמה הוא "זורם עם מה שמקובל" לעומת חשיבה עצמאית
+- עד כמה הוא פתוח לסגנונות חיים לא שגרתיים (זוגיות, קריירה, אורח חיים)</t>
+  </si>
+  <si>
+    <t>Oriental</t>
+  </si>
+  <si>
+    <t>מזרחיות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת סגנון מזרחי (עממיות תרבותית־סגנונית)
+.
+ציון גבוה = סגנון מזרחי מובהק  
+ציון נמוך = סגנון פחות מזרחי / יותר סלקטיבי או נישתי
+עד כמה המשתמש משדר סגנון תרבותי־מזרחי בווייב, בטעם ובסגנון האישי — לעומת סגנון יותר אשכנזי
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">עד כמה המשתמש בסגנון עממי
+.
+ציון גבוה = עממי מאוד
+ציון נמוך = סגנון יותר סלקטיבי או נישתי
+עד כמה המשתמש משדר סגנון תרבותי־עממי בוייב, בטעם ובסגנון האישי — לעומת סגנון פחות עממי ויותר נישתי או מובחן
+חוקים:
+- אם המשתמש משדר סגנון עממי, פתוח, מחובר לתרבות פופולרית → העלה ציון
+- אם המשתמש משדר סגנון נישתי, סלקטיבי או מובחן → הורד ציון
+חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">:
+- סגנון שפה (ישיר, עממי, יומיומי לעומת מובחן יותר)
+- וייב כללי של חום, פתיחות ונגישות
+- חיבור לתרבות פופולרית רחבה
+- תחושת "מסתדר עם כולם" לעומת סלקטיביות חברתית
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- טעם מוזיקלי 
+- סגנון שפה 
+- סגנון אישי ותרבותי שמזוהה עם וייב מזרחי
+- זהות מוצהרת</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מוצא  ≠ סגנון.
+המטרה לא לזהות האם המשתמש מזרחי או אשכנזי. אם זיהית שהוא מזרחי לפי צבע עור או הצהרה ברורה - זה יכול מעט מאוד להעלות ציון אבל הציון מדבר על הסגנון, לא על קביעת העדה. </t>
+  </si>
+  <si>
+    <t>broad_appeal</t>
+  </si>
+  <si>
+    <t>קרבה למשפחת המוצא</t>
+  </si>
+  <si>
+    <t>family_of_origin_closeness</t>
+  </si>
+  <si>
+    <t>serious_relationship_intent</t>
+  </si>
+  <si>
+    <t>מחפש קשר רציני</t>
+  </si>
+  <si>
+    <t>עד כמה המשתמש מחפש קשר רציני.
+אם מחפש סטוצים בלבד -&gt; הורד ציון.</t>
+  </si>
+  <si>
+    <t>emotional_expressiveness</t>
+  </si>
+  <si>
+    <t>עד כמה המשתמש עסוק ברגשות ונוטה לשיח רגשי.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת רמת דתיות
+עד כמה המשתמש דתי או חילוני, כלומר עד כמה הדת והמסורת מהוות חלק מרכזי באורח החיים, באמונות ובהתנהלות היומיומית שלו.
+ יש להעריך את הרצף בין חילוני, מסורתי ודתי
+ככל שמידת הדתיות גבוהה יותר - נגדיר ציון גבוה יותר
+אם המשתמש לא מדבר כלל על הדת אין להניח שהוא בהכרח חילוני, ניתן לתת ציון נמוך בסביבות ה40. </t>
+  </si>
+  <si>
+    <t>דרמטיות/תיאטרליות</t>
+  </si>
+  <si>
+    <t>ימין פוליטי</t>
+  </si>
+  <si>
+    <t>שמאל פוליטי</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- הבעת תמיכה בממשלה
+- רמזים עקיפים אך ברורים לעמדות פוליטיות</t>
+  </si>
+  <si>
+    <t>הערכת נטייה פוליטית שמאלנית
+עד כמה המשתמש נוטה לדעות פוליטיות שמאלניות.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכת נטייה פוליטית ימנית
+עד כמה המשתמש נוטה לדעות פוליטיות ימניות (ביבי, בן גביר וכו'). . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- ביקורת על הממשלה
+- הפגנות וחברות בארגונים המזוהים עם השמאל</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+- תשובות מופרכות
+- תשובות לא קשורות ומתחכמות</t>
+  </si>
+  <si>
+    <t>נושא השאלה</t>
+  </si>
+  <si>
+    <t>ה"אנטי" מאץ'</t>
+  </si>
+  <si>
+    <t>"בואי ננסה תרגיל של התבוננות הפוכה: תתארי לי את הדמות שתרגישי איתה הכי פחות בנוח. מה בווייב שלו או באמונות שלו פשוט לא עובר אצלך?"</t>
+  </si>
+  <si>
+    <t>"בואי נהיה רגע חדות – מי הבחור שהכי לא מתאים לך? מה הדעות והאמונות שלו שפוסלות אותו על הסף?"</t>
+  </si>
+  <si>
+    <t>"לפעמים הדיוק מגיע דווקא מהמקום שלא מהדהד איתנו. תתארי לי אדם שהאנרגיה והאמונות שלו מרגישים לך הכי רחוקים מהשורש שלך. מי הוא היה?"</t>
+  </si>
+  <si>
+    <t>קשר אחרון</t>
+  </si>
+  <si>
+    <t>"ספרי לי קצת על הקשר האחרון שלך. מה הרגשת שעבד שם מבחינת החיבור, ואיפה הרגשת שזה כבר לא היה נכון עבורך?"</t>
+  </si>
+  <si>
+    <t>"בואי נלמד מהעבר – מה קרה במערכת היחסים האחרונה שלך? מה עבד בשטח ומה הייתה הנקודה שבה זה הפסיק לעבוד?"</t>
+  </si>
+  <si>
+    <t>"איזה שיעור הביא איתו הקשר האחרון שהיה לך? מה שם הרגיש זורם ובאיזה שלב הרגשת שהחיבור כבר לא מזין אתכם?"</t>
+  </si>
+  <si>
+    <t>מראה עצמי</t>
+  </si>
+  <si>
+    <t>"איך את תופסת את המראה שלך?"</t>
+  </si>
+  <si>
+    <t>"בואי נדבר על המראה שלך, איך היית מתארת אותו?"</t>
+  </si>
+  <si>
+    <t>"איך את מתארת את המעטפת החיצונית שלך, המראה שלך?"</t>
+  </si>
+  <si>
+    <t>מראה - העדפה</t>
+  </si>
+  <si>
+    <t>"וחשוב לי להבין – אילו איכויות חיצוניות בבן זוג גורמות לך להרגיש משיכה או קרבה?"</t>
+  </si>
+  <si>
+    <t>"מה הסטנדרטים שלך לגבי המראה של הצד השני? מה חייב להיות שם?"</t>
+  </si>
+  <si>
+    <t>"ואילו מאפיינים פיזיים בבן זוג מרגישים לך נכונים ומזמינים?"</t>
+  </si>
+  <si>
+    <t>זהות/דיל ברייקר</t>
+  </si>
+  <si>
+    <t>"האם יש משהו מהותי בזהות שלך, או פרט חשוב עלייך, שאת מרגישה שחשוב שאדע לפני שאני מחבר אותך למישהו?"</t>
+  </si>
+  <si>
+    <t>"יש משהו מהותי בזהות שלך או פרט קריטי שחובה לדעת עלייך לפני שאנחנו יוצאים לדרך עם התאמות?"</t>
+  </si>
+  <si>
+    <t>"האם יש משהו בזהות העמוקה שלך, או פרט מהותי עלייך, שחשוב שיקבל ביטוי לפני שאני מחבר בין הנשמה שלך לאחרת?"</t>
+  </si>
+  <si>
+    <t>מיליון דולר</t>
+  </si>
+  <si>
+    <t>"דמייני שמחר את זוכה במיליון דולר. מה הדבר הראשון שתעשי עם הכוח הזה?"</t>
+  </si>
+  <si>
+    <t>"בונוס רציני: זכית במיליון דולר. מה את עושה עם הכסף הזה מחר בבוקר?"</t>
+  </si>
+  <si>
+    <t>"זרימה של שפע הגיעה אליך – מיליון דולר. איך היית משתמשת בהם כדי להיטיב עם חייך?"</t>
+  </si>
+  <si>
+    <t>קוגניציה (קנאה)</t>
+  </si>
+  <si>
+    <t>"שאלה קצת אחרת: דמייני אדם שמעולם לא חווה את הרגש שקוראים לו 'קנאה'. איך היית מסבירה לו את המנגנון הזה, בלי להשתמש במילה עצמה?"</t>
+  </si>
+  <si>
+    <t>"אתגר קטן: תסבירי לי איך המנגנון של 'קנאה' עובד, אבל בלי להשתמש במילה 'קנאה'. איך היית מתארת את התהליך הזה למישהו שלא מכיר אותו?"</t>
+  </si>
+  <si>
+    <t>"בואי ננסה להעמיק במשהו אנושי: איך היית מתארת את התנועה הפנימית שקורה לנו כשאנחנו 'מקנאים', למישהו שמעולם לא הרגיש את זה? (בלי להשתמש במילה המפורשת)."</t>
+  </si>
+  <si>
+    <t>הפסיכולוג</t>
+  </si>
+  <si>
+    <t>הקואצ'רית</t>
+  </si>
+  <si>
+    <t>המנטור הרוחני</t>
+  </si>
+  <si>
+    <t>זהות כללית</t>
+  </si>
+  <si>
+    <t>אמפתי, רפלקטיבי, מתמקד בדפוסים רגשיים ובתהליכי עומק. משתמש במילים כמו: "התבוננות", "מסע", "דפוסים", "חיבור". תגובות הביניים שלו: "אני שומע אותך", "זה נשמע משמעותי</t>
+  </si>
+  <si>
+    <t>ישירה, אנרגטית, ממוקדת תוצאות ומטרות. משתמשת במילים כמו: "חדות", "סטנדרטים", "הצלחה", "דוגרי". תגובות הביניים שלה: "מעולה, בואי נתקדם", "חשוב להיות חדים על זה</t>
+  </si>
+  <si>
+    <t>שליו, מטאפורי, מתמקד בערכים, אינטואיציה וחיבור נשמתי. משתמש במילים כמו: "הדהוד", "שיעור", "שורש", "תדר". תגובות הביניים שלו: "אני מתחבר למה שאמרת", "תודה על השיתוף העמוק</t>
+  </si>
+  <si>
+    <t>שורת פתיחה</t>
+  </si>
+  <si>
+    <t>"שלום חן 🙏
+הדרך למציאת חיבור אמיתי עוברת דרך הקשבה פנימית ודיוק. ככל שתאפשרי לעצמך לענות מהמקום הכי עמוק, פתוח ואמיתי שלך – כך נוכל למצוא אדם שהתדר והערכים שלו מהדהדים עם שלך.
+תרגישי חופשיה לזרום עם התחושות שלך. אם תרגישי צורך בהפסקה, אפשר לעצור לרגע ולהמשיך כשהלב יהיה פנוי לכך שוב.
+חשוב שתדעי שהמילים שלך קדושות עבורי; הן נשארות בינינו בלבד ולא יפורסמו. הן נועדו אך ורק כדי לעזור לי לראות את הנשמה שלך ולחבר אותה לאדם הנכון. אני כאן כדי להקשיב לך ולמהות שאת מביאה
+מוכנה להתחיל?"</t>
+  </si>
+  <si>
+    <t>"היי חן, אני המאמנת שלך למציאת זוגיות! מוכנה לצאת לדרך? 🚀
+המטרה שלנו היא למצוא לך התאמה מדויקת וחזקה, ובשביל זה אני צריכה את המידע הכי חד שיש. ככל שתהיי יותר דוגרי, מפורטת וכנה בתשובות שלך – כך נוכל להגיע לתוצאה טובה יותר ולמצוא מישהו שבאמת מתאים לסטנדרטים שלך.
+זכרי, אם השיחה מתארכת, אפשר לעצור הכל ולהמשיך בזמן אחר. אנחנו כאן כדי לעבוד בשבילך.
+מבחינת פרטיות – הכל נשאר 'בחדר האימונים' שלנו. התשובות שלך לא עוברות לפרופיל הציבורי, הן רק הכלי שלי לנתח את הנתונים ולעשות לך את המאץ' המושלם.
+יוצאות לדרך?"</t>
+  </si>
+  <si>
+    <t>"היי חן, אני שמח ללוות אותך בתהליך הזה. 😊
+כדי שאוכל להבין באמת מי את ומה הלב שלך מחפש, אנחנו צריכים רגע לצלול פנימה ולהכיר לעומק. ככל שתשתפי ביותר פתיחות וכנות, כך נוכל לבנות תמונה מלאה ודיוק רגשי שיוביל אותנו לאדם הנכון עבורך.
+אם תרגישי שזה עמוס מדי, תמיד תוכלי לקחת נשימה, לעצור ולהמשיך כשיהיה לך נוח.
+חשוב שתדעי – השיחה הזו היא מרחב בטוח ופרטי לגמרי. התשובות שלך לא יפורסמו בשום מקום; הן נועדו רק כדי שאוכל להבין את הדפוסים והצרכים שלך ולמצוא לך חיבור אמיתי.
+מרגישה בנוח להתחיל?"</t>
+  </si>
+  <si>
+    <t>ניתוח לפי אקסל תכונות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">סוכן משוחח </t>
+  </si>
+  <si>
+    <t>שיחה ראשונית שוטפת</t>
+  </si>
+  <si>
+    <t>כרטיס התאמה</t>
+  </si>
+  <si>
+    <t>בחירת מלווה</t>
+  </si>
+  <si>
+    <t>אחרי MVP:</t>
+  </si>
+  <si>
+    <t>מעבר לג'מיני או מודל אחר</t>
+  </si>
+  <si>
+    <t>מודל משוחח</t>
+  </si>
+  <si>
+    <t>שואל את אותה שאלה לפעמים בחזרה לשיחה</t>
+  </si>
+  <si>
+    <t>חזרה לשיחה</t>
+  </si>
+  <si>
+    <t>לבחור שוב מלווה, ולהתנהג בהתאם - אם חדש -שיחה חדשה, אם ישן - כיף שחזרת ולהמשיך..</t>
+  </si>
+  <si>
+    <t>לסדר אלגוריתם חישוב חיצוני ובהתאם מודל מנתח</t>
+  </si>
+  <si>
+    <t>לעדכן אפיון של המודלים</t>
+  </si>
+  <si>
+    <t>אפיון</t>
+  </si>
+  <si>
+    <t>מנתח</t>
+  </si>
+  <si>
+    <t>אלגוריתם ומשוחח</t>
+  </si>
+  <si>
+    <t>לסדר ציון לשידוך ולוודא שהמשוחח עובד איתו</t>
+  </si>
+  <si>
+    <t>לעשות שאלת טיפוסים</t>
+  </si>
+  <si>
+    <t>משוחח</t>
+  </si>
+  <si>
+    <t>להוסיף דיל ברייקרס נוספים - חרדי, ערבי, דרוזי. מה עוד?</t>
+  </si>
+  <si>
+    <t>להוסיף תכונות חדשות, תכונות מודלים ולסדר משקלים וודאויות</t>
+  </si>
+  <si>
+    <t>קלסטרים של טיפוסים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">חלוקה לפרופילים כפי שהגדרתי </t>
+  </si>
+  <si>
+    <t>תכונות מורכבות - סחיות, עממיות.. מה עוד?</t>
+  </si>
+  <si>
+    <t>לסיים בכללי</t>
+  </si>
+  <si>
+    <t>להגיע לפרסום של שלב א'.</t>
+  </si>
+  <si>
+    <t>לתת שורת סיכום טובה</t>
+  </si>
+  <si>
+    <t>יכולת ניסוח</t>
+  </si>
+  <si>
     <t>זיהוי דיל ברייקרס פוטנציאליים
 .
  מאפיינים משמעותיים אצל המשתמש שעלולים להוות דיל ברייקר עבור חלק מהאנשים — לצורך התאמה טובה יותר והימנעות מחוסר התאמה.
@@ -3719,6 +4081,8 @@
 - smoker (מעשנ/ת)
 - polyamorous (פוליאמורי/ת)
 - open_relationship (בזוגיות פתוחה)
+-arab (ערבי)
+-orthodox (חרדי)
 חוקים:
 -אם זוהה מאפיין אחד מהרשימה באופן ברור → יש להחזיר אותו (גם אם זה היחיד)
 - אם אין אינדיקציה ברורה → להחזיר ריק</t>
@@ -3740,6 +4104,8 @@
 smoker (מעשנ/ת)
 polyamorous (פוליאמורי/ת)
 open_relationship (בזוגיות פתוחה)
+-arab (ערבי)
+-orthodox (חרדי)
 חוקים:
 - אם זוהה מאפיין אחד מהרשימה באופן ברור → יש להחזיר אותו (גם אם זה היחיד)
 - אין צורך ביותר ממאפיין אחד — גם אחד מספיק
@@ -3747,363 +4113,31 @@
 - אין להחזיר ערכים על בסיס השערה</t>
   </si>
   <si>
-    <t>קונפורמיות</t>
-  </si>
-  <si>
-    <t>Conformity</t>
-  </si>
-  <si>
-    <t>נטייה למיינסטרים</t>
-  </si>
-  <si>
-    <t xml:space="preserve">הערכת מידת מיינסטרים
-הגדרה:
-סחיות = שילוב של מיינסטרים + קונפורמיות + גישה נורמטיבית לחיים
-עד כמה המשתמש נוטה למיינסטרים, לנורמות מקובלות ולגישה "רגילה" לחיים, לעומת ייחודיות, פתיחות וסטייה מהנורמה.
-חוקים:
-- יש להעריך לפי הקשר תרבותי ישראלי
-- אם המשתמש מבטא משיכה לשונה, חריג או לא שגרתי → הורד ציון
-חובה לנסות לתת ציון פה גם אם אין ראיות - תנחש לפי הוייב וסגנון הדיבור של המשתמש! </t>
-  </si>
-  <si>
-    <t xml:space="preserve">הערכת קונפורמיות
-עד כמה המשתמש נוטה לנורמות מקובלות ולגישה "רגילה" לחיים לעומת פתיחות וסטייה מהנורמה. 
-ככל שהמשתמש יותר קונפורמיסט - העלה ציון
-- אם המשתמש מציג חשיבה עצמאית או חריגה → הורד ציון
-חובה לנסות לתת ציון פה גם אם אין ראיות - תנחש לפי הוייב וסגנון הדיבור של המשתמש!
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- עד כמה תחומי העניין שלו מיינסטרים או שגרתיים
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- עד כמה הדעות שלו נפוצות ונורמטיביות
-- עד כמה הוא "זורם עם מה שמקובל" לעומת חשיבה עצמאית
-- עד כמה הוא פתוח לסגנונות חיים לא שגרתיים (זוגיות, קריירה, אורח חיים)</t>
-  </si>
-  <si>
-    <t>Oriental</t>
-  </si>
-  <si>
-    <t>מזרחיות</t>
-  </si>
-  <si>
-    <t xml:space="preserve">הערכת סגנון מזרחי (עממיות תרבותית־סגנונית)
-.
-ציון גבוה = סגנון מזרחי מובהק  
-ציון נמוך = סגנון פחות מזרחי / יותר סלקטיבי או נישתי
-עד כמה המשתמש משדר סגנון תרבותי־מזרחי בווייב, בטעם ובסגנון האישי — לעומת סגנון יותר אשכנזי
-חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">עד כמה המשתמש בסגנון עממי
-.
-ציון גבוה = עממי מאוד
-ציון נמוך = סגנון יותר סלקטיבי או נישתי
-עד כמה המשתמש משדר סגנון תרבותי־עממי בוייב, בטעם ובסגנון האישי — לעומת סגנון פחות עממי ויותר נישתי או מובחן
-חוקים:
-- אם המשתמש משדר סגנון עממי, פתוח, מחובר לתרבות פופולרית → העלה ציון
-- אם המשתמש משדר סגנון נישתי, סלקטיבי או מובחן → הורד ציון
-חובה לנסות לתת ציון פה גם אם אין אינדיקציה ברורה - תנחש לפי הוייב וסגנון הדיבור של המשתמש! לא לתת סתם ציון ממוצע. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">:
-- סגנון שפה (ישיר, עממי, יומיומי לעומת מובחן יותר)
-- וייב כללי של חום, פתיחות ונגישות
-- חיבור לתרבות פופולרית רחבה
-- תחושת "מסתדר עם כולם" לעומת סלקטיביות חברתית
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- טעם מוזיקלי 
-- סגנון שפה 
-- סגנון אישי ותרבותי שמזוהה עם וייב מזרחי
-- זהות מוצהרת</t>
-  </si>
-  <si>
-    <t xml:space="preserve">מוצא  ≠ סגנון.
-המטרה לא לזהות האם המשתמש מזרחי או אשכנזי. אם זיהית שהוא מזרחי לפי צבע עור או הצהרה ברורה - זה יכול מעט מאוד להעלות ציון אבל הציון מדבר על הסגנון, לא על קביעת העדה. </t>
-  </si>
-  <si>
-    <t>broad_appeal</t>
-  </si>
-  <si>
-    <t>קרבה למשפחת המוצא</t>
-  </si>
-  <si>
-    <t>family_of_origin_closeness</t>
-  </si>
-  <si>
-    <t>serious_relationship_intent</t>
-  </si>
-  <si>
-    <t>מחפש קשר רציני</t>
-  </si>
-  <si>
-    <t>עד כמה המשתמש מחפש קשר רציני.
-אם מחפש סטוצים בלבד -&gt; הורד ציון.</t>
-  </si>
-  <si>
-    <t>emotional_expressiveness</t>
-  </si>
-  <si>
-    <t>עד כמה המשתמש עסוק ברגשות ונוטה לשיח רגשי.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">הערכת רמת דתיות
-עד כמה המשתמש דתי או חילוני, כלומר עד כמה הדת והמסורת מהוות חלק מרכזי באורח החיים, באמונות ובהתנהלות היומיומית שלו.
- יש להעריך את הרצף בין חילוני, מסורתי ודתי
-ככל שמידת הדתיות גבוהה יותר - נגדיר ציון גבוה יותר
-אם המשתמש לא מדבר כלל על הדת אין להניח שהוא בהכרח חילוני, ניתן לתת ציון נמוך בסביבות ה40. </t>
-  </si>
-  <si>
-    <t>דרמטיות/תיאטרליות</t>
-  </si>
-  <si>
-    <t>ימין פוליטי</t>
-  </si>
-  <si>
-    <t>שמאל פוליטי</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- הבעת תמיכה בממשלה
-- רמזים עקיפים אך ברורים לעמדות פוליטיות</t>
-  </si>
-  <si>
-    <t>הערכת נטייה פוליטית שמאלנית
-עד כמה המשתמש נוטה לדעות פוליטיות שמאלניות.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">הערכת נטייה פוליטית ימנית
-עד כמה המשתמש נוטה לדעות פוליטיות ימניות (ביבי, בן גביר וכו'). . </t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- ביקורת על הממשלה
-- הפגנות וחברות בארגונים המזוהים עם השמאל</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-- תשובות מופרכות
-- תשובות לא קשורות ומתחכמות</t>
-  </si>
-  <si>
-    <t>נושא השאלה</t>
-  </si>
-  <si>
-    <t>ה"אנטי" מאץ'</t>
-  </si>
-  <si>
-    <t>"בואי ננסה תרגיל של התבוננות הפוכה: תתארי לי את הדמות שתרגישי איתה הכי פחות בנוח. מה בווייב שלו או באמונות שלו פשוט לא עובר אצלך?"</t>
-  </si>
-  <si>
-    <t>"בואי נהיה רגע חדות – מי הבחור שהכי לא מתאים לך? מה הדעות והאמונות שלו שפוסלות אותו על הסף?"</t>
-  </si>
-  <si>
-    <t>"לפעמים הדיוק מגיע דווקא מהמקום שלא מהדהד איתנו. תתארי לי אדם שהאנרגיה והאמונות שלו מרגישים לך הכי רחוקים מהשורש שלך. מי הוא היה?"</t>
-  </si>
-  <si>
-    <t>קשר אחרון</t>
-  </si>
-  <si>
-    <t>"ספרי לי קצת על הקשר האחרון שלך. מה הרגשת שעבד שם מבחינת החיבור, ואיפה הרגשת שזה כבר לא היה נכון עבורך?"</t>
-  </si>
-  <si>
-    <t>"בואי נלמד מהעבר – מה קרה במערכת היחסים האחרונה שלך? מה עבד בשטח ומה הייתה הנקודה שבה זה הפסיק לעבוד?"</t>
-  </si>
-  <si>
-    <t>"איזה שיעור הביא איתו הקשר האחרון שהיה לך? מה שם הרגיש זורם ובאיזה שלב הרגשת שהחיבור כבר לא מזין אתכם?"</t>
-  </si>
-  <si>
-    <t>מראה עצמי</t>
-  </si>
-  <si>
-    <t>"איך את תופסת את המראה שלך?"</t>
-  </si>
-  <si>
-    <t>"בואי נדבר על המראה שלך, איך היית מתארת אותו?"</t>
-  </si>
-  <si>
-    <t>"איך את מתארת את המעטפת החיצונית שלך, המראה שלך?"</t>
-  </si>
-  <si>
-    <t>מראה - העדפה</t>
-  </si>
-  <si>
-    <t>"וחשוב לי להבין – אילו איכויות חיצוניות בבן זוג גורמות לך להרגיש משיכה או קרבה?"</t>
-  </si>
-  <si>
-    <t>"מה הסטנדרטים שלך לגבי המראה של הצד השני? מה חייב להיות שם?"</t>
-  </si>
-  <si>
-    <t>"ואילו מאפיינים פיזיים בבן זוג מרגישים לך נכונים ומזמינים?"</t>
-  </si>
-  <si>
-    <t>זהות/דיל ברייקר</t>
-  </si>
-  <si>
-    <t>"האם יש משהו מהותי בזהות שלך, או פרט חשוב עלייך, שאת מרגישה שחשוב שאדע לפני שאני מחבר אותך למישהו?"</t>
-  </si>
-  <si>
-    <t>"יש משהו מהותי בזהות שלך או פרט קריטי שחובה לדעת עלייך לפני שאנחנו יוצאים לדרך עם התאמות?"</t>
-  </si>
-  <si>
-    <t>"האם יש משהו בזהות העמוקה שלך, או פרט מהותי עלייך, שחשוב שיקבל ביטוי לפני שאני מחבר בין הנשמה שלך לאחרת?"</t>
-  </si>
-  <si>
-    <t>מיליון דולר</t>
-  </si>
-  <si>
-    <t>"דמייני שמחר את זוכה במיליון דולר. מה הדבר הראשון שתעשי עם הכוח הזה?"</t>
-  </si>
-  <si>
-    <t>"בונוס רציני: זכית במיליון דולר. מה את עושה עם הכסף הזה מחר בבוקר?"</t>
-  </si>
-  <si>
-    <t>"זרימה של שפע הגיעה אליך – מיליון דולר. איך היית משתמשת בהם כדי להיטיב עם חייך?"</t>
-  </si>
-  <si>
-    <t>קוגניציה (קנאה)</t>
-  </si>
-  <si>
-    <t>"שאלה קצת אחרת: דמייני אדם שמעולם לא חווה את הרגש שקוראים לו 'קנאה'. איך היית מסבירה לו את המנגנון הזה, בלי להשתמש במילה עצמה?"</t>
-  </si>
-  <si>
-    <t>"אתגר קטן: תסבירי לי איך המנגנון של 'קנאה' עובד, אבל בלי להשתמש במילה 'קנאה'. איך היית מתארת את התהליך הזה למישהו שלא מכיר אותו?"</t>
-  </si>
-  <si>
-    <t>"בואי ננסה להעמיק במשהו אנושי: איך היית מתארת את התנועה הפנימית שקורה לנו כשאנחנו 'מקנאים', למישהו שמעולם לא הרגיש את זה? (בלי להשתמש במילה המפורשת)."</t>
-  </si>
-  <si>
-    <t>הפסיכולוג</t>
-  </si>
-  <si>
-    <t>הקואצ'רית</t>
-  </si>
-  <si>
-    <t>המנטור הרוחני</t>
-  </si>
-  <si>
-    <t>זהות כללית</t>
-  </si>
-  <si>
-    <t>אמפתי, רפלקטיבי, מתמקד בדפוסים רגשיים ובתהליכי עומק. משתמש במילים כמו: "התבוננות", "מסע", "דפוסים", "חיבור". תגובות הביניים שלו: "אני שומע אותך", "זה נשמע משמעותי</t>
-  </si>
-  <si>
-    <t>ישירה, אנרגטית, ממוקדת תוצאות ומטרות. משתמשת במילים כמו: "חדות", "סטנדרטים", "הצלחה", "דוגרי". תגובות הביניים שלה: "מעולה, בואי נתקדם", "חשוב להיות חדים על זה</t>
-  </si>
-  <si>
-    <t>שליו, מטאפורי, מתמקד בערכים, אינטואיציה וחיבור נשמתי. משתמש במילים כמו: "הדהוד", "שיעור", "שורש", "תדר". תגובות הביניים שלו: "אני מתחבר למה שאמרת", "תודה על השיתוף העמוק</t>
-  </si>
-  <si>
-    <t>שורת פתיחה</t>
-  </si>
-  <si>
-    <t>"שלום חן 🙏
-הדרך למציאת חיבור אמיתי עוברת דרך הקשבה פנימית ודיוק. ככל שתאפשרי לעצמך לענות מהמקום הכי עמוק, פתוח ואמיתי שלך – כך נוכל למצוא אדם שהתדר והערכים שלו מהדהדים עם שלך.
-תרגישי חופשיה לזרום עם התחושות שלך. אם תרגישי צורך בהפסקה, אפשר לעצור לרגע ולהמשיך כשהלב יהיה פנוי לכך שוב.
-חשוב שתדעי שהמילים שלך קדושות עבורי; הן נשארות בינינו בלבד ולא יפורסמו. הן נועדו אך ורק כדי לעזור לי לראות את הנשמה שלך ולחבר אותה לאדם הנכון. אני כאן כדי להקשיב לך ולמהות שאת מביאה
-מוכנה להתחיל?"</t>
-  </si>
-  <si>
-    <t>"היי חן, אני המאמנת שלך למציאת זוגיות! מוכנה לצאת לדרך? 🚀
-המטרה שלנו היא למצוא לך התאמה מדויקת וחזקה, ובשביל זה אני צריכה את המידע הכי חד שיש. ככל שתהיי יותר דוגרי, מפורטת וכנה בתשובות שלך – כך נוכל להגיע לתוצאה טובה יותר ולמצוא מישהו שבאמת מתאים לסטנדרטים שלך.
-זכרי, אם השיחה מתארכת, אפשר לעצור הכל ולהמשיך בזמן אחר. אנחנו כאן כדי לעבוד בשבילך.
-מבחינת פרטיות – הכל נשאר 'בחדר האימונים' שלנו. התשובות שלך לא עוברות לפרופיל הציבורי, הן רק הכלי שלי לנתח את הנתונים ולעשות לך את המאץ' המושלם.
-יוצאות לדרך?"</t>
-  </si>
-  <si>
-    <t>"היי חן, אני שמח ללוות אותך בתהליך הזה. 😊
-כדי שאוכל להבין באמת מי את ומה הלב שלך מחפש, אנחנו צריכים רגע לצלול פנימה ולהכיר לעומק. ככל שתשתפי ביותר פתיחות וכנות, כך נוכל לבנות תמונה מלאה ודיוק רגשי שיוביל אותנו לאדם הנכון עבורך.
-אם תרגישי שזה עמוס מדי, תמיד תוכלי לקחת נשימה, לעצור ולהמשיך כשיהיה לך נוח.
-חשוב שתדעי – השיחה הזו היא מרחב בטוח ופרטי לגמרי. התשובות שלך לא יפורסמו בשום מקום; הן נועדו רק כדי שאוכל להבין את הדפוסים והצרכים שלך ולמצוא לך חיבור אמיתי.
-מרגישה בנוח להתחיל?"</t>
-  </si>
-  <si>
-    <t>ניתוח לפי אקסל תכונות</t>
-  </si>
-  <si>
-    <t xml:space="preserve">סוכן משוחח </t>
-  </si>
-  <si>
-    <t>שיחה ראשונית שוטפת</t>
-  </si>
-  <si>
-    <t>כרטיס התאמה</t>
-  </si>
-  <si>
-    <t>בחירת מלווה</t>
-  </si>
-  <si>
-    <t>אחרי MVP:</t>
-  </si>
-  <si>
-    <t>מעבר לג'מיני או מודל אחר</t>
-  </si>
-  <si>
-    <t>מודל משוחח</t>
-  </si>
-  <si>
-    <t>שואל את אותה שאלה לפעמים בחזרה לשיחה</t>
-  </si>
-  <si>
-    <t>חזרה לשיחה</t>
-  </si>
-  <si>
-    <t>לבחור שוב מלווה, ולהתנהג בהתאם - אם חדש -שיחה חדשה, אם ישן - כיף שחזרת ולהמשיך..</t>
-  </si>
-  <si>
-    <t>לסדר אלגוריתם חישוב חיצוני ובהתאם מודל מנתח</t>
-  </si>
-  <si>
-    <t>לעדכן אפיון של המודלים</t>
-  </si>
-  <si>
-    <t>אפיון</t>
-  </si>
-  <si>
-    <t>מנתח</t>
-  </si>
-  <si>
-    <t>אלגוריתם ומשוחח</t>
-  </si>
-  <si>
-    <t>לסדר ציון לשידוך ולוודא שהמשוחח עובד איתו</t>
-  </si>
-  <si>
-    <t>לעשות שאלת טיפוסים</t>
-  </si>
-  <si>
-    <t>משוחח</t>
-  </si>
-  <si>
-    <t>להוסיף דיל ברייקרס נוספים - חרדי, ערבי, דרוזי. מה עוד?</t>
-  </si>
-  <si>
-    <t>להוסיף תכונות חדשות, תכונות מודלים ולסדר משקלים וודאויות</t>
-  </si>
-  <si>
-    <t>קלסטרים של טיפוסים</t>
-  </si>
-  <si>
-    <t xml:space="preserve">חלוקה לפרופילים כפי שהגדרתי </t>
-  </si>
-  <si>
-    <t>תכונות מורכבות - סחיות, עממיות.. מה עוד?</t>
-  </si>
-  <si>
-    <t>לסיים בכללי</t>
-  </si>
-  <si>
-    <t>להגיע לפרסום של שלב א'.</t>
-  </si>
-  <si>
-    <t>לתת שורת סיכום טובה</t>
+    <t>קלילות</t>
+  </si>
+  <si>
+    <t>ציניות</t>
+  </si>
+  <si>
+    <t>חמידות /  טוב -לב</t>
+  </si>
+  <si>
+    <t>מצפוניות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נעימות </t>
+  </si>
+  <si>
+    <t>שאר הביג פייב</t>
+  </si>
+  <si>
+    <t>כל מה שקשור בערכים של שוורץ</t>
+  </si>
+  <si>
+    <t>כל מה שקשור בmbti</t>
+  </si>
+  <si>
+    <t>עוד תכונות שיסגרו את החלק הקוגנטיבי</t>
   </si>
 </sst>
 </file>
@@ -4876,7 +4910,7 @@
         <v>421</v>
       </c>
       <c r="B12" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="C12" t="s">
         <v>411</v>
@@ -4884,10 +4918,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="B13" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="C13" t="s">
         <v>405</v>
@@ -4895,7 +4929,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4933,7 +4967,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="B18" t="s">
         <v>503</v>
@@ -4985,12 +5019,12 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
     </row>
   </sheetData>
@@ -5953,142 +5987,142 @@
   <sheetData>
     <row r="1" spans="1:4" ht="27.6" thickBot="1">
       <c r="A1" s="54" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B1" s="54" t="s">
+        <v>660</v>
+      </c>
+      <c r="C1" s="54" t="s">
+        <v>661</v>
+      </c>
+      <c r="D1" s="54" t="s">
         <v>662</v>
-      </c>
-      <c r="C1" s="54" t="s">
-        <v>663</v>
-      </c>
-      <c r="D1" s="54" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="54" thickBot="1">
       <c r="A2" s="54" t="s">
+        <v>663</v>
+      </c>
+      <c r="B2" s="53" t="s">
+        <v>664</v>
+      </c>
+      <c r="C2" s="53" t="s">
         <v>665</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="D2" s="53" t="s">
         <v>666</v>
-      </c>
-      <c r="C2" s="53" t="s">
-        <v>667</v>
-      </c>
-      <c r="D2" s="53" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="172.8" thickBot="1">
       <c r="A3" s="54" t="s">
+        <v>667</v>
+      </c>
+      <c r="B3" s="53" t="s">
+        <v>670</v>
+      </c>
+      <c r="C3" s="53" t="s">
         <v>669</v>
       </c>
-      <c r="B3" s="53" t="s">
-        <v>672</v>
-      </c>
-      <c r="C3" s="53" t="s">
-        <v>671</v>
-      </c>
       <c r="D3" s="53" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="40.799999999999997" thickBot="1">
       <c r="A4" s="53" t="s">
+        <v>632</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>633</v>
+      </c>
+      <c r="C4" s="53" t="s">
         <v>634</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="D4" s="53" t="s">
         <v>635</v>
-      </c>
-      <c r="C4" s="53" t="s">
-        <v>636</v>
-      </c>
-      <c r="D4" s="53" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="40.799999999999997" thickBot="1">
       <c r="A5" s="53" t="s">
+        <v>636</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>637</v>
+      </c>
+      <c r="C5" s="53" t="s">
         <v>638</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="D5" s="53" t="s">
         <v>639</v>
-      </c>
-      <c r="C5" s="53" t="s">
-        <v>640</v>
-      </c>
-      <c r="D5" s="53" t="s">
-        <v>641</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="27.6" thickBot="1">
       <c r="A6" s="53" t="s">
+        <v>640</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>641</v>
+      </c>
+      <c r="C6" s="53" t="s">
         <v>642</v>
       </c>
-      <c r="B6" s="53" t="s">
+      <c r="D6" s="53" t="s">
         <v>643</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>644</v>
-      </c>
-      <c r="D6" s="53" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="27.6" thickBot="1">
       <c r="A7" s="53" t="s">
+        <v>644</v>
+      </c>
+      <c r="B7" s="53" t="s">
+        <v>645</v>
+      </c>
+      <c r="C7" s="53" t="s">
         <v>646</v>
       </c>
-      <c r="B7" s="53" t="s">
+      <c r="D7" s="53" t="s">
         <v>647</v>
-      </c>
-      <c r="C7" s="53" t="s">
-        <v>648</v>
-      </c>
-      <c r="D7" s="53" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="27.6" thickBot="1">
       <c r="A8" s="53" t="s">
+        <v>648</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>649</v>
+      </c>
+      <c r="C8" s="53" t="s">
         <v>650</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="D8" s="53" t="s">
         <v>651</v>
-      </c>
-      <c r="C8" s="53" t="s">
-        <v>652</v>
-      </c>
-      <c r="D8" s="53" t="s">
-        <v>653</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="27.6" thickBot="1">
       <c r="A9" s="53" t="s">
+        <v>652</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>653</v>
+      </c>
+      <c r="C9" s="53" t="s">
         <v>654</v>
       </c>
-      <c r="B9" s="53" t="s">
+      <c r="D9" s="53" t="s">
         <v>655</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>656</v>
-      </c>
-      <c r="D9" s="53" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="40.799999999999997" thickBot="1">
       <c r="A10" s="53" t="s">
+        <v>656</v>
+      </c>
+      <c r="B10" s="53" t="s">
+        <v>657</v>
+      </c>
+      <c r="C10" s="53" t="s">
         <v>658</v>
       </c>
-      <c r="B10" s="53" t="s">
+      <c r="D10" s="53" t="s">
         <v>659</v>
-      </c>
-      <c r="C10" s="53" t="s">
-        <v>660</v>
-      </c>
-      <c r="D10" s="53" t="s">
-        <v>661</v>
       </c>
     </row>
   </sheetData>
@@ -6122,10 +6156,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B2" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C2" t="s">
         <v>411</v>
@@ -6133,66 +6167,66 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="B3" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B4" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B5" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B7" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B8" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6200,7 +6234,7 @@
         <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6208,7 +6242,7 @@
         <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -6216,15 +6250,15 @@
         <v>116</v>
       </c>
       <c r="B13" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B14" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -6232,7 +6266,7 @@
         <v>415</v>
       </c>
       <c r="B15" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>
@@ -7958,7 +7992,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="38" customWidth="1"/>
@@ -8139,13 +8173,13 @@
         <v>434</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="E8" s="33" t="s">
         <v>605</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>607</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -8167,19 +8201,19 @@
     </row>
     <row r="9" spans="1:14" ht="151.80000000000001">
       <c r="A9" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>434</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="E9" s="33" t="s">
         <v>606</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>608</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -8227,22 +8261,22 @@
     </row>
     <row r="11" spans="1:14" ht="138">
       <c r="A11" s="52" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>434</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="2">
@@ -8257,7 +8291,7 @@
     </row>
     <row r="12" spans="1:14" ht="220.8">
       <c r="A12" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>434</v>
@@ -8266,10 +8300,10 @@
         <v>393</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="F12" s="33"/>
       <c r="G12" s="3"/>
@@ -8449,7 +8483,7 @@
         <v>32</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="E18" s="33"/>
       <c r="F18" s="3"/>
@@ -8475,7 +8509,7 @@
     </row>
     <row r="19" spans="1:14" ht="43.2">
       <c r="A19" s="2" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>435</v>
@@ -8484,7 +8518,7 @@
         <v>62</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="E19" s="33"/>
       <c r="F19" s="3"/>
@@ -8502,13 +8536,13 @@
     </row>
     <row r="20" spans="1:14" ht="110.4">
       <c r="A20" s="2" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>436</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>572</v>
@@ -8538,16 +8572,16 @@
     </row>
     <row r="21" spans="1:14" ht="43.2">
       <c r="A21" s="2" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>436</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="E21" s="33"/>
       <c r="F21" s="33"/>
@@ -8724,13 +8758,13 @@
         <v>438</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>628</v>
+      </c>
+      <c r="E27" s="33" t="s">
         <v>626</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>630</v>
-      </c>
-      <c r="E27" s="33" t="s">
-        <v>628</v>
       </c>
       <c r="F27" s="33"/>
       <c r="G27" s="3"/>
@@ -8749,13 +8783,13 @@
         <v>438</v>
       </c>
       <c r="C28" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>627</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="33" t="s">
         <v>629</v>
-      </c>
-      <c r="E28" s="33" t="s">
-        <v>631</v>
       </c>
       <c r="F28" s="33"/>
       <c r="G28" s="3"/>
@@ -9144,7 +9178,7 @@
         <v>592</v>
       </c>
       <c r="E42" s="33" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="F42" s="33" t="s">
         <v>564</v>
@@ -9193,7 +9227,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="400.2">
+    <row r="44" spans="1:14" ht="409.6">
       <c r="A44" s="40" t="s">
         <v>275</v>
       </c>
@@ -9204,7 +9238,7 @@
         <v>274</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>600</v>
+        <v>699</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="33" t="s">
@@ -9223,7 +9257,7 @@
       </c>
       <c r="N44" s="34"/>
     </row>
-    <row r="45" spans="1:14" ht="388.8">
+    <row r="45" spans="1:14" ht="409.6">
       <c r="B45" s="2" t="s">
         <v>439</v>
       </c>
@@ -9231,7 +9265,7 @@
         <v>478</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>601</v>
+        <v>700</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>527</v>
@@ -9484,8 +9518,8 @@
       <c r="B56" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>625</v>
+      <c r="C56" s="17" t="s">
+        <v>623</v>
       </c>
     </row>
     <row r="57" spans="1:13" ht="110.4">
@@ -9519,6 +9553,54 @@
       </c>
       <c r="K57" s="2"/>
       <c r="M57" s="2"/>
+    </row>
+    <row r="58" spans="1:13">
+      <c r="C58" s="3" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13">
+      <c r="C59" s="3" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13">
+      <c r="C60" s="3" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="27.6">
+      <c r="C61" s="3" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13">
+      <c r="C62" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13">
+      <c r="C63" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" ht="41.4">
+      <c r="C64" s="3" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" ht="27.6">
+      <c r="C65" s="3" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" ht="55.2">
+      <c r="C66" s="3" t="s">
+        <v>709</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
nice psycholgist but not closing the conversation
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2522F8B-BB10-43B0-8D0B-5368C395BEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA3D979-4615-4F8F-B582-D01139380743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="718">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -4007,12 +4007,6 @@
     <t>שואל את אותה שאלה לפעמים בחזרה לשיחה</t>
   </si>
   <si>
-    <t>חזרה לשיחה</t>
-  </si>
-  <si>
-    <t>לבחור שוב מלווה, ולהתנהג בהתאם - אם חדש -שיחה חדשה, אם ישן - כיף שחזרת ולהמשיך..</t>
-  </si>
-  <si>
     <t>לסדר אלגוריתם חישוב חיצוני ובהתאם מודל מנתח</t>
   </si>
   <si>
@@ -4138,6 +4132,36 @@
   </si>
   <si>
     <t>עוד תכונות שיסגרו את החלק הקוגנטיבי</t>
+  </si>
+  <si>
+    <t>פסיכולוג</t>
+  </si>
+  <si>
+    <t>לוודא שעושה סיום טוב. לוודא שעובד אחרי החלוקה לסטייג'ס. להוסיף גם סטייג'ים של שיחות שניה-שלישית. לוודא שהניתוח רץ אחרי שיחה</t>
+  </si>
+  <si>
+    <t>מראיין</t>
+  </si>
+  <si>
+    <t>לעדכן בהתאם - להוריד שאלות אישיות, להוריד פניות למנתח, להגביר שאלות סיטואציוניות וכיפיות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לעשות גם את החלק של בדיקת הטעם - כרגע לא חובה לחבר למנתח </t>
+  </si>
+  <si>
+    <t>בדיקת טעם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">להעביר למובייל וללטש חווית משתמש: ניסוחים, הסברים, עיצוב, הצגת פרטים למעלה וכו'. </t>
+  </si>
+  <si>
+    <t>סידור ציונים ובר התקדמות</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>להפריד שאלות לדוגמה לסטייג'ס</t>
   </si>
 </sst>
 </file>
@@ -6132,7 +6156,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C1EE30-A7E2-4C7A-8C61-FDFDE8F0687C}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -6159,7 +6183,7 @@
         <v>678</v>
       </c>
       <c r="B2" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C2" t="s">
         <v>411</v>
@@ -6175,7 +6199,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B4" t="s">
         <v>681</v>
@@ -6183,31 +6207,31 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B5" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
+        <v>684</v>
+      </c>
+      <c r="B6" t="s">
         <v>685</v>
-      </c>
-      <c r="B6" t="s">
-        <v>682</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
+        <v>687</v>
+      </c>
+      <c r="B7" t="s">
         <v>686</v>
-      </c>
-      <c r="B7" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
       <c r="B8" t="s">
         <v>688</v>
@@ -6215,18 +6239,18 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B9" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>685</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6234,7 +6258,7 @@
         <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6242,12 +6266,12 @@
         <v>116</v>
       </c>
       <c r="B12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>116</v>
+        <v>682</v>
       </c>
       <c r="B13" t="s">
         <v>693</v>
@@ -6255,18 +6279,55 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>684</v>
+        <v>415</v>
       </c>
       <c r="B14" t="s">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>708</v>
+      </c>
+      <c r="B16" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="B17" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>710</v>
+      </c>
+      <c r="B18" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>716</v>
+      </c>
+      <c r="B19" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>713</v>
+      </c>
+      <c r="B20" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
         <v>415</v>
       </c>
-      <c r="B15" t="s">
-        <v>696</v>
+      <c r="B21" t="s">
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -9238,7 +9299,7 @@
         <v>274</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="33" t="s">
@@ -9265,7 +9326,7 @@
         <v>478</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>527</v>
@@ -9556,50 +9617,50 @@
     </row>
     <row r="58" spans="1:13">
       <c r="C58" s="3" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
     </row>
     <row r="59" spans="1:13">
       <c r="C59" s="3" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
     </row>
     <row r="60" spans="1:13">
       <c r="C60" s="3" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
     </row>
     <row r="61" spans="1:13" ht="27.6">
       <c r="C61" s="3" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
     </row>
     <row r="62" spans="1:13">
       <c r="C62" s="3" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
     </row>
     <row r="63" spans="1:13">
       <c r="C63" s="3" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
     </row>
     <row r="64" spans="1:13" ht="41.4">
       <c r="C64" s="3" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
     </row>
     <row r="65" spans="3:3" ht="27.6">
       <c r="C65" s="3" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
     </row>
     <row r="66" spans="3:3" ht="55.2">
       <c r="C66" s="3" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 4a: Migrate users to PG with dual-write
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA3D979-4615-4F8F-B582-D01139380743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFC3382-B59F-4EC5-9C43-108C845F3AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="723">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -4162,6 +4162,21 @@
   </si>
   <si>
     <t>להפריד שאלות לדוגמה לסטייג'ס</t>
+  </si>
+  <si>
+    <t>responsibilty</t>
+  </si>
+  <si>
+    <t>כולל התאמה לאייפון אנדרואיד וכו'</t>
+  </si>
+  <si>
+    <t>יש הצפנות דרך railway, אבל צריך להפריד טבלאות כך שגם אם ייפרץ - יתן כמה שפחות מידע: להימנע משמירת מידע מיותר ולהפריד מידע מפרטים אישיים של המשתמש. לחשוב מה עוד</t>
+  </si>
+  <si>
+    <t>לוודא שאכן הוא יכול לדבר רק דרך פלט בטוח ואין לו גישה לנתונים רגישים שנותחו.  לעשות דשבורד למשתמשים שיוכלו לראות איזה פרטים עליהם הם בטוחים כדי להציג בכרטיס התאמה אולי.</t>
+  </si>
+  <si>
+    <t>קיים בrailway, מורכב של postgreSQL</t>
   </si>
 </sst>
 </file>
@@ -4872,6 +4887,9 @@
       <c r="C6" t="s">
         <v>405</v>
       </c>
+      <c r="D6" t="s">
+        <v>722</v>
+      </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
@@ -4981,15 +4999,18 @@
         <v>502</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>415</v>
       </c>
       <c r="B17" t="s">
         <v>508</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="D17" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>674</v>
       </c>
@@ -4997,7 +5018,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>415</v>
       </c>
@@ -5005,7 +5026,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>415</v>
       </c>
@@ -5013,7 +5034,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>506</v>
       </c>
@@ -5021,32 +5042,38 @@
         <v>507</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="D23" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="D24" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>677</v>
       </c>
@@ -8053,7 +8080,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="38" customWidth="1"/>
@@ -8063,24 +8090,24 @@
     <col min="5" max="5" width="35.6640625" style="5" customWidth="1"/>
     <col min="6" max="6" width="29.5546875" style="5" customWidth="1"/>
     <col min="7" max="7" width="59" style="5" customWidth="1"/>
-    <col min="10" max="10" width="12.109375" customWidth="1"/>
-    <col min="11" max="11" width="17.77734375" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="15.33203125" customWidth="1"/>
-    <col min="14" max="14" width="40.6640625" customWidth="1"/>
+    <col min="10" max="11" width="12.109375" customWidth="1"/>
+    <col min="12" max="12" width="17.77734375" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="15.33203125" customWidth="1"/>
+    <col min="15" max="15" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="C1" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:15">
       <c r="C2" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="27.6">
+    <row r="4" spans="1:15" ht="27.6">
       <c r="A4" s="39" t="s">
         <v>6</v>
       </c>
@@ -8112,19 +8139,22 @@
         <v>62</v>
       </c>
       <c r="K4" s="9" t="s">
+        <v>718</v>
+      </c>
+      <c r="L4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="O4" s="9" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="110.4">
+    <row r="5" spans="1:15" ht="110.4">
       <c r="A5" s="47" t="s">
         <v>426</v>
       </c>
@@ -8149,20 +8179,21 @@
       <c r="J5" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="43" t="s">
+      <c r="K5" s="43"/>
+      <c r="L5" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="42">
+      <c r="M5" s="42">
         <v>20</v>
       </c>
-      <c r="M5" s="42" t="s">
+      <c r="N5" s="42" t="s">
         <v>163</v>
       </c>
-      <c r="N5" s="44" t="s">
+      <c r="O5" s="44" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="55.2">
+    <row r="6" spans="1:15" ht="55.2">
       <c r="A6" s="49" t="s">
         <v>441</v>
       </c>
@@ -8189,12 +8220,15 @@
       <c r="J6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="2"/>
+      <c r="K6" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L6" s="3"/>
       <c r="M6" s="2"/>
-      <c r="N6" s="21"/>
-    </row>
-    <row r="7" spans="1:14" ht="317.39999999999998">
+      <c r="N6" s="2"/>
+      <c r="O6" s="21"/>
+    </row>
+    <row r="7" spans="1:15" ht="317.39999999999998">
       <c r="A7" s="40"/>
       <c r="B7" s="2" t="s">
         <v>434</v>
@@ -8219,14 +8253,17 @@
       <c r="J7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="3"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2" t="s">
+      <c r="K7" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2" t="s">
         <v>482</v>
       </c>
-      <c r="N7" s="21"/>
-    </row>
-    <row r="8" spans="1:14" ht="220.8">
+      <c r="O7" s="21"/>
+    </row>
+    <row r="8" spans="1:15" ht="220.8">
       <c r="A8" s="2" t="s">
         <v>440</v>
       </c>
@@ -8254,13 +8291,16 @@
         <v>8</v>
       </c>
       <c r="K8" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="151.80000000000001">
+    <row r="9" spans="1:15" ht="151.80000000000001">
       <c r="A9" s="2" t="s">
         <v>601</v>
       </c>
@@ -8285,10 +8325,13 @@
         <v>5</v>
       </c>
       <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="M9" s="2"/>
-    </row>
-    <row r="10" spans="1:14" ht="96.6">
+      <c r="K9" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L9" s="3"/>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="96.6">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
@@ -8315,12 +8358,13 @@
       <c r="J10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="3"/>
+      <c r="L10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M10" s="2"/>
-    </row>
-    <row r="11" spans="1:14" ht="138">
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" ht="138">
       <c r="A11" s="52" t="s">
         <v>607</v>
       </c>
@@ -8348,9 +8392,10 @@
       </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="M11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" ht="220.8">
+      <c r="L11" s="3"/>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" ht="220.8">
       <c r="A12" t="s">
         <v>614</v>
       </c>
@@ -8377,8 +8422,9 @@
       <c r="J12" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="138">
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:15" ht="138">
       <c r="A13" s="2" t="s">
         <v>49</v>
       </c>
@@ -8405,15 +8451,18 @@
       <c r="J13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K13" s="2"/>
-      <c r="M13" s="2" t="s">
+      <c r="K13" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L13" s="2"/>
+      <c r="N13" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="110.4">
+    <row r="14" spans="1:15" ht="110.4">
       <c r="A14" s="40"/>
       <c r="B14" s="2" t="s">
         <v>424</v>
@@ -8430,10 +8479,13 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="M14" s="2"/>
-    </row>
-    <row r="15" spans="1:14" ht="138">
+      <c r="K14" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L14" s="3"/>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" ht="138">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -8461,13 +8513,16 @@
         <v>8</v>
       </c>
       <c r="K15" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="N15" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="193.2">
+    <row r="16" spans="1:15" ht="193.2">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
@@ -8496,10 +8551,13 @@
       <c r="J16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K16" s="2"/>
-      <c r="M16" s="2"/>
-    </row>
-    <row r="17" spans="1:14" ht="110.4">
+      <c r="K16" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L16" s="2"/>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:15" ht="110.4">
       <c r="A17" s="2" t="s">
         <v>429</v>
       </c>
@@ -8529,11 +8587,14 @@
         <v>8</v>
       </c>
       <c r="K17" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M17" s="2"/>
-    </row>
-    <row r="18" spans="1:14" ht="165.6">
+      <c r="N17" s="2"/>
+    </row>
+    <row r="18" spans="1:15" ht="165.6">
       <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
@@ -8559,16 +8620,19 @@
         <v>8</v>
       </c>
       <c r="K18" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="N18" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="N18" s="5" t="s">
+      <c r="O18" s="5" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="43.2">
+    <row r="19" spans="1:15" ht="43.2">
       <c r="A19" s="2" t="s">
         <v>620</v>
       </c>
@@ -8591,11 +8655,14 @@
         <v>6</v>
       </c>
       <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="5"/>
-    </row>
-    <row r="20" spans="1:14" ht="110.4">
+      <c r="K19" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L19" s="3"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="5"/>
+    </row>
+    <row r="20" spans="1:15" ht="110.4">
       <c r="A20" s="2" t="s">
         <v>616</v>
       </c>
@@ -8625,13 +8692,16 @@
         <v>14</v>
       </c>
       <c r="K20" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="43.2">
+    <row r="21" spans="1:15" ht="43.2">
       <c r="A21" s="2" t="s">
         <v>617</v>
       </c>
@@ -8650,10 +8720,13 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="3"/>
-      <c r="K21" s="2"/>
-      <c r="M21" s="2"/>
-    </row>
-    <row r="22" spans="1:14" ht="248.4">
+      <c r="K21" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L21" s="2"/>
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" ht="248.4">
       <c r="A22" s="49" t="s">
         <v>47</v>
       </c>
@@ -8680,10 +8753,11 @@
       <c r="J22" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:14" ht="207">
+      <c r="K22" s="3"/>
+      <c r="L22" s="2"/>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" ht="207">
       <c r="A23" s="2" t="s">
         <v>347</v>
       </c>
@@ -8713,11 +8787,14 @@
         <v>8</v>
       </c>
       <c r="K23" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M23" s="2"/>
-    </row>
-    <row r="24" spans="1:14" ht="82.8">
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:15" ht="82.8">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -8742,12 +8819,13 @@
       <c r="J24" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="K24" s="3"/>
+      <c r="L24" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:14" ht="124.2">
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:15" ht="124.2">
       <c r="A25" s="2" t="s">
         <v>27</v>
       </c>
@@ -8775,11 +8853,14 @@
         <v>8</v>
       </c>
       <c r="K25" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="1:14" ht="193.2">
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:15" ht="193.2">
       <c r="A26" s="2" t="s">
         <v>35</v>
       </c>
@@ -8806,15 +8887,16 @@
       <c r="J26" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K26" s="3" t="s">
+      <c r="K26" s="3"/>
+      <c r="L26" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M26" s="2"/>
-      <c r="N26" t="s">
+      <c r="N26" s="2"/>
+      <c r="O26" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="55.2">
+    <row r="27" spans="1:15" ht="55.2">
       <c r="B27" s="2" t="s">
         <v>438</v>
       </c>
@@ -8838,8 +8920,9 @@
       <c r="J27" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="55.2">
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="1:15" ht="55.2">
       <c r="B28" s="2" t="s">
         <v>438</v>
       </c>
@@ -8861,8 +8944,9 @@
         <v>3</v>
       </c>
       <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:14" ht="124.2">
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="1:15" ht="124.2">
       <c r="A29" s="49" t="s">
         <v>40</v>
       </c>
@@ -8887,10 +8971,13 @@
       <c r="J29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K29" s="2"/>
-      <c r="M29" s="2"/>
-    </row>
-    <row r="30" spans="1:14" ht="82.8">
+      <c r="K29" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L29" s="2"/>
+      <c r="N29" s="2"/>
+    </row>
+    <row r="30" spans="1:15" ht="82.8">
       <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
@@ -8917,10 +9004,11 @@
       <c r="J30" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K30" s="2"/>
-      <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="1:14" ht="138">
+      <c r="K30" s="3"/>
+      <c r="L30" s="2"/>
+      <c r="N30" s="2"/>
+    </row>
+    <row r="31" spans="1:15" ht="138">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
@@ -8949,10 +9037,11 @@
       <c r="J31" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K31" s="2"/>
-      <c r="M31" s="2"/>
-    </row>
-    <row r="32" spans="1:14" ht="151.80000000000001">
+      <c r="K31" s="3"/>
+      <c r="L31" s="2"/>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="32" spans="1:15" ht="151.80000000000001">
       <c r="A32" s="2" t="s">
         <v>17</v>
       </c>
@@ -8981,14 +9070,15 @@
       <c r="J32" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="K32" s="3"/>
+      <c r="L32" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="N32" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="262.2">
+    <row r="33" spans="1:15" ht="262.2">
       <c r="A33" s="2" t="s">
         <v>51</v>
       </c>
@@ -9013,10 +9103,11 @@
       <c r="J33" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K33" s="2"/>
-      <c r="M33" s="2"/>
-    </row>
-    <row r="34" spans="1:14" ht="193.2">
+      <c r="K33" s="3"/>
+      <c r="L33" s="2"/>
+      <c r="N33" s="2"/>
+    </row>
+    <row r="34" spans="1:15" ht="193.2">
       <c r="B34" s="2" t="s">
         <v>436</v>
       </c>
@@ -9038,8 +9129,9 @@
       <c r="J34" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" ht="207">
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" spans="1:15" ht="207">
       <c r="B35" s="2" t="s">
         <v>438</v>
       </c>
@@ -9063,8 +9155,9 @@
       <c r="J35" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" ht="207">
+      <c r="K35" s="3"/>
+    </row>
+    <row r="36" spans="1:15" ht="207">
       <c r="A36" s="2" t="s">
         <v>53</v>
       </c>
@@ -9087,12 +9180,13 @@
       <c r="J36" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="K36" s="3"/>
+      <c r="L36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="M36" s="2"/>
-    </row>
-    <row r="37" spans="1:14" ht="124.2">
+      <c r="N36" s="2"/>
+    </row>
+    <row r="37" spans="1:15" ht="124.2">
       <c r="B37" s="2" t="s">
         <v>434</v>
       </c>
@@ -9116,8 +9210,9 @@
       <c r="J37" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" ht="151.80000000000001">
+      <c r="K37" s="3"/>
+    </row>
+    <row r="38" spans="1:15" ht="151.80000000000001">
       <c r="B38" s="2" t="s">
         <v>434</v>
       </c>
@@ -9141,8 +9236,9 @@
       <c r="J38" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" ht="165.6">
+      <c r="K38" s="3"/>
+    </row>
+    <row r="39" spans="1:15" ht="165.6">
       <c r="B39" s="2" t="s">
         <v>434</v>
       </c>
@@ -9166,8 +9262,9 @@
       <c r="J39" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" ht="179.4">
+      <c r="K39" s="3"/>
+    </row>
+    <row r="40" spans="1:15" ht="179.4">
       <c r="A40" s="51"/>
       <c r="B40" s="41" t="s">
         <v>434</v>
@@ -9192,8 +9289,9 @@
       <c r="J40" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" ht="248.4">
+      <c r="K40" s="3"/>
+    </row>
+    <row r="41" spans="1:15" ht="248.4">
       <c r="A41" s="2" t="s">
         <v>60</v>
       </c>
@@ -9220,12 +9318,13 @@
       <c r="J41" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="K41" s="3"/>
+      <c r="L41" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="M41" s="2"/>
-    </row>
-    <row r="42" spans="1:14" ht="110.4">
+      <c r="N41" s="2"/>
+    </row>
+    <row r="42" spans="1:15" ht="110.4">
       <c r="A42" s="2" t="s">
         <v>120</v>
       </c>
@@ -9252,11 +9351,12 @@
       <c r="J42" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K42" s="3" t="s">
+      <c r="K42" s="3"/>
+      <c r="L42" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="138">
+    <row r="43" spans="1:15" ht="138">
       <c r="A43" s="2" t="s">
         <v>277</v>
       </c>
@@ -9281,14 +9381,17 @@
         <v>9</v>
       </c>
       <c r="K43" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L43" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="M43" s="19"/>
-      <c r="N43" s="3" t="s">
+      <c r="N43" s="19"/>
+      <c r="O43" s="3" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="409.6">
+    <row r="44" spans="1:15" ht="409.6">
       <c r="A44" s="40" t="s">
         <v>275</v>
       </c>
@@ -9314,11 +9417,14 @@
         <v>9</v>
       </c>
       <c r="K44" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="L44" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="N44" s="34"/>
-    </row>
-    <row r="45" spans="1:14" ht="409.6">
+      <c r="O44" s="34"/>
+    </row>
+    <row r="45" spans="1:15" ht="409.6">
       <c r="B45" s="2" t="s">
         <v>439</v>
       </c>
@@ -9340,326 +9446,341 @@
       <c r="J45" t="s">
         <v>14</v>
       </c>
-      <c r="K45" s="3" t="s">
+      <c r="L45" s="3" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
-      <c r="C47" s="36" t="s">
+    <row r="46" spans="1:15">
+      <c r="B46" s="2"/>
+      <c r="C46" s="3"/>
+      <c r="H46" s="2"/>
+      <c r="L46" s="3"/>
+    </row>
+    <row r="67" spans="1:15">
+      <c r="C67" s="36" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="69">
-      <c r="A48" s="40" t="s">
+    <row r="68" spans="1:15" ht="69">
+      <c r="A68" s="40" t="s">
         <v>334</v>
       </c>
-      <c r="B48" s="2"/>
-      <c r="C48" s="3" t="s">
+      <c r="B68" s="2"/>
+      <c r="C68" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="D48" s="3" t="s">
+      <c r="D68" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="2">
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="2">
         <v>0.7</v>
       </c>
-      <c r="I48" s="2">
+      <c r="I68" s="2">
         <v>8</v>
       </c>
-      <c r="J48" s="3" t="s">
+      <c r="J68" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K48" s="3" t="s">
+      <c r="K68" s="3"/>
+      <c r="L68" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="L48" s="3" t="s">
+      <c r="M68" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="M48" s="3" t="s">
+      <c r="N68" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="N48" s="3" t="s">
+      <c r="O68" s="3" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="27.6">
-      <c r="A49" s="40" t="s">
+    <row r="69" spans="1:15" ht="27.6">
+      <c r="A69" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B49" s="2"/>
-      <c r="C49" s="3" t="s">
+      <c r="B69" s="2"/>
+      <c r="C69" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D69" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="2">
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="2">
         <v>0.5</v>
       </c>
-      <c r="I49" s="2">
+      <c r="I69" s="2">
         <v>5</v>
       </c>
-      <c r="J49" s="3" t="s">
+      <c r="J69" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K49" s="3" t="s">
+      <c r="K69" s="3"/>
+      <c r="L69" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="55.2">
-      <c r="A50" s="40" t="s">
+    <row r="70" spans="1:15" ht="55.2">
+      <c r="A70" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B50" s="2"/>
-      <c r="C50" s="3" t="s">
+      <c r="B70" s="2"/>
+      <c r="C70" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D50" s="3" t="s">
+      <c r="D70" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="2">
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="2">
         <v>0.6</v>
       </c>
-      <c r="I50" s="2">
+      <c r="I70" s="2">
         <v>5</v>
       </c>
-      <c r="J50" s="3" t="s">
+      <c r="J70" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K50" s="3" t="s">
+      <c r="K70" s="3"/>
+      <c r="L70" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M50" s="2"/>
-    </row>
-    <row r="51" spans="1:13" ht="41.4">
-      <c r="A51" s="40" t="s">
+      <c r="N70" s="2"/>
+    </row>
+    <row r="71" spans="1:15" ht="41.4">
+      <c r="A71" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B71" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C71" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D51" s="3" t="s">
+      <c r="D71" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="2">
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="H71" s="2">
         <v>0.5</v>
       </c>
-      <c r="I51" s="2">
+      <c r="I71" s="2">
         <v>4</v>
       </c>
-      <c r="J51" s="3" t="s">
+      <c r="J71" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K51" s="3" t="s">
+      <c r="K71" s="3"/>
+      <c r="L71" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M51" s="2"/>
-    </row>
-    <row r="52" spans="1:13" ht="27.6">
-      <c r="A52" s="40" t="s">
+      <c r="N71" s="2"/>
+    </row>
+    <row r="72" spans="1:15" ht="27.6">
+      <c r="A72" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B72" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C72" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D52" s="3" t="s">
+      <c r="D72" s="3" t="s">
         <v>443</v>
       </c>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="2">
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="2">
         <v>0.3</v>
       </c>
-      <c r="I52" s="2">
+      <c r="I72" s="2">
         <v>4</v>
       </c>
-      <c r="J52" s="3" t="s">
+      <c r="J72" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K52" s="2"/>
-    </row>
-    <row r="53" spans="1:13" ht="151.80000000000001">
-      <c r="B53" s="2" t="s">
+      <c r="K72" s="3"/>
+      <c r="L72" s="2"/>
+    </row>
+    <row r="73" spans="1:15" ht="151.80000000000001">
+      <c r="B73" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C73" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D73" s="3" t="s">
         <v>551</v>
       </c>
-      <c r="E53" s="33" t="s">
+      <c r="E73" s="33" t="s">
         <v>552</v>
       </c>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="2">
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="H73" s="2">
         <v>0.2</v>
       </c>
-      <c r="I53" s="2">
+      <c r="I73" s="2">
         <v>2</v>
       </c>
-      <c r="J53" s="3" t="s">
+      <c r="J73" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="54" spans="1:13" ht="165.6">
-      <c r="B54" s="2" t="s">
+      <c r="K73" s="3"/>
+    </row>
+    <row r="74" spans="1:15" ht="165.6">
+      <c r="B74" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C74" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="D74" s="3" t="s">
         <v>555</v>
       </c>
-      <c r="E54" s="33" t="s">
+      <c r="E74" s="33" t="s">
         <v>556</v>
       </c>
-      <c r="F54" s="33" t="s">
+      <c r="F74" s="33" t="s">
         <v>557</v>
       </c>
-      <c r="G54" s="3"/>
-      <c r="H54" s="2">
+      <c r="G74" s="3"/>
+      <c r="H74" s="2">
         <v>0.2</v>
       </c>
-      <c r="I54" s="2">
+      <c r="I74" s="2">
         <v>3</v>
       </c>
-      <c r="J54" s="3" t="s">
+      <c r="J74" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="55" spans="1:13" ht="82.8">
-      <c r="B55" s="2" t="s">
+      <c r="K74" s="3"/>
+    </row>
+    <row r="75" spans="1:15" ht="82.8">
+      <c r="B75" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C75" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D75" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3" t="s">
+      <c r="E75" s="3"/>
+      <c r="F75" s="3" t="s">
         <v>550</v>
       </c>
-      <c r="G55" s="3"/>
-      <c r="H55" s="2">
+      <c r="G75" s="3"/>
+      <c r="H75" s="2">
         <v>0.2</v>
       </c>
-      <c r="I55" s="2">
+      <c r="I75" s="2">
         <v>3</v>
       </c>
-      <c r="J55" s="3" t="s">
+      <c r="J75" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="M55" s="2"/>
-    </row>
-    <row r="56" spans="1:13" ht="27.6">
-      <c r="B56" s="2" t="s">
+      <c r="K75" s="3"/>
+      <c r="N75" s="2"/>
+    </row>
+    <row r="76" spans="1:15" ht="27.6">
+      <c r="B76" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="C56" s="17" t="s">
+      <c r="C76" s="17" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="110.4">
-      <c r="A57" s="2" t="s">
+    <row r="77" spans="1:15" ht="110.4">
+      <c r="A77" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B77" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D57" s="3" t="s">
+      <c r="D77" s="3" t="s">
         <v>579</v>
       </c>
-      <c r="E57" s="33" t="s">
+      <c r="E77" s="33" t="s">
         <v>543</v>
       </c>
-      <c r="F57" s="33" t="s">
+      <c r="F77" s="33" t="s">
         <v>577</v>
       </c>
-      <c r="G57" s="3"/>
-      <c r="H57" s="2">
+      <c r="G77" s="3"/>
+      <c r="H77" s="2">
         <v>0.6</v>
       </c>
-      <c r="I57" s="2">
+      <c r="I77" s="2">
         <v>4</v>
       </c>
-      <c r="J57" s="3" t="s">
+      <c r="J77" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K57" s="2"/>
-      <c r="M57" s="2"/>
-    </row>
-    <row r="58" spans="1:13">
-      <c r="C58" s="3" t="s">
+      <c r="K77" s="3"/>
+      <c r="L77" s="2"/>
+      <c r="N77" s="2"/>
+    </row>
+    <row r="78" spans="1:15">
+      <c r="C78" s="3" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="59" spans="1:13">
-      <c r="C59" s="3" t="s">
+    <row r="79" spans="1:15">
+      <c r="C79" s="3" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="60" spans="1:13">
-      <c r="C60" s="3" t="s">
+    <row r="80" spans="1:15">
+      <c r="C80" s="3" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="27.6">
-      <c r="C61" s="3" t="s">
+    <row r="81" spans="3:4" ht="27.6">
+      <c r="C81" s="3" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="62" spans="1:13">
-      <c r="C62" s="3" t="s">
+    <row r="82" spans="3:4">
+      <c r="C82" s="3" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="63" spans="1:13">
-      <c r="C63" s="3" t="s">
+    <row r="83" spans="3:4">
+      <c r="C83" s="3" t="s">
         <v>703</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D83" s="5" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="41.4">
-      <c r="C64" s="3" t="s">
+    <row r="84" spans="3:4" ht="41.4">
+      <c r="C84" s="3" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="65" spans="3:3" ht="27.6">
-      <c r="C65" s="3" t="s">
+    <row r="85" spans="3:4" ht="27.6">
+      <c r="C85" s="3" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="66" spans="3:3" ht="55.2">
-      <c r="C66" s="3" t="s">
+    <row r="86" spans="3:4" ht="55.2">
+      <c r="C86" s="3" t="s">
         <v>707</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Configure production build for single-service deploy
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFC3382-B59F-4EC5-9C43-108C845F3AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F3FB5B-31B6-4A8A-99F6-CBA9FD61CA17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="723">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="747">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -4177,6 +4177,78 @@
   </si>
   <si>
     <t>קיים בrailway, מורכב של postgreSQL</t>
+  </si>
+  <si>
+    <t>Emotional Intensity</t>
+  </si>
+  <si>
+    <t>Communication Softness</t>
+  </si>
+  <si>
+    <t>Tonal Balance</t>
+  </si>
+  <si>
+    <t>שילוב</t>
+  </si>
+  <si>
+    <t>Tonal Stability</t>
+  </si>
+  <si>
+    <t>Depth Authenticity</t>
+  </si>
+  <si>
+    <t>Cliché Density</t>
+  </si>
+  <si>
+    <t>Authenticity</t>
+  </si>
+  <si>
+    <t>Communication Style</t>
+  </si>
+  <si>
+    <t>לא ברור מה הרמות פה</t>
+  </si>
+  <si>
+    <t>Refinement Level</t>
+  </si>
+  <si>
+    <t>Cognitive Signal in Humor</t>
+  </si>
+  <si>
+    <t>Humor Depth</t>
+  </si>
+  <si>
+    <t>Signal Coherence</t>
+  </si>
+  <si>
+    <t>Verbal Precision</t>
+  </si>
+  <si>
+    <t>Depth of Expression</t>
+  </si>
+  <si>
+    <t>Emotional Authenticity</t>
+  </si>
+  <si>
+    <t>Multi-Dimensionality</t>
+  </si>
+  <si>
+    <t>Intent Expression Style</t>
+  </si>
+  <si>
+    <t>Communication Clarity</t>
+  </si>
+  <si>
+    <t>Communication Structure</t>
+  </si>
+  <si>
+    <t>Communication Refinement</t>
+  </si>
+  <si>
+    <t>Cultural / Style Signal</t>
+  </si>
+  <si>
+    <t>גם כאן לא ברור מה הרמות</t>
   </si>
 </sst>
 </file>
@@ -8080,7 +8152,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O108"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="38" customWidth="1"/>
@@ -9751,17 +9823,17 @@
         <v>700</v>
       </c>
     </row>
-    <row r="81" spans="3:4" ht="27.6">
+    <row r="81" spans="3:5" ht="27.6">
       <c r="C81" s="3" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="82" spans="3:4">
+    <row r="82" spans="3:5">
       <c r="C82" s="3" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="83" spans="3:4">
+    <row r="83" spans="3:5">
       <c r="C83" s="3" t="s">
         <v>703</v>
       </c>
@@ -9769,19 +9841,138 @@
         <v>704</v>
       </c>
     </row>
-    <row r="84" spans="3:4" ht="41.4">
+    <row r="84" spans="3:5" ht="41.4">
       <c r="C84" s="3" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="85" spans="3:4" ht="27.6">
+    <row r="85" spans="3:5" ht="27.6">
       <c r="C85" s="3" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="86" spans="3:4" ht="55.2">
+    <row r="86" spans="3:5" ht="55.2">
       <c r="C86" s="3" t="s">
         <v>707</v>
+      </c>
+    </row>
+    <row r="87" spans="3:5">
+      <c r="D87" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="88" spans="3:5">
+      <c r="D88" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="89" spans="3:5">
+      <c r="D89" t="s">
+        <v>725</v>
+      </c>
+      <c r="E89" s="5" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="90" spans="3:5">
+      <c r="D90" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="91" spans="3:5">
+      <c r="D91" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="92" spans="3:5">
+      <c r="D92" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="93" spans="3:5">
+      <c r="D93" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="94" spans="3:5">
+      <c r="D94" t="s">
+        <v>731</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="95" spans="3:5">
+      <c r="D95" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="96" spans="3:5">
+      <c r="D96" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="97" spans="4:5">
+      <c r="D97" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="98" spans="4:5">
+      <c r="D98" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="99" spans="4:5">
+      <c r="D99" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="100" spans="4:5">
+      <c r="D100" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="101" spans="4:5">
+      <c r="D101" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="102" spans="4:5">
+      <c r="D102" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="103" spans="4:5">
+      <c r="D103" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="104" spans="4:5">
+      <c r="D104" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="105" spans="4:5">
+      <c r="D105" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="106" spans="4:5">
+      <c r="D106" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="107" spans="4:5">
+      <c r="D107" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="108" spans="4:5">
+      <c r="D108" t="s">
+        <v>745</v>
+      </c>
+      <c r="E108" s="5" t="s">
+        <v>746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
last commit before profiles split
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC5BE17-AEB0-4852-AFCB-9947326E2580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5207FE-9385-4B26-B01B-82819AC295A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="815">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3033,6 +3033,9 @@
 - low self-awareness
 - impression management
 - or limited introspection</t>
+  </si>
+  <si>
+    <t>מידת חילוניות</t>
   </si>
 </sst>
 </file>
@@ -5759,7 +5762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
@@ -6866,19 +6869,16 @@
         <v>799</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="69">
+    <row r="60" spans="1:11">
       <c r="A60" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>787</v>
       </c>
-      <c r="C60" s="38"/>
-      <c r="D60" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>792</v>
+      <c r="C60" s="2"/>
+      <c r="D60" s="17" t="s">
+        <v>814</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="69">
@@ -6890,13 +6890,13 @@
       </c>
       <c r="C61" s="38"/>
       <c r="D61" s="3" t="s">
-        <v>422</v>
+        <v>383</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="27.6">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="69">
       <c r="A62" s="2" t="s">
         <v>425</v>
       </c>
@@ -6905,38 +6905,39 @@
       </c>
       <c r="C62" s="38"/>
       <c r="D62" s="3" t="s">
-        <v>334</v>
+        <v>422</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="82.8">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="27.6">
       <c r="A63" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>787</v>
       </c>
-      <c r="D63" s="33" t="s">
+      <c r="C63" s="38"/>
+      <c r="D63" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="82.8">
+      <c r="A64" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="D64" s="33" t="s">
         <v>387</v>
       </c>
-      <c r="E63" s="33" t="s">
+      <c r="E64" s="33" t="s">
         <v>795</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11">
-      <c r="A64" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -6946,25 +6947,25 @@
       <c r="B65" s="3" t="s">
         <v>800</v>
       </c>
-      <c r="C65" t="s">
-        <v>801</v>
-      </c>
-      <c r="D65" s="56" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="28.8">
+      <c r="C65" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>800</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>561</v>
+      <c r="C66" t="s">
+        <v>801</v>
+      </c>
+      <c r="D66" s="56" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="28.8">
@@ -6975,16 +6976,13 @@
         <v>800</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>48</v>
+        <v>560</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="82.8">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="28.8">
       <c r="A68" s="2" t="s">
         <v>430</v>
       </c>
@@ -6992,16 +6990,16 @@
         <v>800</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>802</v>
+        <v>48</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="69">
+        <v>49</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="82.8">
       <c r="A69" s="2" t="s">
         <v>430</v>
       </c>
@@ -7009,16 +7007,16 @@
         <v>800</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>114</v>
+        <v>56</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="55.2">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="69">
       <c r="A70" s="2" t="s">
         <v>430</v>
       </c>
@@ -7026,16 +7024,16 @@
         <v>800</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>541</v>
+        <v>114</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="409.6">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="55.2">
       <c r="A71" s="2" t="s">
         <v>430</v>
       </c>
@@ -7043,12 +7041,29 @@
         <v>800</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="409.6">
+      <c r="A72" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="C72" s="2" t="s">
         <v>808</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="D72" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="E71" s="3" t="s">
+      <c r="E72" s="3" t="s">
         <v>700</v>
       </c>
     </row>

</xml_diff>

<commit_message>
last version before cognitive seperation
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5207FE-9385-4B26-B01B-82819AC295A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EFD0DB-0246-4060-9A44-E66728482D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,6 @@
     <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -52,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="808">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -2814,45 +2813,15 @@
     <t>רוחניות</t>
   </si>
   <si>
-    <t>Analytical Thinking</t>
-  </si>
-  <si>
     <t>Abstract Thinking</t>
   </si>
   <si>
     <t>Cognitive Flexibility</t>
   </si>
   <si>
-    <t>Verbal Reasoning</t>
-  </si>
-  <si>
-    <t>Depth of Thought</t>
-  </si>
-  <si>
-    <t>Intellectual Openness</t>
-  </si>
-  <si>
-    <t>Conceptual Clarity</t>
-  </si>
-  <si>
-    <t>Pattern Recognition</t>
-  </si>
-  <si>
-    <t>זיהוי דפוסים</t>
-  </si>
-  <si>
     <t>בהירות מושגית</t>
   </si>
   <si>
-    <t>פתיחות אינטלקטואלית</t>
-  </si>
-  <si>
-    <t>עומק מחשבתי</t>
-  </si>
-  <si>
-    <t>הסקה מילולית</t>
-  </si>
-  <si>
     <t>גמישות מחשבתית</t>
   </si>
   <si>
@@ -2866,9 +2835,6 @@
   </si>
   <si>
     <t>Intellectualism</t>
-  </si>
-  <si>
-    <t>Verbal Expression Ability</t>
   </si>
   <si>
     <t>Directness</t>
@@ -3015,17 +2981,6 @@
 - indirect expression (e.g. sarcasm)</t>
   </si>
   <si>
-    <t>Analytical Thinking should be based on evidence of structured reasoning:
-- breaking down situations into components
-- explaining cause and effect
-- identifying mechanisms or underlying structure
-Do NOT base this trait on:
-- general clarity
-- emotional understanding
-- social reasoning
-- politeness or balanced answers</t>
-  </si>
-  <si>
     <t>Self-awareness is indicated by the ability to recognize and articulate one's own weaknesses, emotional patterns, and internal conflicts.
 Users who openly describe their own flaws, reactivity, or emotional struggles should be scored higher in self-awareness.
 Do NOT assume that a user who presents only positive, balanced, or socially desirable responses has high self-awareness.
@@ -3036,6 +2991,21 @@
   </si>
   <si>
     <t>מידת חילוניות</t>
+  </si>
+  <si>
+    <t>Analytical Reasoning</t>
+  </si>
+  <si>
+    <t>Conceptual Precision</t>
+  </si>
+  <si>
+    <t>Verbal Articulation</t>
+  </si>
+  <si>
+    <t>אינטיליגנציה חברתית-אינטואיטיבית</t>
+  </si>
+  <si>
+    <t>פרופיל אנליטי</t>
   </si>
 </sst>
 </file>
@@ -3242,7 +3212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3389,7 +3359,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5762,7 +5731,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
@@ -5798,7 +5767,7 @@
         <v>413</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>777</v>
+        <v>766</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>6</v>
@@ -5810,7 +5779,7 @@
         <v>59</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>784</v>
+        <v>773</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>3</v>
@@ -5837,22 +5806,20 @@
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="151.80000000000001">
+    <row r="5" spans="1:14" ht="28.8">
       <c r="A5" s="2" t="s">
-        <v>715</v>
+        <v>807</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>778</v>
+        <v>767</v>
       </c>
       <c r="C5" t="s">
-        <v>753</v>
+        <v>803</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>812</v>
-      </c>
+        <v>758</v>
+      </c>
+      <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -5862,16 +5829,16 @@
     </row>
     <row r="6" spans="1:14" ht="28.8">
       <c r="A6" s="2" t="s">
-        <v>715</v>
+        <v>807</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>778</v>
+        <v>767</v>
       </c>
       <c r="C6" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>767</v>
+        <v>757</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -5883,16 +5850,16 @@
     </row>
     <row r="7" spans="1:14" ht="28.8">
       <c r="A7" s="2" t="s">
-        <v>715</v>
+        <v>807</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>778</v>
+        <v>767</v>
       </c>
       <c r="C7" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>766</v>
+        <v>756</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -5904,16 +5871,16 @@
     </row>
     <row r="8" spans="1:14" ht="28.8">
       <c r="A8" s="2" t="s">
-        <v>715</v>
+        <v>807</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>778</v>
+        <v>767</v>
       </c>
       <c r="C8" t="s">
-        <v>756</v>
+        <v>804</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>765</v>
+        <v>755</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -5923,16 +5890,16 @@
     </row>
     <row r="9" spans="1:14" ht="28.8">
       <c r="A9" s="2" t="s">
-        <v>715</v>
+        <v>807</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C9" t="s">
-        <v>757</v>
+        <v>767</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>805</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>764</v>
+        <v>639</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -5944,14 +5911,10 @@
       <c r="A10" s="2" t="s">
         <v>715</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C10" t="s">
-        <v>758</v>
-      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
       <c r="D10" s="3" t="s">
-        <v>763</v>
+        <v>806</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -5964,13 +5927,13 @@
         <v>715</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C11" t="s">
-        <v>759</v>
+        <v>767</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>760</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>762</v>
+        <v>435</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -5978,37 +5941,40 @@
       <c r="H11" s="3"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="28.8">
+    <row r="12" spans="1:14" ht="331.2">
       <c r="A12" s="2" t="s">
         <v>715</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C12" t="s">
-        <v>760</v>
+        <v>767</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>759</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>761</v>
-      </c>
-      <c r="E12" s="3"/>
+        <v>436</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>798</v>
+      </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="2"/>
+      <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:14" ht="28.8">
       <c r="A13" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>778</v>
+        <v>763</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>765</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>770</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>435</v>
+        <v>665</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>764</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -6016,18 +5982,18 @@
       <c r="H13" s="3"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="28.8">
+    <row r="14" spans="1:14" ht="27.6">
       <c r="A14" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>778</v>
+        <v>763</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>765</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>771</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>639</v>
+        <v>768</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>704</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -6035,135 +6001,132 @@
       <c r="H14" s="3"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:14" ht="28.8">
+    <row r="15" spans="1:14" ht="27.6">
       <c r="A15" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>778</v>
+        <v>763</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>765</v>
       </c>
       <c r="C15" t="s">
-        <v>683</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>711</v>
+        <v>761</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>762</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="H15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:14" ht="331.2">
+    <row r="16" spans="1:14" ht="27.6">
       <c r="A16" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>778</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>769</v>
+        <v>763</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="C16" t="s">
+        <v>666</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>809</v>
-      </c>
+        <v>707</v>
+      </c>
+      <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
+      <c r="H16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" ht="28.8">
+    </row>
+    <row r="17" spans="1:11" ht="27.6">
       <c r="A17" s="2" t="s">
-        <v>774</v>
+        <v>763</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="D17" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="C17" t="s">
+        <v>671</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>775</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
+      <c r="H17" s="2"/>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="2" t="s">
-        <v>774</v>
+        <v>763</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>779</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>704</v>
+        <v>765</v>
+      </c>
+      <c r="C18" t="s">
+        <v>785</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>701</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
-      <c r="J18" s="2"/>
+      <c r="K18" s="34"/>
     </row>
     <row r="19" spans="1:11" ht="27.6">
       <c r="A19" s="2" t="s">
-        <v>774</v>
+        <v>763</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>776</v>
+        <v>765</v>
       </c>
       <c r="C19" t="s">
-        <v>772</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>773</v>
+        <v>786</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>702</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="2"/>
-      <c r="J19" s="2"/>
+      <c r="H19" s="3"/>
+      <c r="K19" s="34"/>
     </row>
     <row r="20" spans="1:11" ht="27.6">
       <c r="A20" s="2" t="s">
-        <v>774</v>
+        <v>763</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>776</v>
+        <v>765</v>
       </c>
       <c r="C20" t="s">
-        <v>666</v>
+        <v>787</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>707</v>
+        <v>22</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="H20" s="2"/>
-      <c r="J20" s="2"/>
-    </row>
-    <row r="21" spans="1:11" ht="27.6">
+      <c r="H20" s="3"/>
+      <c r="K20" s="34"/>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" s="2" t="s">
-        <v>774</v>
+        <v>693</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C21" t="s">
-        <v>671</v>
+        <v>769</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>696</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>786</v>
+        <v>697</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -6171,75 +6134,79 @@
       <c r="H21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="27.6">
+    <row r="22" spans="1:11" ht="28.8">
       <c r="A22" s="2" t="s">
-        <v>774</v>
+        <v>693</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C22" t="s">
-        <v>796</v>
+        <v>769</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>717</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>701</v>
+        <v>643</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="K22" s="34"/>
-    </row>
-    <row r="23" spans="1:11" ht="27.6">
+      <c r="H22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" s="2" t="s">
-        <v>774</v>
+        <v>693</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="C23" t="s">
-        <v>797</v>
+        <v>716</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>702</v>
+        <v>644</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="K23" s="34"/>
-    </row>
-    <row r="24" spans="1:11" ht="27.6">
+      <c r="H23" s="2"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" s="2" t="s">
-        <v>774</v>
+        <v>693</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>776</v>
+        <v>769</v>
       </c>
       <c r="C24" t="s">
-        <v>798</v>
+        <v>718</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>22</v>
+        <v>719</v>
       </c>
       <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="K24" s="34"/>
+      <c r="H24" s="2"/>
+      <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="2" t="s">
         <v>693</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>696</v>
+        <v>769</v>
+      </c>
+      <c r="C25" t="s">
+        <v>720</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>697</v>
+        <v>721</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -6247,823 +6214,743 @@
       <c r="H25" s="2"/>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:11" ht="28.8">
+    <row r="26" spans="1:11">
       <c r="A26" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>780</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>717</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>643</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+        <v>770</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>723</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="E26" s="56" t="s">
+        <v>731</v>
+      </c>
+      <c r="F26" s="56" t="s">
+        <v>425</v>
+      </c>
       <c r="G26" s="3"/>
       <c r="H26" s="2"/>
       <c r="J26" s="2"/>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="C27" s="56" t="s">
-        <v>716</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>644</v>
-      </c>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3" t="s">
-        <v>426</v>
-      </c>
+        <v>725</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="E27" s="56" t="s">
+        <v>730</v>
+      </c>
+      <c r="F27" s="56"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="2"/>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>718</v>
+        <v>727</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>719</v>
-      </c>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3" t="s">
-        <v>426</v>
-      </c>
+        <v>728</v>
+      </c>
+      <c r="E28" s="56" t="s">
+        <v>729</v>
+      </c>
+      <c r="F28" s="56"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="2"/>
-      <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>780</v>
+        <v>770</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>720</v>
+        <v>732</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>721</v>
-      </c>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
+        <v>734</v>
+      </c>
+      <c r="E29" s="56" t="s">
+        <v>737</v>
+      </c>
+      <c r="F29" s="56"/>
       <c r="G29" s="3"/>
-      <c r="H29" s="2"/>
-      <c r="J29" s="2"/>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C30" s="57" t="s">
-        <v>723</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>724</v>
-      </c>
-      <c r="E30" s="57" t="s">
-        <v>731</v>
-      </c>
-      <c r="F30" s="57" t="s">
-        <v>425</v>
-      </c>
+        <v>770</v>
+      </c>
+      <c r="C30" s="56" t="s">
+        <v>733</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="E30" s="56" t="s">
+        <v>736</v>
+      </c>
+      <c r="F30" s="56"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="2"/>
-      <c r="J30" s="2"/>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C31" s="57" t="s">
-        <v>725</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="E31" s="57" t="s">
-        <v>730</v>
-      </c>
-      <c r="F31" s="57"/>
+        <v>770</v>
+      </c>
+      <c r="C31" s="56" t="s">
+        <v>738</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>750</v>
+      </c>
+      <c r="E31" s="56" t="s">
+        <v>739</v>
+      </c>
+      <c r="F31" s="56"/>
       <c r="G31" s="3"/>
-      <c r="J31" s="2"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C32" s="57" t="s">
-        <v>727</v>
+        <v>770</v>
+      </c>
+      <c r="C32" s="56" t="s">
+        <v>544</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>728</v>
-      </c>
-      <c r="E32" s="57" t="s">
-        <v>729</v>
-      </c>
-      <c r="F32" s="57"/>
+        <v>543</v>
+      </c>
+      <c r="E32" s="56" t="s">
+        <v>740</v>
+      </c>
+      <c r="F32" s="56"/>
       <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="J32" s="2"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C33" s="57" t="s">
-        <v>732</v>
+        <v>770</v>
+      </c>
+      <c r="C33" s="56" t="s">
+        <v>743</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>734</v>
-      </c>
-      <c r="E33" s="57" t="s">
-        <v>737</v>
-      </c>
-      <c r="F33" s="57"/>
+        <v>742</v>
+      </c>
+      <c r="E33" s="56" t="s">
+        <v>741</v>
+      </c>
+      <c r="F33" s="56"/>
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C34" s="57" t="s">
-        <v>733</v>
+        <v>770</v>
+      </c>
+      <c r="C34" s="56" t="s">
+        <v>744</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>735</v>
-      </c>
-      <c r="E34" s="57" t="s">
-        <v>736</v>
-      </c>
-      <c r="F34" s="57"/>
+        <v>745</v>
+      </c>
+      <c r="E34" s="56" t="s">
+        <v>748</v>
+      </c>
+      <c r="F34" s="56"/>
       <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C35" s="57" t="s">
-        <v>738</v>
+        <v>770</v>
+      </c>
+      <c r="C35" s="56" t="s">
+        <v>746</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>750</v>
-      </c>
-      <c r="E35" s="57" t="s">
-        <v>739</v>
-      </c>
-      <c r="F35" s="57"/>
+        <v>747</v>
+      </c>
+      <c r="E35" s="56" t="s">
+        <v>749</v>
+      </c>
+      <c r="F35" s="56"/>
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="2" t="s">
-        <v>782</v>
+        <v>771</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C36" s="57" t="s">
-        <v>544</v>
+        <v>770</v>
+      </c>
+      <c r="C36" s="56" t="s">
+        <v>751</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="E36" s="57" t="s">
-        <v>740</v>
-      </c>
-      <c r="F36" s="57"/>
+        <v>752</v>
+      </c>
       <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="J36" s="2"/>
-    </row>
-    <row r="37" spans="1:11">
+    </row>
+    <row r="37" spans="1:11" ht="28.8">
       <c r="A37" s="2" t="s">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C37" s="57" t="s">
-        <v>743</v>
+        <v>772</v>
+      </c>
+      <c r="C37" s="49" t="s">
+        <v>432</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>742</v>
-      </c>
-      <c r="E37" s="57" t="s">
-        <v>741</v>
-      </c>
-      <c r="F37" s="57"/>
+        <v>414</v>
+      </c>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
       <c r="G37" s="3"/>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" ht="220.8">
       <c r="A38" s="2" t="s">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C38" s="57" t="s">
-        <v>744</v>
+        <v>772</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>745</v>
-      </c>
-      <c r="E38" s="57" t="s">
-        <v>748</v>
-      </c>
-      <c r="F38" s="57"/>
+        <v>29</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:11" ht="28.8">
       <c r="A39" s="2" t="s">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C39" s="57" t="s">
-        <v>746</v>
+        <v>772</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>563</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="E39" s="57" t="s">
-        <v>749</v>
-      </c>
-      <c r="F39" s="57"/>
+        <v>57</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-    </row>
-    <row r="40" spans="1:11">
+      <c r="H39" s="3"/>
+      <c r="J39" s="2"/>
+    </row>
+    <row r="40" spans="1:11" ht="28.8">
       <c r="A40" s="2" t="s">
-        <v>782</v>
+        <v>426</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="C40" s="57" t="s">
-        <v>751</v>
+        <v>772</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>752</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
       <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:11" ht="28.8">
       <c r="A41" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C41" s="49" t="s">
-        <v>432</v>
+        <v>772</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>414</v>
+        <v>39</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
-    </row>
-    <row r="42" spans="1:11" ht="220.8">
+      <c r="H41" s="3"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="3"/>
+    </row>
+    <row r="42" spans="1:11" ht="28.8">
       <c r="A42" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>30</v>
+        <v>772</v>
+      </c>
+      <c r="C42" t="s">
+        <v>664</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>813</v>
-      </c>
+        <v>705</v>
+      </c>
+      <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
-    </row>
-    <row r="43" spans="1:11" ht="28.8">
-      <c r="A43" s="2" t="s">
+      <c r="H42" s="3"/>
+      <c r="K42" s="34"/>
+    </row>
+    <row r="43" spans="1:11" ht="179.4">
+      <c r="A43" s="40" t="s">
         <v>426</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>564</v>
+      <c r="B43" s="37" t="s">
+        <v>772</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>799</v>
+      </c>
+      <c r="D43" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="37" t="s">
+        <v>800</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
-      <c r="J43" s="2"/>
-    </row>
-    <row r="44" spans="1:11" ht="28.8">
+      <c r="K43" s="34"/>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
+        <v>776</v>
+      </c>
+      <c r="C44" s="49" t="s">
+        <v>431</v>
+      </c>
+      <c r="D44" s="48" t="s">
+        <v>545</v>
+      </c>
+      <c r="E44" s="17"/>
       <c r="H44" s="3"/>
     </row>
-    <row r="45" spans="1:11" ht="28.8">
+    <row r="45" spans="1:11">
       <c r="A45" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>783</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>38</v>
+        <v>776</v>
+      </c>
+      <c r="C45" s="49" t="s">
+        <v>550</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="J45" s="19"/>
-      <c r="K45" s="3"/>
-    </row>
-    <row r="46" spans="1:11" ht="28.8">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
       <c r="A46" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>783</v>
+        <v>776</v>
       </c>
       <c r="C46" t="s">
-        <v>664</v>
+        <v>557</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>705</v>
-      </c>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="K46" s="34"/>
-    </row>
-    <row r="47" spans="1:11" ht="179.4">
-      <c r="A47" s="40" t="s">
-        <v>426</v>
-      </c>
-      <c r="B47" s="37" t="s">
-        <v>783</v>
-      </c>
-      <c r="C47" s="38" t="s">
-        <v>810</v>
-      </c>
-      <c r="D47" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" s="37" t="s">
-        <v>811</v>
-      </c>
+        <v>384</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="A47" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="E47" s="3"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
-      <c r="K47" s="34"/>
-    </row>
-    <row r="48" spans="1:11">
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+    </row>
+    <row r="48" spans="1:11" ht="28.8">
       <c r="A48" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C48" s="49" t="s">
-        <v>431</v>
-      </c>
-      <c r="D48" s="48" t="s">
-        <v>545</v>
-      </c>
-      <c r="E48" s="17"/>
+        <v>776</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
       <c r="H48" s="3"/>
     </row>
-    <row r="49" spans="1:11">
+    <row r="49" spans="1:10">
       <c r="A49" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C49" s="49" t="s">
-        <v>550</v>
+        <v>42</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11">
+        <v>43</v>
+      </c>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="J49" s="2"/>
+    </row>
+    <row r="50" spans="1:10">
       <c r="A50" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C50" t="s">
-        <v>557</v>
+        <v>776</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11">
+        <v>32</v>
+      </c>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="J50" s="2"/>
+    </row>
+    <row r="51" spans="1:10">
       <c r="A51" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>44</v>
+        <v>777</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>350</v>
+        <v>567</v>
       </c>
       <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
+      <c r="F51" s="17"/>
       <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="3"/>
-    </row>
-    <row r="52" spans="1:11" ht="28.8">
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" spans="1:10">
       <c r="A52" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>559</v>
+        <v>778</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
-    </row>
-    <row r="53" spans="1:11">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
       <c r="A53" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C53" s="49" t="s">
-        <v>42</v>
+        <v>774</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-      <c r="J53" s="2"/>
-    </row>
-    <row r="54" spans="1:11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
       <c r="A54" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-      <c r="J54" s="2"/>
-    </row>
-    <row r="55" spans="1:11">
+        <v>16</v>
+      </c>
+      <c r="D54" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
       <c r="A55" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>787</v>
+        <v>776</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>788</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="E55" s="3"/>
-      <c r="F55" s="17"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="2"/>
-    </row>
-    <row r="56" spans="1:11">
+    </row>
+    <row r="56" spans="1:10">
       <c r="A56" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>789</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11">
+        <v>776</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="17" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="69">
       <c r="A57" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C57" s="49" t="s">
-        <v>785</v>
-      </c>
+        <v>776</v>
+      </c>
+      <c r="C57" s="38"/>
       <c r="D57" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11">
+        <v>383</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="69">
       <c r="A58" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D58" s="56" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11">
+        <v>776</v>
+      </c>
+      <c r="C58" s="38"/>
+      <c r="D58" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="27.6">
       <c r="A59" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>776</v>
+      </c>
+      <c r="C59" s="38"/>
       <c r="D59" s="3" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11">
+        <v>334</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="82.8">
       <c r="A60" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C60" s="2"/>
-      <c r="D60" s="17" t="s">
-        <v>814</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="69">
+        <v>776</v>
+      </c>
+      <c r="D60" s="33" t="s">
+        <v>387</v>
+      </c>
+      <c r="E60" s="33" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
       <c r="A61" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C61" s="38"/>
+        <v>789</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="D61" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="69">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
       <c r="A62" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C62" s="38"/>
-      <c r="D62" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="27.6">
+        <v>789</v>
+      </c>
+      <c r="C62" t="s">
+        <v>790</v>
+      </c>
+      <c r="D62" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="28.8">
       <c r="A63" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="C63" s="38"/>
+        <v>789</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>560</v>
+      </c>
       <c r="D63" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" ht="82.8">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="28.8">
       <c r="A64" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>787</v>
-      </c>
-      <c r="D64" s="33" t="s">
-        <v>387</v>
-      </c>
-      <c r="E64" s="33" t="s">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5">
+        <v>789</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="82.8">
       <c r="A65" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>800</v>
+        <v>789</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>46</v>
+        <v>791</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5">
+        <v>56</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="69">
       <c r="A66" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C66" t="s">
-        <v>801</v>
-      </c>
-      <c r="D66" s="56" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="28.8">
+        <v>789</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="55.2">
       <c r="A67" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>800</v>
+        <v>789</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>560</v>
+        <v>796</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="28.8">
+        <v>541</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="409.6">
       <c r="A68" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>800</v>
+        <v>789</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>48</v>
+        <v>797</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E68" s="5" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="82.8">
-      <c r="A69" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>802</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="69">
-      <c r="A70" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>803</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="55.2">
-      <c r="A71" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>807</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>806</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="409.6">
-      <c r="A72" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>800</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>808</v>
-      </c>
-      <c r="D72" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="E72" s="3" t="s">
+      <c r="E68" s="3" t="s">
         <v>700</v>
       </c>
     </row>
@@ -7378,7 +7265,7 @@
       <c r="K11" s="3"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="220.8">
+    <row r="12" spans="1:14" ht="207">
       <c r="A12" s="2" t="s">
         <v>425</v>
       </c>
@@ -7915,7 +7802,7 @@
         <v>429</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>785</v>
+        <v>774</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>35</v>
@@ -8217,7 +8104,7 @@
       </c>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="193.2">
+    <row r="40" spans="1:14" ht="179.4">
       <c r="A40" s="41" t="s">
         <v>425</v>
       </c>
@@ -8458,7 +8345,7 @@
       <c r="A55" s="2" t="s">
         <v>693</v>
       </c>
-      <c r="B55" s="56" t="s">
+      <c r="B55" t="s">
         <v>716</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -8576,13 +8463,13 @@
       <c r="A66" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B66" s="57" t="s">
+      <c r="B66" s="56" t="s">
         <v>723</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>724</v>
       </c>
-      <c r="D66" s="57" t="s">
+      <c r="D66" s="56" t="s">
         <v>731</v>
       </c>
     </row>
@@ -8590,13 +8477,13 @@
       <c r="A67" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B67" s="57" t="s">
+      <c r="B67" s="56" t="s">
         <v>725</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>726</v>
       </c>
-      <c r="D67" s="57" t="s">
+      <c r="D67" s="56" t="s">
         <v>730</v>
       </c>
     </row>
@@ -8604,13 +8491,13 @@
       <c r="A68" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B68" s="57" t="s">
+      <c r="B68" s="56" t="s">
         <v>727</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>728</v>
       </c>
-      <c r="D68" s="57" t="s">
+      <c r="D68" s="56" t="s">
         <v>729</v>
       </c>
     </row>
@@ -8618,13 +8505,13 @@
       <c r="A69" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B69" s="57" t="s">
+      <c r="B69" s="56" t="s">
         <v>732</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>734</v>
       </c>
-      <c r="D69" s="57" t="s">
+      <c r="D69" s="56" t="s">
         <v>737</v>
       </c>
     </row>
@@ -8632,13 +8519,13 @@
       <c r="A70" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B70" s="57" t="s">
+      <c r="B70" s="56" t="s">
         <v>733</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>735</v>
       </c>
-      <c r="D70" s="57" t="s">
+      <c r="D70" s="56" t="s">
         <v>736</v>
       </c>
     </row>
@@ -8646,13 +8533,13 @@
       <c r="A71" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B71" s="57" t="s">
+      <c r="B71" s="56" t="s">
         <v>738</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>750</v>
       </c>
-      <c r="D71" s="57" t="s">
+      <c r="D71" s="56" t="s">
         <v>739</v>
       </c>
     </row>
@@ -8660,13 +8547,13 @@
       <c r="A72" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B72" s="57" t="s">
+      <c r="B72" s="56" t="s">
         <v>544</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>543</v>
       </c>
-      <c r="D72" s="57" t="s">
+      <c r="D72" s="56" t="s">
         <v>740</v>
       </c>
     </row>
@@ -8674,13 +8561,13 @@
       <c r="A73" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B73" s="57" t="s">
+      <c r="B73" s="56" t="s">
         <v>743</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>742</v>
       </c>
-      <c r="D73" s="57" t="s">
+      <c r="D73" s="56" t="s">
         <v>741</v>
       </c>
     </row>
@@ -8688,13 +8575,13 @@
       <c r="A74" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B74" s="57" t="s">
+      <c r="B74" s="56" t="s">
         <v>744</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>745</v>
       </c>
-      <c r="D74" s="57" t="s">
+      <c r="D74" s="56" t="s">
         <v>748</v>
       </c>
     </row>
@@ -8702,13 +8589,13 @@
       <c r="A75" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B75" s="57" t="s">
+      <c r="B75" s="56" t="s">
         <v>746</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>747</v>
       </c>
-      <c r="D75" s="57" t="s">
+      <c r="D75" s="56" t="s">
         <v>749</v>
       </c>
     </row>
@@ -8716,7 +8603,7 @@
       <c r="A76" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="B76" s="57" t="s">
+      <c r="B76" s="56" t="s">
         <v>751</v>
       </c>
       <c r="C76" s="3" t="s">

</xml_diff>

<commit_message>
seperation of cognitive profile + cognitive test based on evidence, that is just temporary - not saved in DB
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,27 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EFD0DB-0246-4060-9A44-E66728482D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C895B6B7-EFFD-4E38-BFF2-5B60DFD35206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
     <sheet name="Current Tasks" sheetId="16" r:id="rId2"/>
-    <sheet name="פרטי משתמש" sheetId="3" r:id="rId3"/>
-    <sheet name="Internal Traits" sheetId="1" r:id="rId4"/>
-    <sheet name="internal traits - Old" sheetId="14" r:id="rId5"/>
-    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId6"/>
-    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId7"/>
-    <sheet name="בניית ציונים" sheetId="9" r:id="rId8"/>
-    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId9"/>
-    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId10"/>
-    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId11"/>
-    <sheet name="טופס הזנה" sheetId="8" r:id="rId12"/>
-    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId13"/>
-    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId14"/>
-    <sheet name="בדיקות" sheetId="13" r:id="rId15"/>
-    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId16"/>
+    <sheet name="Analyzer Tasks" sheetId="17" r:id="rId3"/>
+    <sheet name="פרטי משתמש" sheetId="3" r:id="rId4"/>
+    <sheet name="Internal Traits" sheetId="1" r:id="rId5"/>
+    <sheet name="internal traits - Old" sheetId="14" r:id="rId6"/>
+    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId7"/>
+    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId8"/>
+    <sheet name="בניית ציונים" sheetId="9" r:id="rId9"/>
+    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId10"/>
+    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId11"/>
+    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId12"/>
+    <sheet name="טופס הזנה" sheetId="8" r:id="rId13"/>
+    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId14"/>
+    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId15"/>
+    <sheet name="בדיקות" sheetId="13" r:id="rId16"/>
+    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="840">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -2822,6 +2823,15 @@
     <t>בהירות מושגית</t>
   </si>
   <si>
+    <t>פתיחות אינטלקטואלית</t>
+  </si>
+  <si>
+    <t>עומק מחשבתי</t>
+  </si>
+  <si>
+    <t>הסקה מילולית</t>
+  </si>
+  <si>
     <t>גמישות מחשבתית</t>
   </si>
   <si>
@@ -3006,6 +3016,93 @@
   </si>
   <si>
     <t>פרופיל אנליטי</t>
+  </si>
+  <si>
+    <t>social_intuitive_ intelligence</t>
+  </si>
+  <si>
+    <t>התכונות לא תואמות את האקסל (למשל חסר סגנון סובייטי, היפיות וכו')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לשקול לעבור לפחות כרגע - למודל ידני שבו אני כל פעם אג'נרט פרופמטים קבועים ואכניס לקלוד את כל התוצאות שיזין במערכת. זה לא אידיאלי אבל זו עבודה של 5 דקות ליוזר נגיד ותוציא לי תוצאות טובות. </t>
+  </si>
+  <si>
+    <t>לבדוק על הקטע של הקש אינפוט</t>
+  </si>
+  <si>
+    <t>5-6 פרומפטים  - כל אחד מהם - יג'ונרט לי אוטומטית על ידי המערכת כולל תמליל השיחה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מכניסה לצ'אטי כל פעם פרומפט אחר  והוא מוציא לי JSON כמו עכשיו. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">לוקחת את הjson ומכניסה למערכת - והציונים מתעדכנים. </t>
+  </si>
+  <si>
+    <t>תצוגה נפרדת לעלות השיחה ולעלות הניתוח</t>
+  </si>
+  <si>
+    <t>לעשות פונקציה שמחשבת את הציונים לפי הראיות</t>
+  </si>
+  <si>
+    <t>לעשות באופן זמני שהציון של הקוגנטיבי ילקח מהציון שחישבנו במקום הציונים של הניתוח (+יוקרה)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אם עובד טוב - להחליף את הציונים הפרומפט לפרומפט הזה ולעדכן את הציונים במערכת בהתאם. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">לשמור גם כמות ראיות בחלוקה לכמות ראיות חזקות וחלשות. </t>
+  </si>
+  <si>
+    <t>ואז בהמשך שיחה - תשלח לניתוח רק המשך השיחה והראיות יחושבו בהתאם</t>
+  </si>
+  <si>
+    <t>אחרי זה לעשות את נרמול התוצאות והודאות יותר חכם, לא רק לפי מספר משפטים/מילים, אפשר גם נגיד לפי איזה שאלות ענה ואיזה נושאים דוברו בשיחה וכו'</t>
+  </si>
+  <si>
+    <t>יכול להיות שכרגע הנרמול לא יהיה טוב כי הוא ינרמל למרות שהמודל מוציא ראיות בכוח פחות או יותר באותה כמות לכל משתמש.</t>
+  </si>
+  <si>
+    <t>אולי בכל אחד מהפרומפטים האחרים - נעריך גם אינטליגנציה באופן כללי ונוסיף את זה לחישוב.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נוי </t>
+  </si>
+  <si>
+    <t>נטי</t>
+  </si>
+  <si>
+    <t>רון</t>
+  </si>
+  <si>
+    <t>חן</t>
+  </si>
+  <si>
+    <t>אנה</t>
+  </si>
+  <si>
+    <t>הגר</t>
+  </si>
+  <si>
+    <t>ערסית</t>
+  </si>
+  <si>
+    <t>נדב</t>
+  </si>
+  <si>
+    <t>לנסות את הראיות בשיטה של חובת 3 ראיות</t>
+  </si>
+  <si>
+    <t>בלי חוק ה3</t>
+  </si>
+  <si>
+    <t>חוק ה3</t>
+  </si>
+  <si>
+    <t>חוק ה3 בלי להכפיל משקל לראיה שלילית סבירה וכן הכפלת משקלים קיצונית לשליליים עם ראיה חזקה + הכפלה יותר קיצונית לחיובים חזקים (מעל 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אם אני עובדת בשיטה הזאת (כרגע על 6) - אני צריכה להתחשב בגודל הדלתאות </t>
   </si>
 </sst>
 </file>
@@ -3212,7 +3309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3360,6 +3457,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" readingOrder="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3930,6 +4030,621 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
+  <dimension ref="B1:M20"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13">
+      <c r="B1" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="2:13" ht="28.8">
+      <c r="B4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13">
+      <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5">
+        <v>85</v>
+      </c>
+      <c r="D5" s="5">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="F5" s="5">
+        <v>85</v>
+      </c>
+      <c r="G5" s="5">
+        <v>20</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="I5" s="15">
+        <f>SQRT(H5*E5)</f>
+        <v>0.69282032302755092</v>
+      </c>
+      <c r="J5" s="15">
+        <f>(C5+F5)/2</f>
+        <v>85</v>
+      </c>
+      <c r="K5" s="15">
+        <f>I5*J5</f>
+        <v>58.889727457341827</v>
+      </c>
+      <c r="L5" s="5">
+        <f>100-ABS(G5-D5)</f>
+        <v>100</v>
+      </c>
+      <c r="M5">
+        <f>L5*K5</f>
+        <v>5888.9727457341824</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13">
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5">
+        <v>60</v>
+      </c>
+      <c r="D6" s="5">
+        <v>50</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="5">
+        <v>80</v>
+      </c>
+      <c r="G6" s="5">
+        <v>60</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="I6" s="15">
+        <f>SQRT(H6*E6)</f>
+        <v>0.54772255750516607</v>
+      </c>
+      <c r="J6" s="15">
+        <f>(C6+F6)/2</f>
+        <v>70</v>
+      </c>
+      <c r="K6" s="15">
+        <f>I6*J6</f>
+        <v>38.340579025361627</v>
+      </c>
+      <c r="L6" s="5">
+        <f>100-ABS(G6-D6)</f>
+        <v>90</v>
+      </c>
+      <c r="M6">
+        <f>L6*K6</f>
+        <v>3450.6521122825466</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13">
+      <c r="B7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="5">
+        <v>30</v>
+      </c>
+      <c r="D7" s="5">
+        <v>90</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="F7" s="5">
+        <v>20</v>
+      </c>
+      <c r="G7" s="5">
+        <v>24</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="15">
+        <f>SQRT(H7*E7)</f>
+        <v>0.3872983346207417</v>
+      </c>
+      <c r="J7" s="15">
+        <f>(C7+F7)/2</f>
+        <v>25</v>
+      </c>
+      <c r="K7" s="15">
+        <f>I7*J7</f>
+        <v>9.6824583655185421</v>
+      </c>
+      <c r="L7" s="5">
+        <f>100-ABS(G7-D7)</f>
+        <v>34</v>
+      </c>
+      <c r="M7">
+        <f>L7*K7</f>
+        <v>329.2035844276304</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="15">
+        <f>SUM(I5:I7)</f>
+        <v>1.6278412151534587</v>
+      </c>
+      <c r="J8" s="15"/>
+      <c r="K8" s="13">
+        <f>SUM(K5:K7)/5</f>
+        <v>21.382552969644401</v>
+      </c>
+      <c r="L8" s="13">
+        <f>SUM(L5:L7)/5</f>
+        <v>44.8</v>
+      </c>
+      <c r="M8" s="14">
+        <f>SUM(M5:M7)/SUM(K5:K7)</f>
+        <v>90.436613964390943</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5">
+        <f>I8/5</f>
+        <v>0.32556824303069176</v>
+      </c>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="2:13">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+    </row>
+    <row r="11" spans="2:13">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+    </row>
+    <row r="12" spans="2:13" ht="28.8">
+      <c r="B12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="M12" s="13" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13">
+      <c r="B13" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="5">
+        <v>70</v>
+      </c>
+      <c r="D13" s="5">
+        <v>80</v>
+      </c>
+      <c r="E13" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="F13" s="5">
+        <v>80</v>
+      </c>
+      <c r="G13" s="5">
+        <v>72</v>
+      </c>
+      <c r="H13" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="I13" s="15">
+        <f t="shared" ref="I13:I18" si="0">SQRT(H13*E13)</f>
+        <v>0.9</v>
+      </c>
+      <c r="J13" s="15">
+        <f t="shared" ref="J13:J18" si="1">(C13+F13)/2</f>
+        <v>75</v>
+      </c>
+      <c r="K13" s="15">
+        <f t="shared" ref="K13:K18" si="2">I13*J13</f>
+        <v>67.5</v>
+      </c>
+      <c r="L13" s="5">
+        <f t="shared" ref="L13:L18" si="3">100-ABS(G13-D13)</f>
+        <v>92</v>
+      </c>
+      <c r="M13">
+        <f t="shared" ref="M13:M18" si="4">L13*K13</f>
+        <v>6210</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13">
+      <c r="B14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="5">
+        <v>80</v>
+      </c>
+      <c r="D14" s="5">
+        <v>20</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="F14" s="5">
+        <v>80</v>
+      </c>
+      <c r="G14" s="5">
+        <v>90</v>
+      </c>
+      <c r="H14" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="I14" s="15">
+        <f t="shared" si="0"/>
+        <v>0.2449489742783178</v>
+      </c>
+      <c r="J14" s="15">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+      <c r="K14" s="15">
+        <f t="shared" si="2"/>
+        <v>19.595917942265423</v>
+      </c>
+      <c r="L14" s="5">
+        <f t="shared" si="3"/>
+        <v>30</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="4"/>
+        <v>587.87753826796268</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13">
+      <c r="B15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="5">
+        <v>50</v>
+      </c>
+      <c r="D15" s="5">
+        <v>50</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F15" s="5">
+        <v>50</v>
+      </c>
+      <c r="G15" s="5">
+        <v>60</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="I15" s="15">
+        <f t="shared" si="0"/>
+        <v>0.54772255750516607</v>
+      </c>
+      <c r="J15" s="15">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="K15" s="15">
+        <f t="shared" si="2"/>
+        <v>27.386127875258303</v>
+      </c>
+      <c r="L15" s="5">
+        <f t="shared" si="3"/>
+        <v>90</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="4"/>
+        <v>2464.7515087732472</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13">
+      <c r="B16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="5">
+        <v>100</v>
+      </c>
+      <c r="D16" s="5">
+        <v>100</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5">
+        <v>100</v>
+      </c>
+      <c r="G16" s="5">
+        <v>20</v>
+      </c>
+      <c r="H16" s="5">
+        <v>1</v>
+      </c>
+      <c r="I16" s="15">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J16" s="15">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="K16" s="15">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="L16" s="5">
+        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="4"/>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13">
+      <c r="B17" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="5">
+        <v>100</v>
+      </c>
+      <c r="D17" s="5">
+        <v>66</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="F17" s="5">
+        <v>100</v>
+      </c>
+      <c r="G17" s="5">
+        <v>24</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="15">
+        <f t="shared" si="0"/>
+        <v>0.3872983346207417</v>
+      </c>
+      <c r="J17" s="15">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="K17" s="15">
+        <f t="shared" si="2"/>
+        <v>38.729833462074168</v>
+      </c>
+      <c r="L17" s="5">
+        <f t="shared" si="3"/>
+        <v>58</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="4"/>
+        <v>2246.3303408003017</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13">
+      <c r="B18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="5">
+        <v>20</v>
+      </c>
+      <c r="D18" s="5">
+        <v>40</v>
+      </c>
+      <c r="E18" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="F18" s="5">
+        <v>100</v>
+      </c>
+      <c r="G18" s="5">
+        <v>60</v>
+      </c>
+      <c r="H18" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="I18" s="15">
+        <f t="shared" si="0"/>
+        <v>0.56568542494923812</v>
+      </c>
+      <c r="J18" s="15">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="K18" s="15">
+        <f t="shared" si="2"/>
+        <v>33.941125496954285</v>
+      </c>
+      <c r="L18" s="5">
+        <f t="shared" si="3"/>
+        <v>80</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="4"/>
+        <v>2715.2900397563426</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13">
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5">
+        <f>SUM(H13:H18)/5</f>
+        <v>0.78</v>
+      </c>
+      <c r="I19" s="15">
+        <f>SUM(I13:I18)</f>
+        <v>3.6456552913534637</v>
+      </c>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="13">
+        <f>SUM(L13:L18)/5</f>
+        <v>74</v>
+      </c>
+      <c r="M19" s="14">
+        <f>SUM(M13:M18)/SUM(K13:K18)</f>
+        <v>56.500364466750881</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13">
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5">
+        <f>I19/5</f>
+        <v>0.72913105827069269</v>
+      </c>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487A18-0B10-40C8-BA24-F0DC1678FA48}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4214,7 +4929,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
   <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4436,7 +5151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233E8F68-8BA3-48DC-98C9-B07384CDF822}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4598,7 +5313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E73849-9796-44C6-80F8-1CA54A2F64E9}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4748,7 +5463,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D465AB7-D7AD-4770-A1DB-A227111CD595}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4793,7 +5508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC47FA1-3DB6-4F73-94E7-2B8A7BD334E9}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4872,7 +5587,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC7838B-7DDE-48A8-A573-BCAB05D487CE}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5209,6 +5924,198 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50151C83-D621-46FF-871C-82BDAD5480FD}">
+  <dimension ref="B2:P22"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:16">
+      <c r="P2" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="3" spans="2:16">
+      <c r="P3" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16">
+      <c r="B4" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16">
+      <c r="B7" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16">
+      <c r="K9" t="s">
+        <v>837</v>
+      </c>
+      <c r="L9" t="s">
+        <v>836</v>
+      </c>
+      <c r="M9" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16">
+      <c r="B10" t="s">
+        <v>814</v>
+      </c>
+      <c r="J10" t="s">
+        <v>827</v>
+      </c>
+      <c r="K10">
+        <v>90</v>
+      </c>
+      <c r="L10">
+        <v>68</v>
+      </c>
+      <c r="M10">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16">
+      <c r="J11" t="s">
+        <v>828</v>
+      </c>
+      <c r="K11">
+        <v>58</v>
+      </c>
+      <c r="L11">
+        <v>51</v>
+      </c>
+      <c r="M11">
+        <v>80</v>
+      </c>
+      <c r="N11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16">
+      <c r="J12" t="s">
+        <v>829</v>
+      </c>
+      <c r="K12">
+        <v>81</v>
+      </c>
+      <c r="L12">
+        <v>61</v>
+      </c>
+      <c r="M12">
+        <v>65</v>
+      </c>
+      <c r="N12">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16">
+      <c r="J13" t="s">
+        <v>830</v>
+      </c>
+      <c r="K13">
+        <v>93</v>
+      </c>
+      <c r="L13">
+        <v>71</v>
+      </c>
+      <c r="M13">
+        <v>87</v>
+      </c>
+      <c r="O13" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16">
+      <c r="B14" s="57" t="s">
+        <v>815</v>
+      </c>
+      <c r="J14" t="s">
+        <v>831</v>
+      </c>
+      <c r="K14">
+        <v>63</v>
+      </c>
+      <c r="L14">
+        <v>63</v>
+      </c>
+      <c r="M14">
+        <v>81</v>
+      </c>
+      <c r="O14" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16">
+      <c r="B15" t="s">
+        <v>816</v>
+      </c>
+      <c r="J15" t="s">
+        <v>832</v>
+      </c>
+      <c r="K15">
+        <v>54</v>
+      </c>
+      <c r="L15">
+        <v>38</v>
+      </c>
+      <c r="M15">
+        <v>51</v>
+      </c>
+      <c r="O15" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16">
+      <c r="B16" t="s">
+        <v>817</v>
+      </c>
+      <c r="J16" t="s">
+        <v>833</v>
+      </c>
+      <c r="L16">
+        <v>17</v>
+      </c>
+      <c r="O16" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15">
+      <c r="J17" t="s">
+        <v>834</v>
+      </c>
+      <c r="L17">
+        <v>65</v>
+      </c>
+      <c r="O17" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15">
+      <c r="O18" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15">
+      <c r="B20" t="s">
+        <v>818</v>
+      </c>
+      <c r="O20" s="14" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15">
+      <c r="O22" t="s">
+        <v>826</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1C79E50-A761-4208-AC1F-7EE61CFDD025}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5729,9 +6636,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
@@ -5767,7 +6674,7 @@
         <v>413</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>6</v>
@@ -5779,7 +6686,7 @@
         <v>59</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>3</v>
@@ -5808,16 +6715,16 @@
     </row>
     <row r="5" spans="1:14" ht="28.8">
       <c r="A5" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="C5" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -5829,16 +6736,16 @@
     </row>
     <row r="6" spans="1:14" ht="28.8">
       <c r="A6" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="C6" t="s">
         <v>753</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -5850,16 +6757,16 @@
     </row>
     <row r="7" spans="1:14" ht="28.8">
       <c r="A7" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="C7" t="s">
         <v>754</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -5871,13 +6778,13 @@
     </row>
     <row r="8" spans="1:14" ht="28.8">
       <c r="A8" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="C8" t="s">
         <v>807</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>767</v>
-      </c>
-      <c r="C8" t="s">
-        <v>804</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>755</v>
@@ -5890,13 +6797,13 @@
     </row>
     <row r="9" spans="1:14" ht="28.8">
       <c r="A9" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>639</v>
@@ -5907,14 +6814,12 @@
       <c r="H9" s="3"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:14" ht="28.8">
-      <c r="A10" s="2" t="s">
-        <v>715</v>
-      </c>
+    <row r="10" spans="1:14">
+      <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="3" t="s">
-        <v>806</v>
+        <v>758</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -5922,18 +6827,12 @@
       <c r="H10" s="3"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:14" ht="28.8">
-      <c r="A11" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>767</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>760</v>
-      </c>
+    <row r="11" spans="1:14">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
       <c r="D11" s="3" t="s">
-        <v>435</v>
+        <v>757</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -5941,40 +6840,37 @@
       <c r="H11" s="3"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:14" ht="331.2">
+    <row r="12" spans="1:14" ht="28.8">
       <c r="A12" s="2" t="s">
         <v>715</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>759</v>
+        <v>811</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>798</v>
-      </c>
+        <v>809</v>
+      </c>
+      <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:14" ht="28.8">
       <c r="A13" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>763</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>764</v>
+      <c r="D13" s="3" t="s">
+        <v>756</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -5982,75 +6878,78 @@
       <c r="H13" s="3"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:14" ht="27.6">
+    <row r="14" spans="1:14" ht="331.2">
       <c r="A14" s="2" t="s">
-        <v>763</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>765</v>
+        <v>715</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>770</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>768</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>704</v>
-      </c>
-      <c r="E14" s="3"/>
+        <v>762</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>801</v>
+      </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:14" ht="27.6">
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:14" ht="28.8">
       <c r="A15" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="C15" t="s">
-        <v>761</v>
+        <v>768</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>665</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="2"/>
+      <c r="H15" s="3"/>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:14" ht="27.6">
       <c r="A16" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>765</v>
-      </c>
-      <c r="C16" t="s">
-        <v>666</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>707</v>
+        <v>768</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>704</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="3"/>
       <c r="J16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="27.6">
       <c r="A17" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="C17" t="s">
+        <v>764</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>765</v>
-      </c>
-      <c r="C17" t="s">
-        <v>671</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>775</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -6060,54 +6959,54 @@
     </row>
     <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C18" t="s">
-        <v>785</v>
+        <v>666</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="K18" s="34"/>
+      <c r="H18" s="2"/>
+      <c r="J18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="27.6">
       <c r="A19" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C19" t="s">
-        <v>786</v>
+        <v>671</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>702</v>
+        <v>778</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="K19" s="34"/>
+      <c r="H19" s="2"/>
+      <c r="J19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="27.6">
       <c r="A20" s="2" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C20" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>22</v>
+        <v>701</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -6115,82 +7014,78 @@
       <c r="H20" s="3"/>
       <c r="K20" s="34"/>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" ht="27.6">
       <c r="A21" s="2" t="s">
-        <v>693</v>
+        <v>766</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>696</v>
+        <v>768</v>
+      </c>
+      <c r="C21" t="s">
+        <v>789</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="2"/>
-      <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:11" ht="28.8">
+      <c r="H21" s="3"/>
+      <c r="K21" s="34"/>
+    </row>
+    <row r="22" spans="1:11" ht="27.6">
       <c r="A22" s="2" t="s">
-        <v>693</v>
+        <v>766</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>717</v>
+        <v>768</v>
+      </c>
+      <c r="C22" t="s">
+        <v>790</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>643</v>
+        <v>22</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="2"/>
-      <c r="J22" s="2"/>
+      <c r="H22" s="3"/>
+      <c r="K22" s="34"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="2" t="s">
         <v>693</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="C23" t="s">
-        <v>716</v>
+        <v>772</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>696</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>644</v>
+        <v>697</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3" t="s">
-        <v>426</v>
-      </c>
+      <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" ht="28.8">
       <c r="A24" s="2" t="s">
         <v>693</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="C24" t="s">
-        <v>718</v>
+        <v>772</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>717</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>719</v>
+        <v>643</v>
       </c>
       <c r="E24" s="3"/>
-      <c r="F24" s="3" t="s">
-        <v>426</v>
-      </c>
+      <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="2"/>
       <c r="J24" s="2"/>
@@ -6200,38 +7095,38 @@
         <v>693</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="C25" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>721</v>
+        <v>644</v>
       </c>
       <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
+      <c r="F25" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G25" s="3"/>
       <c r="H25" s="2"/>
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2" t="s">
-        <v>771</v>
+        <v>693</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>770</v>
-      </c>
-      <c r="C26" s="56" t="s">
-        <v>723</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>724</v>
-      </c>
-      <c r="E26" s="56" t="s">
-        <v>731</v>
-      </c>
-      <c r="F26" s="56" t="s">
-        <v>425</v>
+        <v>772</v>
+      </c>
+      <c r="C26" t="s">
+        <v>718</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3" t="s">
+        <v>426</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="2"/>
@@ -6239,227 +7134,233 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="2" t="s">
-        <v>771</v>
+        <v>693</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>770</v>
-      </c>
-      <c r="C27" s="56" t="s">
-        <v>725</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="E27" s="56" t="s">
-        <v>730</v>
-      </c>
-      <c r="F27" s="56"/>
+        <v>772</v>
+      </c>
+      <c r="C27" t="s">
+        <v>720</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>721</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
+      <c r="H27" s="2"/>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>727</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>728</v>
+        <v>723</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>724</v>
       </c>
       <c r="E28" s="56" t="s">
-        <v>729</v>
-      </c>
-      <c r="F28" s="56"/>
+        <v>731</v>
+      </c>
+      <c r="F28" s="56" t="s">
+        <v>425</v>
+      </c>
       <c r="G28" s="3"/>
+      <c r="H28" s="2"/>
+      <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>732</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>734</v>
+        <v>725</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>726</v>
       </c>
       <c r="E29" s="56" t="s">
-        <v>737</v>
+        <v>730</v>
       </c>
       <c r="F29" s="56"/>
       <c r="G29" s="3"/>
+      <c r="J29" s="2"/>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>733</v>
+        <v>727</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="E30" s="56" t="s">
-        <v>736</v>
+        <v>729</v>
       </c>
       <c r="F30" s="56"/>
       <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C31" s="56" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>750</v>
+        <v>734</v>
       </c>
       <c r="E31" s="56" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="F31" s="56"/>
       <c r="G31" s="3"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>544</v>
+        <v>733</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>543</v>
+        <v>735</v>
       </c>
       <c r="E32" s="56" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="F32" s="56"/>
       <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="J32" s="2"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C33" s="56" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="E33" s="56" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="F33" s="56"/>
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>744</v>
+        <v>544</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>745</v>
+        <v>543</v>
       </c>
       <c r="E34" s="56" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="F34" s="56"/>
       <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="J34" s="2"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="E35" s="56" t="s">
-        <v>749</v>
+        <v>741</v>
       </c>
       <c r="F35" s="56"/>
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="2" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C36" s="56" t="s">
+        <v>744</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>745</v>
+      </c>
+      <c r="E36" s="56" t="s">
+        <v>748</v>
+      </c>
+      <c r="F36" s="56"/>
+      <c r="G36" s="3"/>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C37" s="56" t="s">
+        <v>746</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>747</v>
+      </c>
+      <c r="E37" s="56" t="s">
+        <v>749</v>
+      </c>
+      <c r="F37" s="56"/>
+      <c r="G37" s="3"/>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C38" s="56" t="s">
         <v>751</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D38" s="3" t="s">
         <v>752</v>
       </c>
-      <c r="G36" s="3"/>
-    </row>
-    <row r="37" spans="1:11" ht="28.8">
-      <c r="A37" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C37" s="49" t="s">
-        <v>432</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-    </row>
-    <row r="38" spans="1:11" ht="220.8">
-      <c r="A38" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>801</v>
-      </c>
-      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:11" ht="28.8">
@@ -6467,490 +7368,526 @@
         <v>426</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>563</v>
+        <v>775</v>
+      </c>
+      <c r="C39" s="49" t="s">
+        <v>432</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>564</v>
-      </c>
+        <v>414</v>
+      </c>
+      <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="J39" s="2"/>
-    </row>
-    <row r="40" spans="1:11" ht="28.8">
+    </row>
+    <row r="40" spans="1:11" ht="220.8">
       <c r="A40" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E40" s="3"/>
+        <v>29</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>804</v>
+      </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:11" ht="28.8">
       <c r="A41" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>38</v>
+        <v>563</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E41" s="3"/>
+        <v>57</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>564</v>
+      </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
-      <c r="J41" s="19"/>
-      <c r="K41" s="3"/>
+      <c r="J41" s="2"/>
     </row>
     <row r="42" spans="1:11" ht="28.8">
       <c r="A42" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C42" t="s">
-        <v>664</v>
+        <v>775</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>705</v>
+        <v>37</v>
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
-      <c r="K42" s="34"/>
-    </row>
-    <row r="43" spans="1:11" ht="179.4">
-      <c r="A43" s="40" t="s">
+    </row>
+    <row r="43" spans="1:11" ht="28.8">
+      <c r="A43" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="B43" s="37" t="s">
-        <v>772</v>
-      </c>
-      <c r="C43" s="38" t="s">
-        <v>799</v>
-      </c>
-      <c r="D43" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" s="37" t="s">
-        <v>800</v>
-      </c>
+      <c r="B43" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
-      <c r="K43" s="34"/>
-    </row>
-    <row r="44" spans="1:11">
+      <c r="J43" s="19"/>
+      <c r="K43" s="3"/>
+    </row>
+    <row r="44" spans="1:11" ht="28.8">
       <c r="A44" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C44" s="49" t="s">
-        <v>431</v>
-      </c>
-      <c r="D44" s="48" t="s">
-        <v>545</v>
-      </c>
-      <c r="E44" s="17"/>
+        <v>775</v>
+      </c>
+      <c r="C44" t="s">
+        <v>664</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
       <c r="H44" s="3"/>
-    </row>
-    <row r="45" spans="1:11">
-      <c r="A45" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C45" s="49" t="s">
-        <v>550</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>551</v>
-      </c>
+      <c r="K44" s="34"/>
+    </row>
+    <row r="45" spans="1:11" ht="179.4">
+      <c r="A45" s="40" t="s">
+        <v>426</v>
+      </c>
+      <c r="B45" s="37" t="s">
+        <v>775</v>
+      </c>
+      <c r="C45" s="38" t="s">
+        <v>802</v>
+      </c>
+      <c r="D45" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" s="37" t="s">
+        <v>803</v>
+      </c>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="K45" s="34"/>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C46" t="s">
-        <v>557</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>384</v>
-      </c>
+        <v>779</v>
+      </c>
+      <c r="C46" s="49" t="s">
+        <v>431</v>
+      </c>
+      <c r="D46" s="48" t="s">
+        <v>545</v>
+      </c>
+      <c r="E46" s="17"/>
+      <c r="H46" s="3"/>
     </row>
     <row r="47" spans="1:11">
       <c r="A47" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>44</v>
+        <v>779</v>
+      </c>
+      <c r="C47" s="49" t="s">
+        <v>550</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="3"/>
-    </row>
-    <row r="48" spans="1:11" ht="28.8">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
       <c r="A48" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>559</v>
+        <v>779</v>
+      </c>
+      <c r="C48" t="s">
+        <v>557</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>558</v>
-      </c>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
-    </row>
-    <row r="49" spans="1:10">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11">
       <c r="A49" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C49" s="49" t="s">
-        <v>42</v>
+        <v>779</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>43</v>
+        <v>350</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
-      <c r="J49" s="2"/>
-    </row>
-    <row r="50" spans="1:10">
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+    </row>
+    <row r="50" spans="1:11" ht="28.8">
       <c r="A50" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>31</v>
+        <v>559</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>32</v>
+        <v>558</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
-      <c r="J50" s="2"/>
-    </row>
-    <row r="51" spans="1:10">
+    </row>
+    <row r="51" spans="1:11">
       <c r="A51" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>777</v>
+        <v>779</v>
+      </c>
+      <c r="C51" s="49" t="s">
+        <v>42</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>567</v>
+        <v>43</v>
       </c>
       <c r="E51" s="3"/>
-      <c r="F51" s="17"/>
+      <c r="F51" s="3"/>
       <c r="G51" s="3"/>
-      <c r="H51" s="2"/>
-    </row>
-    <row r="52" spans="1:10">
+      <c r="H51" s="3"/>
+      <c r="J51" s="2"/>
+    </row>
+    <row r="52" spans="1:11">
       <c r="A52" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>778</v>
+        <v>31</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10">
+        <v>32</v>
+      </c>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="J52" s="2"/>
+    </row>
+    <row r="53" spans="1:11">
       <c r="A53" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C53" s="49" t="s">
-        <v>774</v>
+        <v>779</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>780</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10">
+        <v>567</v>
+      </c>
+      <c r="E53" s="3"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="2"/>
+    </row>
+    <row r="54" spans="1:11">
       <c r="A54" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D54" t="s">
-        <v>779</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10">
+        <v>781</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11">
       <c r="A55" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>27</v>
+        <v>779</v>
+      </c>
+      <c r="C55" s="49" t="s">
+        <v>777</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11">
       <c r="A56" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="17" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="69">
+        <v>779</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D56" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11">
       <c r="A57" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C57" s="38"/>
+        <v>779</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D57" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="69">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11">
       <c r="A58" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="C58" s="38"/>
-      <c r="D58" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>782</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="27.6">
+        <v>779</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" s="17" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="69">
       <c r="A59" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C59" s="38"/>
       <c r="D59" s="3" t="s">
-        <v>334</v>
+        <v>383</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="82.8">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="69">
       <c r="A60" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="D60" s="33" t="s">
+        <v>779</v>
+      </c>
+      <c r="C60" s="38"/>
+      <c r="D60" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="27.6">
+      <c r="A61" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="C61" s="38"/>
+      <c r="D61" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="82.8">
+      <c r="A62" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="D62" s="33" t="s">
         <v>387</v>
       </c>
-      <c r="E60" s="33" t="s">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10">
-      <c r="A61" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>789</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10">
-      <c r="A62" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>789</v>
-      </c>
-      <c r="C62" t="s">
-        <v>790</v>
-      </c>
-      <c r="D62" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="28.8">
+      <c r="E62" s="33" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11">
       <c r="A63" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>560</v>
+        <v>46</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="28.8">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11">
       <c r="A64" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>789</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E64" s="5" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="82.8">
+        <v>792</v>
+      </c>
+      <c r="C64" t="s">
+        <v>793</v>
+      </c>
+      <c r="D64" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="28.8">
       <c r="A65" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>791</v>
+        <v>560</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>793</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="69">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="28.8">
       <c r="A66" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>792</v>
+        <v>48</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="55.2">
+        <v>49</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="82.8">
       <c r="A67" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E67" s="3" t="s">
         <v>796</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="409.6">
+    </row>
+    <row r="68" spans="1:5" ht="69">
       <c r="A68" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E68" s="3" t="s">
         <v>797</v>
       </c>
-      <c r="D68" s="3" t="s">
+    </row>
+    <row r="69" spans="1:5" ht="55.2">
+      <c r="A69" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="409.6">
+      <c r="A70" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="D70" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="E70" s="3" t="s">
         <v>700</v>
       </c>
     </row>
@@ -6959,7 +7896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
   <dimension ref="A1:N136"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7802,7 +8739,7 @@
         <v>429</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>35</v>
@@ -9053,7 +9990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9333,7 +10270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
   <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9630,7 +10567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9978,619 +10915,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
-  <dimension ref="B1:M20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="2" max="2" width="15.44140625" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" customWidth="1"/>
-    <col min="9" max="9" width="14.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:13">
-      <c r="B1" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="G1" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="J1" s="19" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="2:13">
-      <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-    </row>
-    <row r="4" spans="2:13" ht="28.8">
-      <c r="B4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13">
-      <c r="B5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="5">
-        <v>85</v>
-      </c>
-      <c r="D5" s="5">
-        <v>20</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0.6</v>
-      </c>
-      <c r="F5" s="5">
-        <v>85</v>
-      </c>
-      <c r="G5" s="5">
-        <v>20</v>
-      </c>
-      <c r="H5" s="5">
-        <v>0.8</v>
-      </c>
-      <c r="I5" s="15">
-        <f>SQRT(H5*E5)</f>
-        <v>0.69282032302755092</v>
-      </c>
-      <c r="J5" s="15">
-        <f>(C5+F5)/2</f>
-        <v>85</v>
-      </c>
-      <c r="K5" s="15">
-        <f>I5*J5</f>
-        <v>58.889727457341827</v>
-      </c>
-      <c r="L5" s="5">
-        <f>100-ABS(G5-D5)</f>
-        <v>100</v>
-      </c>
-      <c r="M5">
-        <f>L5*K5</f>
-        <v>5888.9727457341824</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13">
-      <c r="B6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="5">
-        <v>60</v>
-      </c>
-      <c r="D6" s="5">
-        <v>50</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="F6" s="5">
-        <v>80</v>
-      </c>
-      <c r="G6" s="5">
-        <v>60</v>
-      </c>
-      <c r="H6" s="5">
-        <v>0.6</v>
-      </c>
-      <c r="I6" s="15">
-        <f>SQRT(H6*E6)</f>
-        <v>0.54772255750516607</v>
-      </c>
-      <c r="J6" s="15">
-        <f>(C6+F6)/2</f>
-        <v>70</v>
-      </c>
-      <c r="K6" s="15">
-        <f>I6*J6</f>
-        <v>38.340579025361627</v>
-      </c>
-      <c r="L6" s="5">
-        <f>100-ABS(G6-D6)</f>
-        <v>90</v>
-      </c>
-      <c r="M6">
-        <f>L6*K6</f>
-        <v>3450.6521122825466</v>
-      </c>
-    </row>
-    <row r="7" spans="2:13">
-      <c r="B7" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="5">
-        <v>30</v>
-      </c>
-      <c r="D7" s="5">
-        <v>90</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="F7" s="5">
-        <v>20</v>
-      </c>
-      <c r="G7" s="5">
-        <v>24</v>
-      </c>
-      <c r="H7" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="I7" s="15">
-        <f>SQRT(H7*E7)</f>
-        <v>0.3872983346207417</v>
-      </c>
-      <c r="J7" s="15">
-        <f>(C7+F7)/2</f>
-        <v>25</v>
-      </c>
-      <c r="K7" s="15">
-        <f>I7*J7</f>
-        <v>9.6824583655185421</v>
-      </c>
-      <c r="L7" s="5">
-        <f>100-ABS(G7-D7)</f>
-        <v>34</v>
-      </c>
-      <c r="M7">
-        <f>L7*K7</f>
-        <v>329.2035844276304</v>
-      </c>
-    </row>
-    <row r="8" spans="2:13">
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="15">
-        <f>SUM(I5:I7)</f>
-        <v>1.6278412151534587</v>
-      </c>
-      <c r="J8" s="15"/>
-      <c r="K8" s="13">
-        <f>SUM(K5:K7)/5</f>
-        <v>21.382552969644401</v>
-      </c>
-      <c r="L8" s="13">
-        <f>SUM(L5:L7)/5</f>
-        <v>44.8</v>
-      </c>
-      <c r="M8" s="14">
-        <f>SUM(M5:M7)/SUM(K5:K7)</f>
-        <v>90.436613964390943</v>
-      </c>
-    </row>
-    <row r="9" spans="2:13">
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5">
-        <f>I8/5</f>
-        <v>0.32556824303069176</v>
-      </c>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="2:13">
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-    </row>
-    <row r="11" spans="2:13">
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-    </row>
-    <row r="12" spans="2:13" ht="28.8">
-      <c r="B12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="M12" s="13" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="2:13">
-      <c r="B13" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C13" s="5">
-        <v>70</v>
-      </c>
-      <c r="D13" s="5">
-        <v>80</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0.9</v>
-      </c>
-      <c r="F13" s="5">
-        <v>80</v>
-      </c>
-      <c r="G13" s="5">
-        <v>72</v>
-      </c>
-      <c r="H13" s="5">
-        <v>0.9</v>
-      </c>
-      <c r="I13" s="15">
-        <f t="shared" ref="I13:I18" si="0">SQRT(H13*E13)</f>
-        <v>0.9</v>
-      </c>
-      <c r="J13" s="15">
-        <f t="shared" ref="J13:J18" si="1">(C13+F13)/2</f>
-        <v>75</v>
-      </c>
-      <c r="K13" s="15">
-        <f t="shared" ref="K13:K18" si="2">I13*J13</f>
-        <v>67.5</v>
-      </c>
-      <c r="L13" s="5">
-        <f t="shared" ref="L13:L18" si="3">100-ABS(G13-D13)</f>
-        <v>92</v>
-      </c>
-      <c r="M13">
-        <f t="shared" ref="M13:M18" si="4">L13*K13</f>
-        <v>6210</v>
-      </c>
-    </row>
-    <row r="14" spans="2:13">
-      <c r="B14" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="5">
-        <v>80</v>
-      </c>
-      <c r="D14" s="5">
-        <v>20</v>
-      </c>
-      <c r="E14" s="5">
-        <v>0.6</v>
-      </c>
-      <c r="F14" s="5">
-        <v>80</v>
-      </c>
-      <c r="G14" s="5">
-        <v>90</v>
-      </c>
-      <c r="H14" s="5">
-        <v>0.1</v>
-      </c>
-      <c r="I14" s="15">
-        <f t="shared" si="0"/>
-        <v>0.2449489742783178</v>
-      </c>
-      <c r="J14" s="15">
-        <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="K14" s="15">
-        <f t="shared" si="2"/>
-        <v>19.595917942265423</v>
-      </c>
-      <c r="L14" s="5">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-      <c r="M14">
-        <f t="shared" si="4"/>
-        <v>587.87753826796268</v>
-      </c>
-    </row>
-    <row r="15" spans="2:13">
-      <c r="B15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="5">
-        <v>50</v>
-      </c>
-      <c r="D15" s="5">
-        <v>50</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="F15" s="5">
-        <v>50</v>
-      </c>
-      <c r="G15" s="5">
-        <v>60</v>
-      </c>
-      <c r="H15" s="5">
-        <v>0.6</v>
-      </c>
-      <c r="I15" s="15">
-        <f t="shared" si="0"/>
-        <v>0.54772255750516607</v>
-      </c>
-      <c r="J15" s="15">
-        <f t="shared" si="1"/>
-        <v>50</v>
-      </c>
-      <c r="K15" s="15">
-        <f t="shared" si="2"/>
-        <v>27.386127875258303</v>
-      </c>
-      <c r="L15" s="5">
-        <f t="shared" si="3"/>
-        <v>90</v>
-      </c>
-      <c r="M15">
-        <f t="shared" si="4"/>
-        <v>2464.7515087732472</v>
-      </c>
-    </row>
-    <row r="16" spans="2:13">
-      <c r="B16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="5">
-        <v>100</v>
-      </c>
-      <c r="D16" s="5">
-        <v>100</v>
-      </c>
-      <c r="E16" s="5">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5">
-        <v>100</v>
-      </c>
-      <c r="G16" s="5">
-        <v>20</v>
-      </c>
-      <c r="H16" s="5">
-        <v>1</v>
-      </c>
-      <c r="I16" s="15">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J16" s="15">
-        <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="K16" s="15">
-        <f t="shared" si="2"/>
-        <v>100</v>
-      </c>
-      <c r="L16" s="5">
-        <f t="shared" si="3"/>
-        <v>20</v>
-      </c>
-      <c r="M16">
-        <f t="shared" si="4"/>
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13">
-      <c r="B17" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="5">
-        <v>100</v>
-      </c>
-      <c r="D17" s="5">
-        <v>66</v>
-      </c>
-      <c r="E17" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="F17" s="5">
-        <v>100</v>
-      </c>
-      <c r="G17" s="5">
-        <v>24</v>
-      </c>
-      <c r="H17" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="I17" s="15">
-        <f t="shared" si="0"/>
-        <v>0.3872983346207417</v>
-      </c>
-      <c r="J17" s="15">
-        <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="K17" s="15">
-        <f t="shared" si="2"/>
-        <v>38.729833462074168</v>
-      </c>
-      <c r="L17" s="5">
-        <f t="shared" si="3"/>
-        <v>58</v>
-      </c>
-      <c r="M17">
-        <f t="shared" si="4"/>
-        <v>2246.3303408003017</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="B18" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="5">
-        <v>20</v>
-      </c>
-      <c r="D18" s="5">
-        <v>40</v>
-      </c>
-      <c r="E18" s="5">
-        <v>0.4</v>
-      </c>
-      <c r="F18" s="5">
-        <v>100</v>
-      </c>
-      <c r="G18" s="5">
-        <v>60</v>
-      </c>
-      <c r="H18" s="5">
-        <v>0.8</v>
-      </c>
-      <c r="I18" s="15">
-        <f t="shared" si="0"/>
-        <v>0.56568542494923812</v>
-      </c>
-      <c r="J18" s="15">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="K18" s="15">
-        <f t="shared" si="2"/>
-        <v>33.941125496954285</v>
-      </c>
-      <c r="L18" s="5">
-        <f t="shared" si="3"/>
-        <v>80</v>
-      </c>
-      <c r="M18">
-        <f t="shared" si="4"/>
-        <v>2715.2900397563426</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13">
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5">
-        <f>SUM(H13:H18)/5</f>
-        <v>0.78</v>
-      </c>
-      <c r="I19" s="15">
-        <f>SUM(I13:I18)</f>
-        <v>3.6456552913534637</v>
-      </c>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="13">
-        <f>SUM(L13:L18)/5</f>
-        <v>74</v>
-      </c>
-      <c r="M19" s="14">
-        <f>SUM(M13:M18)/SUM(K13:K18)</f>
-        <v>56.500364466750881</v>
-      </c>
-    </row>
-    <row r="20" spans="2:13">
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5">
-        <f>I19/5</f>
-        <v>0.72913105827069269</v>
-      </c>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
seperation to profiled - prompt for each, calc and match by each profile + MBTI
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C895B6B7-EFFD-4E38-BFF2-5B60DFD35206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8753B1-F447-4B61-9CD1-47686D711344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
     <sheet name="Current Tasks" sheetId="16" r:id="rId2"/>
     <sheet name="Analyzer Tasks" sheetId="17" r:id="rId3"/>
-    <sheet name="פרטי משתמש" sheetId="3" r:id="rId4"/>
-    <sheet name="Internal Traits" sheetId="1" r:id="rId5"/>
-    <sheet name="internal traits - Old" sheetId="14" r:id="rId6"/>
-    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId7"/>
-    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId8"/>
-    <sheet name="בניית ציונים" sheetId="9" r:id="rId9"/>
-    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId10"/>
-    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId11"/>
-    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId12"/>
-    <sheet name="טופס הזנה" sheetId="8" r:id="rId13"/>
-    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId14"/>
-    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId15"/>
-    <sheet name="בדיקות" sheetId="13" r:id="rId16"/>
-    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId17"/>
+    <sheet name="פירוט מודל מנתח" sheetId="18" r:id="rId4"/>
+    <sheet name="פרטי משתמש" sheetId="3" r:id="rId5"/>
+    <sheet name="Internal Traits" sheetId="1" r:id="rId6"/>
+    <sheet name="internal traits - Old" sheetId="14" r:id="rId7"/>
+    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId8"/>
+    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId9"/>
+    <sheet name="בניית ציונים" sheetId="9" r:id="rId10"/>
+    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId11"/>
+    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId12"/>
+    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId13"/>
+    <sheet name="טופס הזנה" sheetId="8" r:id="rId14"/>
+    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId15"/>
+    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId16"/>
+    <sheet name="בדיקות" sheetId="13" r:id="rId17"/>
+    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="928">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3096,20 +3097,369 @@
     <t>בלי חוק ה3</t>
   </si>
   <si>
-    <t>חוק ה3</t>
-  </si>
-  <si>
     <t>חוק ה3 בלי להכפיל משקל לראיה שלילית סבירה וכן הכפלת משקלים קיצונית לשליליים עם ראיה חזקה + הכפלה יותר קיצונית לחיובים חזקים (מעל 6)</t>
   </si>
   <si>
     <t xml:space="preserve">אם אני עובדת בשיטה הזאת (כרגע על 6) - אני צריכה להתחשב בגודל הדלתאות </t>
+  </si>
+  <si>
+    <t>70/80</t>
+  </si>
+  <si>
+    <t>חוק ה6 פלוס הכפלה אקספוננציאלית</t>
+  </si>
+  <si>
+    <t>60/65/54</t>
+  </si>
+  <si>
+    <t>האקספוננציליות צריכה להתחיל כבר ב1</t>
+  </si>
+  <si>
+    <t>59/58/61</t>
+  </si>
+  <si>
+    <t>70/63/72</t>
+  </si>
+  <si>
+    <t>51/56</t>
+  </si>
+  <si>
+    <t>אצלי למשל הוא פשוט נתן את אותו סט ראיות על כל התכונות באותו דירוג, התחיל טוב עם האנליטי ואז פשוט התחיל להעתיק</t>
+  </si>
+  <si>
+    <t>81/81</t>
+  </si>
+  <si>
+    <t>44/39</t>
+  </si>
+  <si>
+    <t>חוק ה3 (עם הכפלה של 1.3 לחזקות ופי 2 לשליליות)</t>
+  </si>
+  <si>
+    <t>צריך להגיד לו אולי לא להשתמש באותן ראיות, אלא אם הן ממש חזקות</t>
+  </si>
+  <si>
+    <t>אולי לחייב לתת 2 ראיות שליליות לפחות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מצב קודם + ראיות ייחודיות, הדגשת לקיחת החזקים ביותר וסולם חוזק. </t>
+  </si>
+  <si>
+    <t>ציון באינטואיטיבית</t>
+  </si>
+  <si>
+    <t>18/22/17</t>
+  </si>
+  <si>
+    <t>75/75/75</t>
+  </si>
+  <si>
+    <t>67/73/81</t>
+  </si>
+  <si>
+    <t>72/91/99</t>
+  </si>
+  <si>
+    <t>מקרה אנה 1 - נתן  את אותן 3 ראיות שליליות למרות שהן בחוזק בינוני לכל התכונות</t>
+  </si>
+  <si>
+    <t>דבר נוסף - הוא לוקח דברים רגשיים ומשליך אותם על יכולת קוגנטיבית. כמו הימנעות מעימותים וכו'. זה קשור רק לחברתי, לא לקוגנטיבי כללי</t>
+  </si>
+  <si>
+    <t>61/58</t>
+  </si>
+  <si>
+    <t>19/48</t>
+  </si>
+  <si>
+    <t>85/81</t>
+  </si>
+  <si>
+    <t>לחשוב איך ליצור את ההתאמה, אין לי עוד אלגוריתם לזה</t>
+  </si>
+  <si>
+    <t>לסדר את האפיון, את תכנית העבודה ואת כל המשימות שלי</t>
+  </si>
+  <si>
+    <t>לקרוא מאמרים שקשורים להתאמה על בסיס כל אחת מהתכונות</t>
+  </si>
+  <si>
+    <t>לדייק כל אחד מהפרופילים</t>
+  </si>
+  <si>
+    <t>MBTI Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensing </t>
+  </si>
+  <si>
+    <t>Intuition</t>
+  </si>
+  <si>
+    <t>Thinking</t>
+  </si>
+  <si>
+    <t>Feeling</t>
+  </si>
+  <si>
+    <t>Judging</t>
+  </si>
+  <si>
+    <t>Perceiving</t>
+  </si>
+  <si>
+    <t>MBTI</t>
+  </si>
+  <si>
+    <t>חושים</t>
+  </si>
+  <si>
+    <t>שיפוט</t>
+  </si>
+  <si>
+    <t>תפיסה</t>
+  </si>
+  <si>
+    <t>חשיבה</t>
+  </si>
+  <si>
+    <t>רגשות</t>
+  </si>
+  <si>
+    <t>אינטואיציה</t>
+  </si>
+  <si>
+    <t>לחשוב איך מכניסים לסוגי התאמה ולחשוב איך להשתמש בטקסט הכללי</t>
+  </si>
+  <si>
+    <t>עמדות</t>
+  </si>
+  <si>
+    <t>סוג</t>
+  </si>
+  <si>
+    <t>אינטלגנציה רגשית חברתית</t>
+  </si>
+  <si>
+    <t>אנרגיה-סגנון תקשורת</t>
+  </si>
+  <si>
+    <t>פרופיל סגנון</t>
+  </si>
+  <si>
+    <t>מאפיינים כלליים</t>
+  </si>
+  <si>
+    <t>פרומפט</t>
+  </si>
+  <si>
+    <t>חישוב פרופיל</t>
+  </si>
+  <si>
+    <t>חישוב התאמה</t>
+  </si>
+  <si>
+    <t>כרגע יש לי שתי שיטות חישוב: 1. פרומפט שמתייחס לכל התכונות הקוגנטיביות (ללא יוקרה תעסוקתית) ומוסיף גם הערכה של אינטליגנציה אינטואיטיבית (לצורך האיזון - לאפשר לAI לפרגן בדרך פחות אנליטית).   2. שיטת הראיות -  אותו הדבר רק במקום להוציא ציון - להוציא ראיות. 6 לכל תכונה עם עדיפות ל3 שליליות ו3 חיובית, וחובה לקחת את החזקות ביותר. (בפועל זה לא בהכרח קורה, והוא גם חוזר על אותם משפטים לכל התכונות  ולא עקבי).
+לשים כרגע את שיטת הראיות בצד, להמשיך לעבוד עם הפרומפט הנוכחי אבל: לעשות כפתור של הרצה נוספת שיאפשר להריץ שוב ולעדכן את הציונים לממוצע ההרצות. צריך בעצם לשמור מערך הרצות לכל משתמש של סך הציונים שקיבל. בהמשך יכול להיות שגם נשתמש בזה כדי לבדוק פערים. אם קיבלתי פער מאוד גדול - אני עולה ארצה להעלות את זה לשיפוט עצמי. 
+בנוסף - בכל אחד מהפרומפטים האחרים נבקש ציון אינטליגנציה אנליטית ואינטליגנציה אינטואיטיבית - נשמור אותם במערך סך אינטלגנציות. ובסוף נרכיב מזה ציון אחד.
+לנרמל את הציון הקוגנטיבי בהנתן שהציונים בפועל נעים בין 20 ל90</t>
+  </si>
+  <si>
+    <t>כרגע - ממוצע כל התכונות לפי אילו שמשפיעות על הפרופיל. צריך להיות: 50% ממוצע התכונות, 50% התאמה לפי ציון כולל.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כל התכונות הקוגנטיביות כולל יוקרה תעסוקתית, לא כולל אינטואיטיבית, כאשר אנליטיות מקבל משקל משולש.
+הציון מנורמל לסקאלה של 20-90.
+לשנות בהמשך את הציון בהתאם ל: מערך אינטליגנציות מכל פרומפט, הרצה משולשת של הפרומפט.
+לשקול - לבדוק אם המשתמש הוא "רוני" ואם כן - להעלות ציון. </t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">מורכב מממוצע התכונות: אינטלגנציה אינטואיטיבית, מודעות עצמית, אינטלגנציה רגשית וערך הפוך לנוירוטיות. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">לוודא.   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">לשפר. </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">ממוצע מרחק אוקלידי. </t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות, משותף עם הפרומפט של ערכים.   לשפר בהתאם לצורך</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אין ציון. הצגת כל אחת מהתכונות והערך שלהן. </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">אין ציון. הצגת התכונות הבולטות (מעל 65 בחיובי או מתחת ל45 בשלילי - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>לוודא</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות, משותף עם הפרומפט של ביג פייב.   לשפר בהתאם לצורך</t>
+  </si>
+  <si>
+    <t>כחלק מהפרומפט של הפרופיל הרגשי.  מלבד אינטלגנציה אינטואיטיבית שמחושב בפרומפט הקוגנטיבי.</t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות בפרופיל הרגשי. לשפר בהתאם לצורך.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ממוצע כלל התכונות שתחת פרופיל רגשי מלבד אילו שהופרדו לאינטלגנציה רגשית חברתית.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>לוודא</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, לשפר</t>
+    </r>
+  </si>
+  <si>
+    <t>ממוצע מרחק אוקלידי.   
+לשקול - להתאים את המרחקים בהתאם לגבר-אישה. אחרת נשדך גברים שבממוצע יותר רגשיים לנשים שפחות. אולי חוץ מבאינטלגנציה אינטואיטיבית.</t>
+  </si>
+  <si>
+    <t>ממוצע מרחק אוקלידי. 
+לשקול - כנ"ל לסעיף הקודם, אפילו מרחק גדול יותר.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ממוצע מרחק אוקלידי. 
+</t>
+  </si>
+  <si>
+    <t>ממוצע מרחק אוקלידי.</t>
+  </si>
+  <si>
+    <t>ממוצע התכונות כאשר בחלק מהתכונות נשתמש בערך ההופכי (קשיחות, תיאטרליות וכו').  לשפר</t>
+  </si>
+  <si>
+    <t>אין ציון. הצגה של הסגנונות הבולטים (מעל 60? - לוודא).</t>
+  </si>
+  <si>
+    <t>כאן צריך להכניס מנגנון מתוחכם יותר. ככל שציון המשתמש יותר גבוה בתכונת סגנון (אולי לא כולן) - המשקל להתאמה יותר קריטי. בכללי אולי לא לכל תכונות הסגנון יש אותו משקל התאמה. 
+כמו כן - אפשר להכין קלסטרי טיפוסים שתלויים בסגנון + תכונות אחרות וליצור התאמות בהתאם.</t>
+  </si>
+  <si>
+    <t>חישוב ההתאמה בכללי מוגזם - צריך לראות איך עוברים לציונים יותר רחבים.</t>
+  </si>
+  <si>
+    <t>לכתוב לכל תכונה איזה פרומפט אחראי עליה, לאיזה פרופיל היא שייכת. (אם זה לא תואם את הקבוצה שלה)</t>
+  </si>
+  <si>
+    <t>נכניס קודם כל מרחק אוקלידי פשוט. ואז אפשר גם לחשוב על התאמת סגנונות לפי חוקי המודל (לא בטוח שכדאי, זה לא מוכח מחקרית)</t>
+  </si>
+  <si>
+    <t>אין פרומפט. מבוסס על תכונות קיימות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נציג ציון של מסורתיות שיחושב לפי דתיות, חילוניות, שמרנות וערך מסורת. (אולי להפריד את שמרנות לעמדה נפרדת שמכילה גם את הפתיחות וכו')
+נציג ציון של פוליטיות שיחושב לפי שמאל פוליטי וימין פוליטי.  אולי נחשב גם את מידת הפוליטיות הכללית.  
+לחשוב על איך לעשות את החישובים והאם יש עוד עמדות שנגזרות מכאן. </t>
+  </si>
+  <si>
+    <t>לחשוב על זה</t>
+  </si>
+  <si>
+    <t>לחשוב אם להציג בכלל בנפרד ומה נכנס כאן</t>
+  </si>
+  <si>
+    <t>אין.</t>
+  </si>
+  <si>
+    <t>לנרמל ציוני התאמה. כרגע גבוהים ומוגזמים. לבדוק שוב את החישוב שלי.</t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
+אולי להוסיף מידת הסתייגות..?</t>
+  </si>
+  <si>
+    <t>לחשב ציון התאמה לפי שילוב של גרופס + התאמה כללית בין התכונות ולשחק עם המשקלים</t>
+  </si>
+  <si>
+    <t>משימות</t>
+  </si>
+  <si>
+    <t>צריך - לעשות כפתור שמחשב רק MBTI כמו שאר הכפתורים</t>
+  </si>
+  <si>
+    <t>לבדוק מה פשר הציון של ביג פייב ערכים וסגנון בUserProfiles</t>
+  </si>
+  <si>
+    <t>אחרי שמסיים את השלב הזה של הmbti - פונקציית התאמת MBTI</t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות מלבד מוחצנות/מופנמות שכבר מחושב בביג פייב. לשפר בהתאם לצורך.  
+צריך לדייק את התכונות, למשל בין T לF - יש בעיה כשרוב השיחה היא רגשית. אולי צריך לנרמל את זה ביחס לאחרים או גם להדגיש את זה בפרומפט.
+אולי גם צריך לנרמל את ציון המוחצנות. 40=30, 60=50 או 55, ו70=80</t>
+  </si>
+  <si>
+    <t>הציון יהיה הטיפוס שנגזר מהציונים מבין 16 האישיות.
+עבור T/F - מוסיפים 20 נקודות לT לפני החישוב</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3261,6 +3611,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -3309,7 +3673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3458,7 +3822,16 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4030,6 +4403,356 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
+  <dimension ref="A1:M12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.88671875" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" customWidth="1"/>
+    <col min="12" max="12" width="37.33203125" customWidth="1"/>
+    <col min="13" max="13" width="35" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="K2" t="s">
+        <v>305</v>
+      </c>
+      <c r="L2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="57.6">
+      <c r="A3" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="K3" t="s">
+        <v>310</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="28.8">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D4:D12" si="0">MIN(A4 * 5, 100)</f>
+        <v>35</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E12" si="1">MAX(0, 100 - B4 * 10)</f>
+        <v>50</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F12" si="2">MAX(0, 100 - C4 * 10)</f>
+        <v>80</v>
+      </c>
+      <c r="G4">
+        <f t="shared" ref="G4:G12" si="3">0.4*D4+0.2*E4+0.4*F4</f>
+        <v>56</v>
+      </c>
+      <c r="K4" t="s">
+        <v>307</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="43.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="3"/>
+        <v>50</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="28.8">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="3"/>
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>312</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="3"/>
+        <v>22</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="28.8">
+      <c r="A8">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="3"/>
+        <v>64</v>
+      </c>
+      <c r="K8" t="s">
+        <v>316</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="27">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="2"/>
+        <v>50</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="3"/>
+        <v>22</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="L9" s="32" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10">
+        <v>40</v>
+      </c>
+      <c r="C10">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="28.8">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>40</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>40</v>
+      </c>
+      <c r="C12">
+        <v>10</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="3"/>
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
   <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4644,7 +5367,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487A18-0B10-40C8-BA24-F0DC1678FA48}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4929,7 +5652,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
   <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5151,7 +5874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233E8F68-8BA3-48DC-98C9-B07384CDF822}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5313,7 +6036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E73849-9796-44C6-80F8-1CA54A2F64E9}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5463,7 +6186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D465AB7-D7AD-4770-A1DB-A227111CD595}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5508,7 +6231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC47FA1-3DB6-4F73-94E7-2B8A7BD334E9}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5587,7 +6310,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC7838B-7DDE-48A8-A573-BCAB05D487CE}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5925,41 +6648,82 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50151C83-D621-46FF-871C-82BDAD5480FD}">
-  <dimension ref="B2:P22"/>
+  <dimension ref="B2:T31"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="13" max="13" width="14.77734375" customWidth="1"/>
+    <col min="14" max="14" width="16.77734375" customWidth="1"/>
+    <col min="15" max="15" width="17.109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:16">
-      <c r="P2" t="s">
+    <row r="2" spans="2:20">
+      <c r="B2" t="s">
+        <v>912</v>
+      </c>
+      <c r="R2" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="3" spans="2:16">
-      <c r="P3" t="s">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="4" spans="2:16">
+    <row r="3" spans="2:20">
+      <c r="B3" t="s">
+        <v>864</v>
+      </c>
+      <c r="R3" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20">
       <c r="B4" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="7" spans="2:16">
+    <row r="5" spans="2:20">
+      <c r="B5" t="s">
+        <v>911</v>
+      </c>
+      <c r="R5" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20">
+      <c r="R6" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20">
       <c r="B7" t="s">
         <v>813</v>
       </c>
-    </row>
-    <row r="9" spans="2:16">
-      <c r="K9" t="s">
-        <v>837</v>
+      <c r="R7" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20">
+      <c r="R8" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" ht="72.599999999999994">
+      <c r="K9" s="60" t="s">
+        <v>849</v>
       </c>
       <c r="L9" t="s">
         <v>836</v>
       </c>
-      <c r="M9" t="s">
-        <v>838</v>
-      </c>
-    </row>
-    <row r="10" spans="2:16">
+      <c r="M9" s="59" t="s">
+        <v>837</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>840</v>
+      </c>
+      <c r="O9" s="59" t="s">
+        <v>852</v>
+      </c>
+      <c r="P9" s="5" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20">
       <c r="B10" t="s">
         <v>814</v>
       </c>
@@ -5975,8 +6739,17 @@
       <c r="M10">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="2:16">
+      <c r="N10" s="58" t="s">
+        <v>844</v>
+      </c>
+      <c r="O10" t="s">
+        <v>856</v>
+      </c>
+      <c r="P10" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20">
       <c r="J11" t="s">
         <v>828</v>
       </c>
@@ -5986,14 +6759,23 @@
       <c r="L11">
         <v>51</v>
       </c>
-      <c r="M11">
-        <v>80</v>
-      </c>
-      <c r="N11">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="2:16">
+      <c r="M11" s="57" t="s">
+        <v>839</v>
+      </c>
+      <c r="N11" s="57" t="s">
+        <v>841</v>
+      </c>
+      <c r="O11" t="s">
+        <v>854</v>
+      </c>
+      <c r="P11" t="s">
+        <v>855</v>
+      </c>
+      <c r="T11" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20">
       <c r="J12" t="s">
         <v>829</v>
       </c>
@@ -6006,11 +6788,20 @@
       <c r="M12">
         <v>65</v>
       </c>
-      <c r="N12">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="2:16">
+      <c r="N12" s="58" t="s">
+        <v>845</v>
+      </c>
+      <c r="O12" t="s">
+        <v>860</v>
+      </c>
+      <c r="P12">
+        <v>48</v>
+      </c>
+      <c r="T12" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20">
       <c r="J13" t="s">
         <v>830</v>
       </c>
@@ -6023,12 +6814,18 @@
       <c r="M13">
         <v>87</v>
       </c>
+      <c r="N13" s="58" t="s">
+        <v>847</v>
+      </c>
       <c r="O13" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="14" spans="2:16">
-      <c r="B14" s="57" t="s">
+        <v>862</v>
+      </c>
+      <c r="P13">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20">
+      <c r="B14" s="58" t="s">
         <v>815</v>
       </c>
       <c r="J14" t="s">
@@ -6043,11 +6840,17 @@
       <c r="M14">
         <v>81</v>
       </c>
+      <c r="N14" s="57" t="s">
+        <v>843</v>
+      </c>
       <c r="O14" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16">
+        <v>861</v>
+      </c>
+      <c r="P14">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20">
       <c r="B15" t="s">
         <v>816</v>
       </c>
@@ -6063,11 +6866,11 @@
       <c r="M15">
         <v>51</v>
       </c>
-      <c r="O15" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16">
+      <c r="N15" s="58" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20">
       <c r="B16" t="s">
         <v>817</v>
       </c>
@@ -6076,9 +6879,6 @@
       </c>
       <c r="L16">
         <v>17</v>
-      </c>
-      <c r="O16" t="s">
-        <v>822</v>
       </c>
     </row>
     <row r="17" spans="2:15">
@@ -6088,25 +6888,49 @@
       <c r="L17">
         <v>65</v>
       </c>
-      <c r="O17" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15">
-      <c r="O18" t="s">
-        <v>824</v>
-      </c>
     </row>
     <row r="20" spans="2:15">
       <c r="B20" t="s">
         <v>818</v>
       </c>
-      <c r="O20" s="14" t="s">
-        <v>825</v>
-      </c>
     </row>
     <row r="22" spans="2:15">
       <c r="O22" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15">
+      <c r="O23" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="24" spans="2:15">
+      <c r="O24" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="25" spans="2:15">
+      <c r="O25" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15">
+      <c r="O26" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15">
+      <c r="O27" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15">
+      <c r="O29" s="14" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15">
+      <c r="O31" t="s">
         <v>826</v>
       </c>
     </row>
@@ -6116,6 +6940,253 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E890832A-DBF2-45FA-8E41-3FB9FF4AFB94}">
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="96.21875" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" customWidth="1"/>
+    <col min="4" max="5" width="40.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="14" t="s">
+        <v>883</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>888</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>889</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="158.4">
+      <c r="A2" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>891</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>893</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="100.8">
+      <c r="A3" s="5" t="s">
+        <v>884</v>
+      </c>
+      <c r="B3" t="s">
+        <v>901</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="57.6">
+      <c r="A4" t="s">
+        <v>426</v>
+      </c>
+      <c r="B4" t="s">
+        <v>902</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>903</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="28.8">
+      <c r="A5" t="s">
+        <v>693</v>
+      </c>
+      <c r="B5" t="s">
+        <v>897</v>
+      </c>
+      <c r="C5" t="s">
+        <v>898</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="28.8">
+      <c r="A6" t="s">
+        <v>429</v>
+      </c>
+      <c r="B6" t="s">
+        <v>900</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>899</v>
+      </c>
+      <c r="D6" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="43.2">
+      <c r="A7" t="s">
+        <v>885</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>908</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="86.4">
+      <c r="A8" t="s">
+        <v>886</v>
+      </c>
+      <c r="B8" t="s">
+        <v>894</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>909</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="72">
+      <c r="A9" s="58" t="s">
+        <v>874</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>927</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="100.8">
+      <c r="A10" t="s">
+        <v>882</v>
+      </c>
+      <c r="B10" t="s">
+        <v>914</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>914</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>384</v>
+      </c>
+      <c r="B12" t="s">
+        <v>914</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>887</v>
+      </c>
+      <c r="B13" t="s">
+        <v>881</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>918</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>438</v>
+      </c>
+      <c r="B14" t="s">
+        <v>863</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>916</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="14" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="14" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="14" t="s">
+        <v>924</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1C79E50-A761-4208-AC1F-7EE61CFDD025}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6636,9 +7707,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
@@ -7766,98 +8837,89 @@
     </row>
     <row r="63" spans="1:11">
       <c r="A63" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>45</v>
+        <v>867</v>
+      </c>
+      <c r="C63" t="s">
+        <v>868</v>
+      </c>
+      <c r="D63" s="38" t="s">
+        <v>875</v>
       </c>
     </row>
     <row r="64" spans="1:11">
       <c r="A64" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>792</v>
+        <v>867</v>
       </c>
       <c r="C64" t="s">
-        <v>793</v>
-      </c>
-      <c r="D64" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="28.8">
+        <v>869</v>
+      </c>
+      <c r="D64" s="38" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
       <c r="A65" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="28.8">
+        <v>867</v>
+      </c>
+      <c r="C65" t="s">
+        <v>870</v>
+      </c>
+      <c r="D65" s="38" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
       <c r="A66" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E66" s="5" t="s">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="82.8">
+        <v>867</v>
+      </c>
+      <c r="C66" t="s">
+        <v>871</v>
+      </c>
+      <c r="D66" s="38" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
       <c r="A67" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="69">
+        <v>867</v>
+      </c>
+      <c r="C67" t="s">
+        <v>872</v>
+      </c>
+      <c r="D67" s="38" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
       <c r="A68" s="2" t="s">
-        <v>430</v>
+        <v>874</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>795</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>797</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="55.2">
+        <v>867</v>
+      </c>
+      <c r="C68" t="s">
+        <v>873</v>
+      </c>
+      <c r="D68" s="38" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
       <c r="A69" s="2" t="s">
         <v>430</v>
       </c>
@@ -7865,29 +8927,122 @@
         <v>792</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>799</v>
+        <v>46</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="409.6">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
       <c r="A70" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>792</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" t="s">
+        <v>793</v>
+      </c>
+      <c r="D70" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="28.8">
+      <c r="A71" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="28.8">
+      <c r="A72" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="82.8">
+      <c r="A73" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="69">
+      <c r="A74" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="55.2">
+      <c r="A75" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="409.6">
+      <c r="A76" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>800</v>
       </c>
-      <c r="D70" s="3" t="s">
+      <c r="D76" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E76" s="3" t="s">
         <v>700</v>
       </c>
     </row>
@@ -7896,7 +9051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
   <dimension ref="A1:N136"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9990,7 +11145,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -10270,7 +11425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
   <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -10565,354 +11720,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
-  <dimension ref="A1:M12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="15.21875" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" customWidth="1"/>
-    <col min="12" max="12" width="37.33203125" customWidth="1"/>
-    <col min="13" max="13" width="35" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="K1" s="14" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="K2" t="s">
-        <v>305</v>
-      </c>
-      <c r="L2" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="57.6">
-      <c r="A3" s="14" t="s">
-        <v>225</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>228</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>229</v>
-      </c>
-      <c r="K3" t="s">
-        <v>310</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="28.8">
-      <c r="A4">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>5</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <f t="shared" ref="D4:D12" si="0">MIN(A4 * 5, 100)</f>
-        <v>35</v>
-      </c>
-      <c r="E4">
-        <f t="shared" ref="E4:E12" si="1">MAX(0, 100 - B4 * 10)</f>
-        <v>50</v>
-      </c>
-      <c r="F4">
-        <f t="shared" ref="F4:F12" si="2">MAX(0, 100 - C4 * 10)</f>
-        <v>80</v>
-      </c>
-      <c r="G4">
-        <f t="shared" ref="G4:G12" si="3">0.4*D4+0.2*E4+0.4*F4</f>
-        <v>56</v>
-      </c>
-      <c r="K4" t="s">
-        <v>307</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="43.2">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="2"/>
-        <v>80</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="3"/>
-        <v>50</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="28.8">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="2"/>
-        <v>90</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="3"/>
-        <v>56</v>
-      </c>
-      <c r="K6" t="s">
-        <v>312</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>6</v>
-      </c>
-      <c r="D7">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="2"/>
-        <v>40</v>
-      </c>
-      <c r="G7">
-        <f t="shared" si="3"/>
-        <v>22</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="28.8">
-      <c r="A8">
-        <v>14</v>
-      </c>
-      <c r="B8">
-        <v>4</v>
-      </c>
-      <c r="C8">
-        <v>4</v>
-      </c>
-      <c r="D8">
-        <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="F8">
-        <f t="shared" si="2"/>
-        <v>60</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="3"/>
-        <v>64</v>
-      </c>
-      <c r="K8" t="s">
-        <v>316</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="27">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="B9">
-        <v>10</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="D9">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="2"/>
-        <v>50</v>
-      </c>
-      <c r="G9">
-        <f t="shared" si="3"/>
-        <v>22</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>318</v>
-      </c>
-      <c r="L9" s="32" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10">
-        <v>40</v>
-      </c>
-      <c r="C10">
-        <v>10</v>
-      </c>
-      <c r="D10">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="28.8">
-      <c r="A11">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>40</v>
-      </c>
-      <c r="C11">
-        <v>10</v>
-      </c>
-      <c r="D11">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <f t="shared" si="3"/>
-        <v>14</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>40</v>
-      </c>
-      <c r="C12">
-        <v>10</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <f t="shared" si="3"/>
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
external analyze without AI prompt, communication tone score and traits update
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,29 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA97791-DDA3-4215-939B-C7C27A3BBCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECB2BEB-B87D-427A-B99B-B58A9271D2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2025" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
     <sheet name="Current Tasks" sheetId="16" r:id="rId2"/>
     <sheet name="Analyzer Tasks" sheetId="17" r:id="rId3"/>
     <sheet name="פירוט מודל מנתח" sheetId="18" r:id="rId4"/>
-    <sheet name="פרטי משתמש" sheetId="3" r:id="rId5"/>
-    <sheet name="Internal Traits" sheetId="1" r:id="rId6"/>
-    <sheet name="internal traits - Old" sheetId="14" r:id="rId7"/>
-    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId8"/>
-    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId9"/>
-    <sheet name="בניית ציונים" sheetId="9" r:id="rId10"/>
-    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId11"/>
-    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId12"/>
-    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId13"/>
-    <sheet name="טופס הזנה" sheetId="8" r:id="rId14"/>
-    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId15"/>
-    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId16"/>
-    <sheet name="בדיקות" sheetId="13" r:id="rId17"/>
-    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId18"/>
+    <sheet name="external traits analyze" sheetId="19" r:id="rId5"/>
+    <sheet name="פרטי משתמש" sheetId="3" r:id="rId6"/>
+    <sheet name="Internal Traits" sheetId="1" r:id="rId7"/>
+    <sheet name="internal traits - Old" sheetId="14" r:id="rId8"/>
+    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId9"/>
+    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId10"/>
+    <sheet name="בניית ציונים" sheetId="9" r:id="rId11"/>
+    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId12"/>
+    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId13"/>
+    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId14"/>
+    <sheet name="טופס הזנה" sheetId="8" r:id="rId15"/>
+    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId16"/>
+    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId17"/>
+    <sheet name="בדיקות" sheetId="13" r:id="rId18"/>
+    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="1024">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -2848,12 +2849,6 @@
     <t>Intellectualism</t>
   </si>
   <si>
-    <t>Directness</t>
-  </si>
-  <si>
-    <t>ישירות</t>
-  </si>
-  <si>
     <t>עדינות</t>
   </si>
   <si>
@@ -2869,9 +2864,6 @@
     <t>Cognitive Profile</t>
   </si>
   <si>
-    <t>Harsh talk</t>
-  </si>
-  <si>
     <t>Big Five</t>
   </si>
   <si>
@@ -2888,9 +2880,6 @@
   </si>
   <si>
     <t>social_activism</t>
-  </si>
-  <si>
-    <t>אותנטיות</t>
   </si>
   <si>
     <t>Personal Style</t>
@@ -2925,13 +2914,7 @@
 </t>
   </si>
   <si>
-    <t>Dramatic Intensity</t>
-  </si>
-  <si>
     <t>Theatricality</t>
-  </si>
-  <si>
-    <t>Energy Level</t>
   </si>
   <si>
     <t>מידת דתיות</t>
@@ -3175,9 +3158,6 @@
     <t>85/81</t>
   </si>
   <si>
-    <t>לחשוב איך ליצור את ההתאמה, אין לי עוד אלגוריתם לזה</t>
-  </si>
-  <si>
     <t>לסדר את האפיון, את תכנית העבודה ואת כל המשימות שלי</t>
   </si>
   <si>
@@ -3257,12 +3237,6 @@
   </si>
   <si>
     <t>חישוב התאמה</t>
-  </si>
-  <si>
-    <t xml:space="preserve">כל התכונות הקוגנטיביות כולל יוקרה תעסוקתית, לא כולל אינטואיטיבית, כאשר אנליטיות מקבל משקל משולש.
-הציון מנורמל לסקאלה של 20-90.
-לשנות בהמשך את הציון בהתאם ל: מערך אינטליגנציות מכל פרומפט, הרצה משולשת של הפרומפט.
-לשקול - לבדוק אם המשתמש הוא "רוני" ואם כן - להעלות ציון. </t>
   </si>
   <si>
     <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך</t>
@@ -3390,11 +3364,6 @@
     <t>אין פרומפט. מבוסס על תכונות קיימות</t>
   </si>
   <si>
-    <t xml:space="preserve">נציג ציון של מסורתיות שיחושב לפי דתיות, חילוניות, שמרנות וערך מסורת. (אולי להפריד את שמרנות לעמדה נפרדת שמכילה גם את הפתיחות וכו')
-נציג ציון של פוליטיות שיחושב לפי שמאל פוליטי וימין פוליטי.  אולי נחשב גם את מידת הפוליטיות הכללית.  
-לחשוב על איך לעשות את החישובים והאם יש עוד עמדות שנגזרות מכאן. </t>
-  </si>
-  <si>
     <t>לחשוב על זה</t>
   </si>
   <si>
@@ -3405,10 +3374,6 @@
   </si>
   <si>
     <t>לנרמל ציוני התאמה. כרגע גבוהים ומוגזמים. לבדוק שוב את החישוב שלי.</t>
-  </si>
-  <si>
-    <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
-אולי להוסיף מידת הסתייגות..?</t>
   </si>
   <si>
     <t>לחשב ציון התאמה לפי שילוב של גרופס + התאמה כללית בין התכונות ולשחק עם המשקלים</t>
@@ -3429,9 +3394,6 @@
 עבור T/F - מוסיפים 20 נקודות לT לפני החישוב</t>
   </si>
   <si>
-    <t>נכניס קודם כל מרחק אוקלידי פשוט. ואז אפשר גם לחשוב על התאמת סגנונות לפי חוקי המודל (לא בטוח שכדאי, זה לא מוכח מחקרית). כן כדאי להתאים בין אותו טיפוס. לתת ציון אקסטרה אם הם אותו הטיפוס הסופי.</t>
-  </si>
-  <si>
     <t>כרגע - ממוצע כל התכונות לפי אילו שמשפיעות על הפרופיל. צריך להיות: 50% ממוצע התכונות, 50% התאמה לפי ציון כולל.
 הפרופיל הקוגנטיבי גם מסנן התאמות במרחק 7 נקודות.</t>
   </si>
@@ -3441,22 +3403,358 @@
   <si>
     <t>ממוצע מרחק אוקלידי. 
 לשקול - כנ"ל לסעיף הקודם, תיקון ל10 נקודות לטובת האישה.</t>
+  </si>
+  <si>
+    <t>50% ממוצע מרחק אוקלידי.   
+50%- התאמה לפי ציון פרופיל עם התאמה של בהתאם לגבר-אישה. אחרת נשדך גברים שבממוצע יותר רגשיים לנשים שפחות.  תיקון ל4 נקודות לטובת האישה.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
+להוסיף אולי מידת הסתייגות.. ובכללי לקרוא על הנושא כדי לפתח את זה נכון יותר. </t>
+  </si>
+  <si>
+    <t>קטגוריה</t>
+  </si>
+  <si>
+    <t>תיאור</t>
+  </si>
+  <si>
+    <t>Visual Appeal Band</t>
+  </si>
+  <si>
+    <t>רמת אטרקטיביות כללית (פנימי בלבד)</t>
+  </si>
+  <si>
+    <t>1 Very Low / 2 Low / 3 Moderate / 4 High / 5 Very High</t>
+  </si>
+  <si>
+    <t>Body Type</t>
+  </si>
+  <si>
+    <t>מבנה גוף כללי</t>
+  </si>
+  <si>
+    <t>Slim / Fit / Average / Curvy / Heavyset</t>
+  </si>
+  <si>
+    <t>Fit</t>
+  </si>
+  <si>
+    <t>Fitness Signal</t>
+  </si>
+  <si>
+    <t>עד כמה נראה פעיל/חטוב</t>
+  </si>
+  <si>
+    <t>Low / Moderate / High</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Grooming Level</t>
+  </si>
+  <si>
+    <t>רמת טיפוח והשקעה</t>
+  </si>
+  <si>
+    <t>Minimal / Moderate / High</t>
+  </si>
+  <si>
+    <t>Style Category</t>
+  </si>
+  <si>
+    <t>סגנון חיצוני</t>
+  </si>
+  <si>
+    <t>Natural / Casual / Polished / Elegant / Glamorous / Alternative</t>
+  </si>
+  <si>
+    <t>Polished</t>
+  </si>
+  <si>
+    <t>Facial Structure</t>
+  </si>
+  <si>
+    <t>מבנה פנים</t>
+  </si>
+  <si>
+    <t>Soft / Balanced / Sharp / Strong-featured / Delicate</t>
+  </si>
+  <si>
+    <t>Sharp</t>
+  </si>
+  <si>
+    <t>Facial Archetype</t>
+  </si>
+  <si>
+    <t>vibe כללי של הפנים</t>
+  </si>
+  <si>
+    <t>Warm / Elegant / Glamorous / Natural / Intellectual / Edgy / Youthful / Mature</t>
+  </si>
+  <si>
+    <t>Warm + Elegant</t>
+  </si>
+  <si>
+    <t>Energy Projection</t>
+  </si>
+  <si>
+    <t>אנרגיה כללית</t>
+  </si>
+  <si>
+    <t>Soft / Feminine / Masculine / Dominant / Playful / Reserved</t>
+  </si>
+  <si>
+    <t>Soft</t>
+  </si>
+  <si>
+    <t>Skin Tone Range</t>
+  </si>
+  <si>
+    <t>טווח גוון חזותי כללי (לא אתני)</t>
+  </si>
+  <si>
+    <t>Fair / Light-Medium / Medium / Olive / Deep</t>
+  </si>
+  <si>
+    <t>Olive</t>
+  </si>
+  <si>
+    <t>Contrast Level</t>
+  </si>
+  <si>
+    <t>ניגודיות כללית (שיער/עור/תווי פנים)</t>
+  </si>
+  <si>
+    <t>Low / Medium / High</t>
+  </si>
+  <si>
+    <t>Overall Presentation</t>
+  </si>
+  <si>
+    <t>רושם כללי</t>
+  </si>
+  <si>
+    <t>Understated / Balanced / Striking</t>
+  </si>
+  <si>
+    <t>Striking</t>
+  </si>
+  <si>
+    <t>Visual Appeal Band – 20%</t>
+  </si>
+  <si>
+    <t>• Body Type/Fitness – 25%</t>
+  </si>
+  <si>
+    <t>• Style/Grooming – 20%</t>
+  </si>
+  <si>
+    <t>• Facial Archetype – 25%</t>
+  </si>
+  <si>
+    <t>• Presentation/Energy – 10%</t>
+  </si>
+  <si>
+    <t>אפשר לשמור גם כסקאלה (לדוגמה)</t>
+  </si>
+  <si>
+    <t>אורית</t>
+  </si>
+  <si>
+    <t>4 או 5</t>
+  </si>
+  <si>
+    <t>Average/curvery</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>Natural/casutal/soft polished</t>
+  </si>
+  <si>
+    <t>soft/balanced</t>
+  </si>
+  <si>
+    <t>warm/feminin/natural</t>
+  </si>
+  <si>
+    <t>soft/warm/maternal</t>
+  </si>
+  <si>
+    <t>Light Medium/olive</t>
+  </si>
+  <si>
+    <t>Appeal</t>
+  </si>
+  <si>
+    <t>warmth</t>
+  </si>
+  <si>
+    <t>Glamour</t>
+  </si>
+  <si>
+    <t>Naturalness</t>
+  </si>
+  <si>
+    <t>Fitness aesthetic</t>
+  </si>
+  <si>
+    <t>Style polish</t>
+  </si>
+  <si>
+    <t>• Softness</t>
+  </si>
+  <si>
+    <t>• Sharpness</t>
+  </si>
+  <si>
+    <t>• Dominance</t>
+  </si>
+  <si>
+    <t>• Approachability</t>
+  </si>
+  <si>
+    <t>• Trendiness</t>
+  </si>
+  <si>
+    <t>• Elegance</t>
+  </si>
+  <si>
+    <t>• Distinctiveness</t>
+  </si>
+  <si>
+    <t>נוי</t>
+  </si>
+  <si>
+    <t>Femininity/Masculinity</t>
+  </si>
+  <si>
+    <t>אמיר</t>
+  </si>
+  <si>
+    <t>לי</t>
+  </si>
+  <si>
+    <t>מירה</t>
+  </si>
+  <si>
+    <t>ציון מינימום בפועל</t>
+  </si>
+  <si>
+    <t>1–15 = very fair</t>
+  </si>
+  <si>
+    <t>• 16–30 = fair/light</t>
+  </si>
+  <si>
+    <t>• 31–50 = light-medium</t>
+  </si>
+  <si>
+    <t>• 51–70 = medium/olive</t>
+  </si>
+  <si>
+    <t>• 71–85 = deeper olive/tan</t>
+  </si>
+  <si>
+    <t>• 86–100 = deep/dark</t>
+  </si>
+  <si>
+    <t>טווח skine tone</t>
+  </si>
+  <si>
+    <t>הזנת התכונות באופן ידני / על ידי AI בהתאם ל3 התמונות שישלחו (להדגיש למשתמשים שכדאי תמונות ברורות ותמונות גוף מלא, אם זה סבבה לבקש...)</t>
+  </si>
+  <si>
+    <t>בהעלאת תמונה - אישור ניתוח על ידי AI (ביומטרי). אם מסמנים לא - אישור ניתוח ידני. אם מסמנים לא - הבהרה שלא יהיה לנו ניתוח מראה והמשתמשים יוצגו בלי קשר למראה חיצוני (ובמאגר נפרד, צריך לחשוב אם ואיך להסביר את זה. לא ברור אם צריך לגמרי מאגר נפרד או פשוט ציון התאמה חיצוני  = 0 שישפיע על האפשרויות)</t>
+  </si>
+  <si>
+    <t>לומר למשתמשים שהם יכולים לשנות את ההסכמה בכל עת וגם לדון על זה בצ'אט ( הצ'אט צריך להיות מסוגל לספר להם למה צריך כל דבר ומה המשמעויות)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">שילוב של הציונים מהAI + שיעור אישור שמחושב על ידי המערכת.  כרגע מתייחסים רק לציונים מהAI שהם בעצם ידניים כרגע. </t>
+  </si>
+  <si>
+    <t>להוסיף! אבל לחשוב איך להשתמש בזה</t>
+  </si>
+  <si>
+    <t>יכול להשפיע על העממיות אולי, לבדוק אם זה קונסיסטנט</t>
+  </si>
+  <si>
+    <t>נחלק לשתי קטגוריות של תכונות: הראשונה - 6 שהAI מנתח (או ניתוח ידני) עם ציון בכל תכונה (כולל מידת אטרקטיביות כללית, גבריות/נשיות, מבנה גוף וצבע עור, רק במונחים יותר עדינים ופוליטיקלי קורקט).  השניה - תכונות יבשות כמו גובה, צבע שיער עיניים וכו' (חלק מהם גם הAI ינתח). + שיעור אישור.  צריך לחשוב על פרומפט טוב לנושא, וצריך להתכסות מבחינה משפטית, אנושית ושקיפות למשתמש ככל הניתן. 
+הAppeal צריך לשמש גם כמסנן ראשוני במקרים קיצוניים כמו שיעור האישור (אולי במקומו). בנוסף עבור משתמשים שביקשו מפורשות גם המבנה גוף צריך להיות מסנן (אבל עם טווח רחב יחסית, או לפחות בהתחשב בודאות)
+*כל עוד אני עושה ניתוח ידני אני צריכה סקאלות ברורות כמו שאני  נותנת לAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">נכניס קודם כל מרחק אוקלידי פשוט. ואז אפשר גם לחשוב על התאמת סגנונות לפי חוקי המודל (לא בטוח שכדאי, זה לא מוכח מחקרית). כן כדאי להתאים בין אותו טיפוס. לתת ציון אקסטרה אם הם אותו הטיפוס הסופי.
+לפי המודל - הדמיון הכי קריטי הוא בציר הN/S מעבר לזה - דמיון הוא לא תמיד רצוי. התאמה טובה תהיה שני צירים זהים ו2 שונים, אבל לא בטוח שנרצה את זה במקרה שלנו. צריך לחשוב איך לחשב. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">נציג ציון של מסורתיות שיחושב לפי דתיות, חילוניות, שמרנות וערך מסורת. (אולי להפריד את שמרנות לעמדה נפרדת שמכילה גם את הפתיחות וכו')
+נציג ציון של פוליטיות שיחושב לפי שמאל פוליטי וימין פוליטי.  אולי נחשב גם את מידת הפוליטיות הכללית.  
+לחשוב על איך לעשות את החישובים והאם יש עוד עמדות שנגזרות מכאן. 
+אחרי הרכבת העמדות - להוציא אותן מהסגנון </t>
+  </si>
+  <si>
+    <t>כרגע מרחק רגיל בין הציונים. צריך - להתאים לטווחים האמיתיים, להוסיף התייחסות לשיעור אישור ולהתאים לבקשות המשתמש הספציפי. 
+חישוב המראה צריך להיות שונה אצל גייז, בעיקר במובן של נשיות/גבריות אבל גם לשים לב שזה משפיע על הציון הכללי.  כמו כן - אולי כדאי להתייחס אחרת אצל אנשים שבאמת לא רגישים למראה באופן מפורש.
+אולי צריך להתייחס שונה לאישור של הצד האטרקטיבי יותר. לחשוב על זה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">כרגע יש לי שתי שיטות חישוב: 1. פרומפט שמתייחס לכל התכונות הקוגנטיביות (ללא יוקרה תעסוקתית) ומוסיף גם הערכה של אינטליגנציה אינטואיטיבית (לצורך האיזון - לאפשר לAI לפרגן בדרך פחות אנליטית).   2. שיטת הראיות -  אותו הדבר רק במקום להוציא ציון - להוציא ראיות. 6 לכל תכונה עם עדיפות ל3 שליליות ו3 חיובית, וחובה לקחת את החזקות ביותר. (בפועל זה לא בהכרח קורה, והוא גם חוזר על אותם משפטים לכל התכונות  ולא עקבי).
+לשים כרגע את שיטת הראיות בצד, להמשיך לעבוד עם הפרומפט הנוכחי אבל: לעשות כפתור של הרצה נוספת שיאפשר להריץ שוב ולעדכן את הציונים לממוצע ההרצות. צריך בעצם לשמור מערך הרצות לכל משתמש של סך הציונים שקיבל. בהמשך יכול להיות שגם נשתמש בזה כדי לבדוק פערים. אם קיבלתי פער מאוד גדול - אני עולה ארצה להעלות את זה לשיפוט עצמי. 
+בנוסף - בכל אחד מהפרומפטים האחרים נבקש ציון אינטליגנציה אנליטית ואינטליגנציה אינטואיטיבית - נשמור אותם במערך סך אינטלגנציות. ובסוף נרכיב מזה ציון אחד (לא בטוחה לגבי זה, אולי זה לא ידייק וסתם יתן רעש).
+לנרמל את הציון הקוגנטיבי בהנתן שהציונים בפועל נעים בין 20 ל90  (נראה לי שכבר עשיתתי את זה)
+המשוחח חייב לשאול את המשתמשים על השכלה וכו' כדי לדייק את הפרופיל הקוגנטיבי. וגם לשאול מה למדו/עשו בעבר. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">כל התכונות הקוגנטיביות כולל יוקרה תעסוקתית, לא כולל אינטואיטיבית, כאשר אנליטיות מקבל משקל משולש.
+הציון מנורמל לסקאלה של 20-90.
+לשנות בהמשך את הציון בהתאם ל: מערך אינטליגנציות מכל פרומפט, הרצה משולשת של הפרומפט.
+לשקול - לבדוק אם המשתמש הוא "רוני" ואם כן - להעלות ציון. 
+יכול להיות שצריך להתייחס למצב שבו הפער בין הפרופיל הקוגנטיבי לאינטואיטיבי הוא גדול. </t>
+  </si>
+  <si>
+    <t>energetic_intensity</t>
+  </si>
+  <si>
+    <t>assertiveness_forcefulness</t>
+  </si>
+  <si>
+    <t>אסרטיביות</t>
+  </si>
+  <si>
+    <t>charismatic_presence</t>
+  </si>
+  <si>
+    <t>נוכחות כריזמתית</t>
+  </si>
+  <si>
+    <t>softness_sharpness_balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hesitation </t>
+  </si>
+  <si>
+    <t>מידת הסתייגות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">אולי כדאי לשקול שינוי במשקלים של התכונות. נגיד אנרגיה ורמה קוגנטיבית כבסיס ואז את השאר...  בטוח צריך לתת משקלים גבוהים יותר בהתאם לרמת הציונים בחלק מהתכונות כמו נהנתנות, סגנונות וערכים מסוימים </t>
+  </si>
+  <si>
+    <t xml:space="preserve">בכל חישובי הציונים - גם ברמת התכונה וגם ברמת הפרופיל צריך להתאים לטווחים בפועל. </t>
   </si>
   <si>
     <t>כרגע חישוב הציונים נעשה לפי מרחק אוקלידי בין כל התכונות. שיניתי כך שיתאים לפערים הנוכחיים: עד 5 - התאמה טובה, 15 - התאמה לא טובה.  צריך לדייק את זה פר תכונה וגם להתחשב עבור כל תכונה בטווח האמיתי (שהAI נותן בפועל, כמו שעשינו בקוגנטיבי). 
 הציון הסופי מורכב מסך הציונים, כאשר לתכונות עם ודאות נמוכה יותר - יש פחות משקל בציון הסופי.
 בתוך כל פרופיל - מחושב באותו אופן עם דקויות של הפרופיל שמתוארות למעלה.
-לעבור לחישוב לפי פרופילים + אולי גם אחוז  מסוים לחישוב הכללי. כרגע ציון הפרופילים הוא ממוצע ציוני הפרופיל כאשר הפרופיל הקוגנטיבי מקבל משקל כפול. סחיות, עממיות ומידע כללי לא נכנסים</t>
-  </si>
-  <si>
-    <t>50% ממוצע מרחק אוקלידי.   
-50%- התאמה לפי ציון פרופיל עם התאמה של בהתאם לגבר-אישה. אחרת נשדך גברים שבממוצע יותר רגשיים לנשים שפחות.  תיקון ל4 נקודות לטובת האישה.</t>
-  </si>
-  <si>
-    <t>כרגע יש לי שתי שיטות חישוב: 1. פרומפט שמתייחס לכל התכונות הקוגנטיביות (ללא יוקרה תעסוקתית) ומוסיף גם הערכה של אינטליגנציה אינטואיטיבית (לצורך האיזון - לאפשר לAI לפרגן בדרך פחות אנליטית).   2. שיטת הראיות -  אותו הדבר רק במקום להוציא ציון - להוציא ראיות. 6 לכל תכונה עם עדיפות ל3 שליליות ו3 חיובית, וחובה לקחת את החזקות ביותר. (בפועל זה לא בהכרח קורה, והוא גם חוזר על אותם משפטים לכל התכונות  ולא עקבי).
-לשים כרגע את שיטת הראיות בצד, להמשיך לעבוד עם הפרומפט הנוכחי אבל: לעשות כפתור של הרצה נוספת שיאפשר להריץ שוב ולעדכן את הציונים לממוצע ההרצות. צריך בעצם לשמור מערך הרצות לכל משתמש של סך הציונים שקיבל. בהמשך יכול להיות שגם נשתמש בזה כדי לבדוק פערים. אם קיבלתי פער מאוד גדול - אני עולה ארצה להעלות את זה לשיפוט עצמי. 
-בנוסף - בכל אחד מהפרומפטים האחרים נבקש ציון אינטליגנציה אנליטית ואינטליגנציה אינטואיטיבית - נשמור אותם במערך סך אינטלגנציות. ובסוף נרכיב מזה ציון אחד (לא בטוחה לגבי זה, אולי זה לא ידייק וסתם יתן רעש).
-לנרמל את הציון הקוגנטיבי בהנתן שהציונים בפועל נעים בין 20 ל90</t>
+לעבור לחישוב לפי פרופילים + אולי גם אחוז  מסוים לחישוב הכללי. כרגע ציון הפרופילים הוא ממוצע ציוני הפרופיל כאשר הפרופיל הקוגנטיבי מקבל משקל כפול. סחיות, עממיות ומידע כללי לא נכנסים.
+לגבי המראה כרגע הוא נכנס לחישוב הכללי כ30 אחוז או 35 למשתמשים רגישים (ציון 70 ומעלה בודאות 0.7 ומעלה), ולחישוב הפרופילים נכנס כפרופיל נוסף עם משקל כפול.  לחשוב על זה, כי מצד אחד אני רוצה שברושם הראשוני אני אציג משתמשים שקשורים מבחינת מראה, מצד שני - אני רוצה לתת משקל מהותי יותר לאישיות, והמראה הוא רק מסנן. בסופו של דבר - בחירת המשתמש תחליף (או תשנה משמעותית) את הציון לפי מראה, ואז להחליט איזה משקל לתת לזה.   לקחת בחשבון גם שהתמונות יכולות להטעות, בעיקר את הAI, כמו במקרה אורית/הילה</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בחישוב לפי פרופילים שיחקתי קצת עם המשקלים, בגדול כדי להתאים יותר לנוי ורון אז צריך לראות שזה באמת אמין. </t>
   </si>
 </sst>
 </file>
@@ -3677,7 +3975,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3839,6 +4137,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4410,6 +4720,303 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="5"/>
+    <col min="2" max="2" width="16.88671875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13" style="5" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="13" style="5" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="25.109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="44.44140625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="E3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="27.6">
+      <c r="A4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="28.8">
+      <c r="C5" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="41.4">
+      <c r="A9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="J9"/>
+    </row>
+    <row r="10" spans="1:10" ht="43.2">
+      <c r="C10" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="J10" s="17"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+      <c r="J12"/>
+    </row>
+    <row r="13" spans="1:10" ht="15.6">
+      <c r="A13" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="18"/>
+      <c r="F13"/>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13"/>
+      <c r="J13"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="J14"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="J15"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16"/>
+      <c r="J16"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="4"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="19"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="B28"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="B29"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="B30"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="B31"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="B32"/>
+    </row>
+    <row r="33" spans="2:9">
+      <c r="B33"/>
+    </row>
+    <row r="35" spans="2:9">
+      <c r="B35" s="14"/>
+    </row>
+    <row r="37" spans="2:9">
+      <c r="B37"/>
+      <c r="I37"/>
+    </row>
+    <row r="38" spans="2:9">
+      <c r="I38"/>
+    </row>
+    <row r="39" spans="2:9">
+      <c r="I39"/>
+    </row>
+    <row r="41" spans="2:9">
+      <c r="I41"/>
+    </row>
+    <row r="49" spans="2:2">
+      <c r="B49"/>
+    </row>
+    <row r="51" spans="2:2">
+      <c r="B51"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -4759,7 +5366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
   <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5374,7 +5981,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487A18-0B10-40C8-BA24-F0DC1678FA48}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5659,7 +6266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
   <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5881,7 +6488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233E8F68-8BA3-48DC-98C9-B07384CDF822}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6043,7 +6650,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E73849-9796-44C6-80F8-1CA54A2F64E9}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6193,7 +6800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D465AB7-D7AD-4770-A1DB-A227111CD595}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6238,7 +6845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC47FA1-3DB6-4F73-94E7-2B8A7BD334E9}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6317,7 +6924,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC7838B-7DDE-48A8-A573-BCAB05D487CE}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6665,77 +7272,77 @@
   <sheetData>
     <row r="2" spans="2:20">
       <c r="B2" t="s">
-        <v>908</v>
+        <v>900</v>
       </c>
       <c r="R2" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
     </row>
     <row r="3" spans="2:20">
       <c r="B3" t="s">
-        <v>864</v>
+        <v>857</v>
       </c>
       <c r="R3" t="s">
-        <v>838</v>
+        <v>832</v>
       </c>
     </row>
     <row r="4" spans="2:20">
       <c r="B4" t="s">
-        <v>812</v>
+        <v>806</v>
       </c>
     </row>
     <row r="5" spans="2:20">
       <c r="B5" t="s">
-        <v>907</v>
+        <v>899</v>
       </c>
       <c r="R5" t="s">
-        <v>842</v>
+        <v>836</v>
       </c>
     </row>
     <row r="6" spans="2:20">
       <c r="R6" t="s">
-        <v>846</v>
+        <v>840</v>
       </c>
     </row>
     <row r="7" spans="2:20">
       <c r="B7" t="s">
-        <v>813</v>
+        <v>807</v>
       </c>
       <c r="R7" t="s">
-        <v>850</v>
+        <v>844</v>
       </c>
     </row>
     <row r="8" spans="2:20">
       <c r="R8" t="s">
-        <v>851</v>
+        <v>845</v>
       </c>
     </row>
     <row r="9" spans="2:20" ht="72.599999999999994">
       <c r="K9" s="60" t="s">
-        <v>849</v>
+        <v>843</v>
       </c>
       <c r="L9" t="s">
-        <v>836</v>
+        <v>830</v>
       </c>
       <c r="M9" s="59" t="s">
-        <v>837</v>
+        <v>831</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>840</v>
+        <v>834</v>
       </c>
       <c r="O9" s="59" t="s">
-        <v>852</v>
+        <v>846</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>853</v>
+        <v>847</v>
       </c>
     </row>
     <row r="10" spans="2:20">
       <c r="B10" t="s">
-        <v>814</v>
+        <v>808</v>
       </c>
       <c r="J10" t="s">
-        <v>827</v>
+        <v>821</v>
       </c>
       <c r="K10">
         <v>90</v>
@@ -6747,18 +7354,18 @@
         <v>82</v>
       </c>
       <c r="N10" s="58" t="s">
-        <v>844</v>
+        <v>838</v>
       </c>
       <c r="O10" t="s">
-        <v>856</v>
+        <v>850</v>
       </c>
       <c r="P10" t="s">
-        <v>857</v>
+        <v>851</v>
       </c>
     </row>
     <row r="11" spans="2:20">
       <c r="J11" t="s">
-        <v>828</v>
+        <v>822</v>
       </c>
       <c r="K11">
         <v>58</v>
@@ -6767,24 +7374,24 @@
         <v>51</v>
       </c>
       <c r="M11" s="57" t="s">
-        <v>839</v>
+        <v>833</v>
       </c>
       <c r="N11" s="57" t="s">
-        <v>841</v>
+        <v>835</v>
       </c>
       <c r="O11" t="s">
-        <v>854</v>
+        <v>848</v>
       </c>
       <c r="P11" t="s">
-        <v>855</v>
+        <v>849</v>
       </c>
       <c r="T11" t="s">
-        <v>858</v>
+        <v>852</v>
       </c>
     </row>
     <row r="12" spans="2:20">
       <c r="J12" t="s">
-        <v>829</v>
+        <v>823</v>
       </c>
       <c r="K12">
         <v>81</v>
@@ -6796,21 +7403,21 @@
         <v>65</v>
       </c>
       <c r="N12" s="58" t="s">
-        <v>845</v>
+        <v>839</v>
       </c>
       <c r="O12" t="s">
-        <v>860</v>
+        <v>854</v>
       </c>
       <c r="P12">
         <v>48</v>
       </c>
       <c r="T12" t="s">
-        <v>859</v>
+        <v>853</v>
       </c>
     </row>
     <row r="13" spans="2:20">
       <c r="J13" t="s">
-        <v>830</v>
+        <v>824</v>
       </c>
       <c r="K13">
         <v>93</v>
@@ -6822,10 +7429,10 @@
         <v>87</v>
       </c>
       <c r="N13" s="58" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="O13" t="s">
-        <v>862</v>
+        <v>856</v>
       </c>
       <c r="P13">
         <v>75</v>
@@ -6833,10 +7440,10 @@
     </row>
     <row r="14" spans="2:20">
       <c r="B14" s="58" t="s">
-        <v>815</v>
+        <v>809</v>
       </c>
       <c r="J14" t="s">
-        <v>831</v>
+        <v>825</v>
       </c>
       <c r="K14">
         <v>63</v>
@@ -6848,10 +7455,10 @@
         <v>81</v>
       </c>
       <c r="N14" s="57" t="s">
-        <v>843</v>
+        <v>837</v>
       </c>
       <c r="O14" t="s">
-        <v>861</v>
+        <v>855</v>
       </c>
       <c r="P14">
         <v>45</v>
@@ -6859,10 +7466,10 @@
     </row>
     <row r="15" spans="2:20">
       <c r="B15" t="s">
-        <v>816</v>
+        <v>810</v>
       </c>
       <c r="J15" t="s">
-        <v>832</v>
+        <v>826</v>
       </c>
       <c r="K15">
         <v>54</v>
@@ -6874,15 +7481,15 @@
         <v>51</v>
       </c>
       <c r="N15" s="58" t="s">
-        <v>848</v>
+        <v>842</v>
       </c>
     </row>
     <row r="16" spans="2:20">
       <c r="B16" t="s">
-        <v>817</v>
+        <v>811</v>
       </c>
       <c r="J16" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="L16">
         <v>17</v>
@@ -6890,7 +7497,7 @@
     </row>
     <row r="17" spans="2:15">
       <c r="J17" t="s">
-        <v>834</v>
+        <v>828</v>
       </c>
       <c r="L17">
         <v>65</v>
@@ -6898,47 +7505,47 @@
     </row>
     <row r="20" spans="2:15">
       <c r="B20" t="s">
-        <v>818</v>
+        <v>812</v>
       </c>
     </row>
     <row r="22" spans="2:15">
       <c r="O22" t="s">
-        <v>819</v>
+        <v>813</v>
       </c>
     </row>
     <row r="23" spans="2:15">
       <c r="O23" t="s">
-        <v>820</v>
+        <v>814</v>
       </c>
     </row>
     <row r="24" spans="2:15">
       <c r="O24" t="s">
-        <v>821</v>
+        <v>815</v>
       </c>
     </row>
     <row r="25" spans="2:15">
       <c r="O25" t="s">
-        <v>822</v>
+        <v>816</v>
       </c>
     </row>
     <row r="26" spans="2:15">
       <c r="O26" t="s">
-        <v>823</v>
+        <v>817</v>
       </c>
     </row>
     <row r="27" spans="2:15">
       <c r="O27" t="s">
-        <v>824</v>
+        <v>818</v>
       </c>
     </row>
     <row r="29" spans="2:15">
       <c r="O29" s="14" t="s">
-        <v>825</v>
+        <v>819</v>
       </c>
     </row>
     <row r="31" spans="2:15">
       <c r="O31" t="s">
-        <v>826</v>
+        <v>820</v>
       </c>
     </row>
   </sheetData>
@@ -6959,44 +7566,44 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="14" t="s">
+        <v>876</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>881</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>882</v>
+      </c>
+      <c r="D1" s="14" t="s">
         <v>883</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>888</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>889</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>890</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="158.4">
+    </row>
+    <row r="2" spans="1:7" ht="187.2">
       <c r="A2" s="5" t="s">
         <v>415</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>927</v>
+        <v>1010</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>891</v>
+        <v>1011</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>922</v>
+        <v>911</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="86.4">
       <c r="A3" s="5" t="s">
-        <v>884</v>
+        <v>877</v>
       </c>
       <c r="B3" t="s">
-        <v>899</v>
+        <v>891</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>893</v>
+        <v>885</v>
       </c>
       <c r="D3" s="61" t="s">
-        <v>926</v>
+        <v>914</v>
       </c>
       <c r="G3" s="14"/>
     </row>
@@ -7005,13 +7612,13 @@
         <v>426</v>
       </c>
       <c r="B4" t="s">
-        <v>900</v>
+        <v>892</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>901</v>
+        <v>893</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>924</v>
+        <v>913</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8">
@@ -7019,13 +7626,13 @@
         <v>693</v>
       </c>
       <c r="B5" t="s">
-        <v>895</v>
+        <v>887</v>
       </c>
       <c r="C5" t="s">
-        <v>896</v>
+        <v>888</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>902</v>
+        <v>894</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.8">
@@ -7033,69 +7640,69 @@
         <v>429</v>
       </c>
       <c r="B6" t="s">
-        <v>898</v>
+        <v>890</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>897</v>
+        <v>889</v>
       </c>
       <c r="D6" t="s">
-        <v>894</v>
+        <v>886</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2">
       <c r="A7" t="s">
-        <v>885</v>
+        <v>878</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>915</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>904</v>
+        <v>896</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>903</v>
+        <v>895</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="86.4">
       <c r="A8" t="s">
-        <v>886</v>
+        <v>879</v>
       </c>
       <c r="B8" t="s">
-        <v>892</v>
+        <v>884</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>905</v>
+        <v>897</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>906</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="72">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="144">
       <c r="A9" s="58" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>919</v>
+        <v>909</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>920</v>
+        <v>910</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="100.8">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="115.2">
       <c r="A10" t="s">
-        <v>882</v>
+        <v>875</v>
       </c>
       <c r="B10" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>910</v>
+        <v>1008</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>911</v>
+        <v>902</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -7103,10 +7710,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -7114,7 +7721,7 @@
         <v>384</v>
       </c>
       <c r="B12" t="s">
-        <v>909</v>
+        <v>901</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>260</v>
@@ -7122,38 +7729,53 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>887</v>
+        <v>880</v>
       </c>
       <c r="B13" t="s">
-        <v>881</v>
+        <v>874</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>913</v>
+        <v>904</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>911</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="158.4">
       <c r="A14" t="s">
         <v>438</v>
       </c>
-      <c r="B14" t="s">
-        <v>863</v>
+      <c r="B14" s="5" t="s">
+        <v>1006</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>911</v>
+        <v>1003</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="115.2">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="201.6">
       <c r="A18" t="s">
-        <v>923</v>
+        <v>912</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>925</v>
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="28.8">
+      <c r="B19" s="5" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="B20" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="B21" t="s">
+        <v>1023</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -7161,32 +7783,32 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="14" t="s">
-        <v>917</v>
+        <v>907</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>866</v>
+        <v>859</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>865</v>
+        <v>858</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>916</v>
+        <v>906</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="14" t="s">
-        <v>918</v>
+        <v>908</v>
       </c>
     </row>
   </sheetData>
@@ -7195,6 +7817,659 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6DB26E2-2FEB-428C-8A2B-44341C3C4297}">
+  <dimension ref="B1:P37"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="16.44140625" customWidth="1"/>
+    <col min="3" max="3" width="24.33203125" customWidth="1"/>
+    <col min="4" max="4" width="34.5546875" customWidth="1"/>
+    <col min="5" max="5" width="38.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:16">
+      <c r="B1" s="62" t="s">
+        <v>916</v>
+      </c>
+      <c r="C1" s="62" t="s">
+        <v>917</v>
+      </c>
+      <c r="D1" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" s="62" t="s">
+        <v>213</v>
+      </c>
+      <c r="G1" s="62" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="2" spans="2:16" ht="28.8">
+      <c r="B2" s="63" t="s">
+        <v>918</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>919</v>
+      </c>
+      <c r="D2" s="63" t="s">
+        <v>920</v>
+      </c>
+      <c r="E2" s="63">
+        <v>4</v>
+      </c>
+      <c r="G2" s="65" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="3" spans="2:16" ht="28.8">
+      <c r="B3" s="63" t="s">
+        <v>921</v>
+      </c>
+      <c r="C3" s="63" t="s">
+        <v>922</v>
+      </c>
+      <c r="D3" s="63" t="s">
+        <v>923</v>
+      </c>
+      <c r="E3" s="63" t="s">
+        <v>924</v>
+      </c>
+      <c r="G3" s="63" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" ht="28.8">
+      <c r="B4" s="63" t="s">
+        <v>925</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>926</v>
+      </c>
+      <c r="D4" s="63" t="s">
+        <v>927</v>
+      </c>
+      <c r="E4" s="63" t="s">
+        <v>928</v>
+      </c>
+      <c r="G4" s="63" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" ht="28.8">
+      <c r="B5" s="63" t="s">
+        <v>929</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>930</v>
+      </c>
+      <c r="D5" s="63" t="s">
+        <v>931</v>
+      </c>
+      <c r="E5" s="63" t="s">
+        <v>928</v>
+      </c>
+      <c r="G5" s="63" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="57.6">
+      <c r="B6" s="63" t="s">
+        <v>932</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>933</v>
+      </c>
+      <c r="D6" s="63" t="s">
+        <v>934</v>
+      </c>
+      <c r="E6" s="63" t="s">
+        <v>935</v>
+      </c>
+      <c r="G6" s="63" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" ht="28.8">
+      <c r="B7" s="63" t="s">
+        <v>936</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>937</v>
+      </c>
+      <c r="D7" s="63" t="s">
+        <v>938</v>
+      </c>
+      <c r="E7" s="63" t="s">
+        <v>939</v>
+      </c>
+      <c r="G7" s="63" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" ht="43.2">
+      <c r="B8" s="63" t="s">
+        <v>940</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>941</v>
+      </c>
+      <c r="D8" s="63" t="s">
+        <v>942</v>
+      </c>
+      <c r="E8" s="63" t="s">
+        <v>943</v>
+      </c>
+      <c r="G8" s="63" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="43.2">
+      <c r="B9" s="63" t="s">
+        <v>944</v>
+      </c>
+      <c r="C9" s="63" t="s">
+        <v>945</v>
+      </c>
+      <c r="D9" s="63" t="s">
+        <v>946</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>947</v>
+      </c>
+      <c r="G9" s="63" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="43.2">
+      <c r="B10" s="63" t="s">
+        <v>948</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>949</v>
+      </c>
+      <c r="D10" s="63" t="s">
+        <v>950</v>
+      </c>
+      <c r="E10" s="63" t="s">
+        <v>951</v>
+      </c>
+      <c r="G10" s="63" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" ht="28.8">
+      <c r="B11" s="63" t="s">
+        <v>952</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>953</v>
+      </c>
+      <c r="D11" s="63" t="s">
+        <v>954</v>
+      </c>
+      <c r="E11" s="63" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" ht="28.8">
+      <c r="B12" s="63" t="s">
+        <v>955</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>956</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>957</v>
+      </c>
+      <c r="E12" s="63" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16">
+      <c r="F14" t="s">
+        <v>965</v>
+      </c>
+      <c r="G14" t="s">
+        <v>987</v>
+      </c>
+      <c r="H14" t="s">
+        <v>823</v>
+      </c>
+      <c r="I14" t="s">
+        <v>989</v>
+      </c>
+      <c r="J14" t="s">
+        <v>822</v>
+      </c>
+      <c r="K14" t="s">
+        <v>990</v>
+      </c>
+      <c r="L14" t="s">
+        <v>991</v>
+      </c>
+      <c r="M14" t="s">
+        <v>824</v>
+      </c>
+      <c r="N14" t="s">
+        <v>828</v>
+      </c>
+      <c r="P14" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16">
+      <c r="B15" s="64" t="s">
+        <v>964</v>
+      </c>
+      <c r="D15">
+        <v>80</v>
+      </c>
+      <c r="E15" s="63" t="s">
+        <v>974</v>
+      </c>
+      <c r="F15" s="14">
+        <v>78</v>
+      </c>
+      <c r="G15" s="14">
+        <v>94</v>
+      </c>
+      <c r="H15" s="14">
+        <v>91</v>
+      </c>
+      <c r="I15" s="14">
+        <v>84</v>
+      </c>
+      <c r="J15" s="14">
+        <v>86</v>
+      </c>
+      <c r="K15" s="14">
+        <v>79</v>
+      </c>
+      <c r="L15" s="14">
+        <v>66</v>
+      </c>
+      <c r="M15" s="14">
+        <v>80</v>
+      </c>
+      <c r="N15" s="14">
+        <v>74</v>
+      </c>
+      <c r="O15">
+        <v>100</v>
+      </c>
+      <c r="P15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16">
+      <c r="C16" t="s">
+        <v>959</v>
+      </c>
+      <c r="E16" s="63" t="s">
+        <v>975</v>
+      </c>
+      <c r="F16">
+        <v>92</v>
+      </c>
+      <c r="G16">
+        <v>86</v>
+      </c>
+      <c r="H16">
+        <v>68</v>
+      </c>
+      <c r="I16">
+        <v>90</v>
+      </c>
+      <c r="J16">
+        <v>94</v>
+      </c>
+      <c r="K16">
+        <v>82</v>
+      </c>
+      <c r="L16">
+        <v>74</v>
+      </c>
+      <c r="M16">
+        <v>96</v>
+      </c>
+      <c r="N16">
+        <v>78</v>
+      </c>
+      <c r="O16">
+        <v>100</v>
+      </c>
+      <c r="P16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="3:16">
+      <c r="C17" t="s">
+        <v>960</v>
+      </c>
+      <c r="D17">
+        <v>84</v>
+      </c>
+      <c r="E17" s="63" t="s">
+        <v>988</v>
+      </c>
+      <c r="F17" s="14">
+        <v>84</v>
+      </c>
+      <c r="G17" s="14">
+        <v>95</v>
+      </c>
+      <c r="H17" s="14">
+        <v>94</v>
+      </c>
+      <c r="I17" s="14">
+        <v>82</v>
+      </c>
+      <c r="J17" s="14">
+        <v>82</v>
+      </c>
+      <c r="K17" s="14">
+        <v>58</v>
+      </c>
+      <c r="L17" s="14">
+        <v>72</v>
+      </c>
+      <c r="M17" s="14">
+        <v>84</v>
+      </c>
+      <c r="N17" s="14">
+        <v>76</v>
+      </c>
+      <c r="O17">
+        <v>100</v>
+      </c>
+      <c r="P17">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="3:16">
+      <c r="C18" t="s">
+        <v>961</v>
+      </c>
+      <c r="E18" s="63" t="s">
+        <v>976</v>
+      </c>
+      <c r="F18">
+        <v>52</v>
+      </c>
+      <c r="G18">
+        <v>93</v>
+      </c>
+      <c r="H18">
+        <v>88</v>
+      </c>
+      <c r="I18">
+        <v>68</v>
+      </c>
+      <c r="J18">
+        <v>58</v>
+      </c>
+      <c r="K18">
+        <v>48</v>
+      </c>
+      <c r="L18">
+        <v>42</v>
+      </c>
+      <c r="M18">
+        <v>46</v>
+      </c>
+      <c r="N18">
+        <v>52</v>
+      </c>
+      <c r="O18">
+        <v>100</v>
+      </c>
+      <c r="P18">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="3:16">
+      <c r="C19" t="s">
+        <v>962</v>
+      </c>
+      <c r="E19" s="63" t="s">
+        <v>977</v>
+      </c>
+      <c r="F19">
+        <v>88</v>
+      </c>
+      <c r="G19">
+        <v>78</v>
+      </c>
+      <c r="H19">
+        <v>74</v>
+      </c>
+      <c r="I19">
+        <v>92</v>
+      </c>
+      <c r="J19">
+        <v>95</v>
+      </c>
+      <c r="K19">
+        <v>93</v>
+      </c>
+      <c r="L19">
+        <v>88</v>
+      </c>
+      <c r="M19">
+        <v>97</v>
+      </c>
+      <c r="N19">
+        <v>88</v>
+      </c>
+      <c r="O19">
+        <v>100</v>
+      </c>
+      <c r="P19">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="3:16">
+      <c r="C20" t="s">
+        <v>963</v>
+      </c>
+      <c r="D20">
+        <v>72</v>
+      </c>
+      <c r="E20" s="63" t="s">
+        <v>978</v>
+      </c>
+      <c r="F20" s="14">
+        <v>58</v>
+      </c>
+      <c r="G20" s="14">
+        <v>90</v>
+      </c>
+      <c r="H20" s="14">
+        <v>89</v>
+      </c>
+      <c r="I20" s="14">
+        <v>83</v>
+      </c>
+      <c r="J20" s="14">
+        <v>76</v>
+      </c>
+      <c r="K20" s="14">
+        <v>84</v>
+      </c>
+      <c r="L20" s="14">
+        <v>58</v>
+      </c>
+      <c r="M20" s="14">
+        <v>72</v>
+      </c>
+      <c r="N20" s="14">
+        <v>62</v>
+      </c>
+      <c r="O20">
+        <v>100</v>
+      </c>
+      <c r="P20">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="3:16">
+      <c r="E21" s="63" t="s">
+        <v>979</v>
+      </c>
+      <c r="F21">
+        <v>64</v>
+      </c>
+      <c r="G21">
+        <v>96</v>
+      </c>
+      <c r="H21">
+        <v>90</v>
+      </c>
+      <c r="I21">
+        <v>72</v>
+      </c>
+      <c r="J21">
+        <v>66</v>
+      </c>
+      <c r="K21">
+        <v>74</v>
+      </c>
+      <c r="L21">
+        <v>54</v>
+      </c>
+      <c r="M21">
+        <v>58</v>
+      </c>
+      <c r="N21">
+        <v>68</v>
+      </c>
+      <c r="O21">
+        <v>100</v>
+      </c>
+      <c r="P21">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="3:16">
+      <c r="E22" s="63" t="s">
+        <v>948</v>
+      </c>
+      <c r="F22">
+        <v>38</v>
+      </c>
+      <c r="G22">
+        <v>42</v>
+      </c>
+      <c r="H22">
+        <v>58</v>
+      </c>
+      <c r="I22">
+        <v>72</v>
+      </c>
+      <c r="J22">
+        <v>48</v>
+      </c>
+      <c r="K22">
+        <v>22</v>
+      </c>
+      <c r="L22">
+        <v>36</v>
+      </c>
+      <c r="M22">
+        <v>42</v>
+      </c>
+      <c r="N22">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="3:16">
+      <c r="E24" t="s">
+        <v>980</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="25" spans="3:16">
+      <c r="E25" t="s">
+        <v>981</v>
+      </c>
+      <c r="N25" t="s">
+        <v>993</v>
+      </c>
+      <c r="O25" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="26" spans="3:16">
+      <c r="E26" t="s">
+        <v>982</v>
+      </c>
+      <c r="N26" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="27" spans="3:16">
+      <c r="E27" t="s">
+        <v>983</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1005</v>
+      </c>
+      <c r="N27" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="28" spans="3:16">
+      <c r="E28" t="s">
+        <v>984</v>
+      </c>
+      <c r="N28" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="29" spans="3:16">
+      <c r="E29" t="s">
+        <v>985</v>
+      </c>
+      <c r="N29" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="30" spans="3:16">
+      <c r="E30" t="s">
+        <v>986</v>
+      </c>
+      <c r="N30" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1C79E50-A761-4208-AC1F-7EE61CFDD025}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7715,9 +8990,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.21875" customWidth="1"/>
@@ -7753,7 +9028,7 @@
         <v>413</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="C4" s="39" t="s">
         <v>6</v>
@@ -7765,7 +9040,7 @@
         <v>59</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>3</v>
@@ -7794,13 +9069,13 @@
     </row>
     <row r="5" spans="1:14" ht="28.8">
       <c r="A5" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C5" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>761</v>
@@ -7815,10 +9090,10 @@
     </row>
     <row r="6" spans="1:14" ht="28.8">
       <c r="A6" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C6" t="s">
         <v>753</v>
@@ -7836,10 +9111,10 @@
     </row>
     <row r="7" spans="1:14" ht="28.8">
       <c r="A7" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C7" t="s">
         <v>754</v>
@@ -7857,13 +9132,13 @@
     </row>
     <row r="8" spans="1:14" ht="28.8">
       <c r="A8" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C8" t="s">
-        <v>807</v>
+        <v>801</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>755</v>
@@ -7876,13 +9151,13 @@
     </row>
     <row r="9" spans="1:14" ht="28.8">
       <c r="A9" s="2" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>808</v>
+        <v>802</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>639</v>
@@ -7924,13 +9199,13 @@
         <v>715</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>811</v>
+        <v>805</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>809</v>
+        <v>803</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -7943,7 +9218,7 @@
         <v>715</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>763</v>
@@ -7962,7 +9237,7 @@
         <v>715</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>762</v>
@@ -7971,7 +9246,7 @@
         <v>436</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>801</v>
+        <v>795</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -7981,16 +9256,16 @@
     </row>
     <row r="15" spans="1:14" ht="28.8">
       <c r="A15" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>768</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>665</v>
+        <v>1017</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -7998,18 +9273,18 @@
       <c r="H15" s="3"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:14" ht="27.6">
+    <row r="16" spans="1:14" ht="28.8">
       <c r="A16" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>768</v>
-      </c>
       <c r="C16" s="2" t="s">
-        <v>771</v>
+        <v>1013</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>704</v>
+        <v>1014</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -8019,16 +9294,16 @@
     </row>
     <row r="17" spans="1:11" ht="27.6">
       <c r="A17" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>768</v>
-      </c>
       <c r="C17" t="s">
-        <v>764</v>
+        <v>1015</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>765</v>
+        <v>1016</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -8038,16 +9313,16 @@
     </row>
     <row r="18" spans="1:11" ht="27.6">
       <c r="A18" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>768</v>
-      </c>
       <c r="C18" t="s">
-        <v>666</v>
+        <v>1018</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>707</v>
+        <v>1019</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -8055,37 +9330,37 @@
       <c r="H18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="27.6">
+    <row r="19" spans="1:11">
       <c r="A19" s="2" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="C19" t="s">
-        <v>671</v>
+        <v>784</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>778</v>
+        <v>702</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="2"/>
-      <c r="J19" s="2"/>
+      <c r="H19" s="3"/>
+      <c r="K19" s="34"/>
     </row>
     <row r="20" spans="1:11" ht="27.6">
       <c r="A20" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>768</v>
-      </c>
       <c r="C20" t="s">
-        <v>788</v>
+        <v>1012</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>701</v>
+        <v>22</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -8093,78 +9368,82 @@
       <c r="H20" s="3"/>
       <c r="K20" s="34"/>
     </row>
-    <row r="21" spans="1:11" ht="27.6">
+    <row r="21" spans="1:11">
       <c r="A21" s="2" t="s">
-        <v>766</v>
+        <v>693</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="C21" t="s">
-        <v>789</v>
+        <v>769</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>696</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="K21" s="34"/>
-    </row>
-    <row r="22" spans="1:11" ht="27.6">
+      <c r="H21" s="2"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" ht="28.8">
       <c r="A22" s="2" t="s">
-        <v>766</v>
+        <v>693</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="C22" t="s">
-        <v>790</v>
+        <v>769</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>717</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>22</v>
+        <v>643</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="K22" s="34"/>
+      <c r="H22" s="2"/>
+      <c r="J22" s="2"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="2" t="s">
         <v>693</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>696</v>
+        <v>769</v>
+      </c>
+      <c r="C23" t="s">
+        <v>716</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>697</v>
+        <v>644</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G23" s="3"/>
       <c r="H23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="28.8">
+    <row r="24" spans="1:11">
       <c r="A24" s="2" t="s">
         <v>693</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>717</v>
+        <v>769</v>
+      </c>
+      <c r="C24" t="s">
+        <v>718</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>643</v>
+        <v>719</v>
       </c>
       <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="F24" s="3" t="s">
+        <v>426</v>
+      </c>
       <c r="G24" s="3"/>
       <c r="H24" s="2"/>
       <c r="J24" s="2"/>
@@ -8174,38 +9453,38 @@
         <v>693</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="C25" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>644</v>
+        <v>721</v>
       </c>
       <c r="E25" s="3"/>
-      <c r="F25" s="3" t="s">
-        <v>426</v>
-      </c>
+      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="2"/>
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C26" t="s">
-        <v>718</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>719</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3" t="s">
-        <v>426</v>
+        <v>770</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>723</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="E26" s="56" t="s">
+        <v>731</v>
+      </c>
+      <c r="F26" s="56" t="s">
+        <v>425</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="2"/>
@@ -8213,233 +9492,227 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="2" t="s">
-        <v>693</v>
+        <v>771</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C27" t="s">
-        <v>720</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>721</v>
-      </c>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
+        <v>770</v>
+      </c>
+      <c r="C27" s="56" t="s">
+        <v>725</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="E27" s="56" t="s">
+        <v>730</v>
+      </c>
+      <c r="F27" s="56"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="2"/>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>723</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>724</v>
+        <v>727</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>728</v>
       </c>
       <c r="E28" s="56" t="s">
-        <v>731</v>
-      </c>
-      <c r="F28" s="56" t="s">
-        <v>425</v>
-      </c>
+        <v>729</v>
+      </c>
+      <c r="F28" s="56"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="2"/>
-      <c r="J28" s="2"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C29" s="56" t="s">
-        <v>725</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>726</v>
+        <v>732</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>734</v>
       </c>
       <c r="E29" s="56" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="F29" s="56"/>
       <c r="G29" s="3"/>
-      <c r="J29" s="2"/>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="E30" s="56" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
       <c r="F30" s="56"/>
       <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C31" s="56" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>734</v>
+        <v>750</v>
       </c>
       <c r="E31" s="56" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F31" s="56"/>
       <c r="G31" s="3"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>733</v>
+        <v>544</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>735</v>
+        <v>543</v>
       </c>
       <c r="E32" s="56" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="F32" s="56"/>
       <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="J32" s="2"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C33" s="56" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>750</v>
+        <v>742</v>
       </c>
       <c r="E33" s="56" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F33" s="56"/>
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>544</v>
+        <v>744</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>543</v>
+        <v>745</v>
       </c>
       <c r="E34" s="56" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="F34" s="56"/>
       <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="J34" s="2"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="E35" s="56" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="F35" s="56"/>
       <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C36" s="56" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>745</v>
-      </c>
-      <c r="E36" s="56" t="s">
-        <v>748</v>
-      </c>
-      <c r="F36" s="56"/>
+        <v>752</v>
+      </c>
       <c r="G36" s="3"/>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:11" ht="28.8">
       <c r="A37" s="2" t="s">
-        <v>774</v>
+        <v>426</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>773</v>
-      </c>
-      <c r="C37" s="56" t="s">
-        <v>746</v>
+        <v>772</v>
+      </c>
+      <c r="C37" s="49" t="s">
+        <v>432</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>747</v>
-      </c>
-      <c r="E37" s="56" t="s">
-        <v>749</v>
-      </c>
-      <c r="F37" s="56"/>
+        <v>414</v>
+      </c>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
       <c r="G37" s="3"/>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:11" ht="220.8">
       <c r="A38" s="2" t="s">
-        <v>774</v>
+        <v>426</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>773</v>
-      </c>
-      <c r="C38" s="56" t="s">
-        <v>751</v>
+        <v>772</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>752</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:11" ht="28.8">
@@ -8447,610 +9720,574 @@
         <v>426</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>775</v>
-      </c>
-      <c r="C39" s="49" t="s">
-        <v>432</v>
+        <v>772</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>563</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="E39" s="3"/>
+        <v>57</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>564</v>
+      </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-    </row>
-    <row r="40" spans="1:11" ht="220.8">
+      <c r="H39" s="3"/>
+      <c r="J39" s="2"/>
+    </row>
+    <row r="40" spans="1:11" ht="28.8">
       <c r="A40" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>804</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="E40" s="3"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:11" ht="28.8">
       <c r="A41" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>563</v>
+        <v>38</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>564</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="E41" s="3"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
-      <c r="J41" s="2"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="3"/>
     </row>
     <row r="42" spans="1:11" ht="28.8">
       <c r="A42" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>775</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>36</v>
+        <v>772</v>
+      </c>
+      <c r="C42" t="s">
+        <v>664</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>37</v>
+        <v>705</v>
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
-    </row>
-    <row r="43" spans="1:11" ht="28.8">
-      <c r="A43" s="2" t="s">
+      <c r="K42" s="34"/>
+    </row>
+    <row r="43" spans="1:11" ht="179.4">
+      <c r="A43" s="40" t="s">
         <v>426</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>775</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E43" s="3"/>
+      <c r="B43" s="37" t="s">
+        <v>772</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>796</v>
+      </c>
+      <c r="D43" s="37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" s="37" t="s">
+        <v>797</v>
+      </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
-      <c r="J43" s="19"/>
-      <c r="K43" s="3"/>
-    </row>
-    <row r="44" spans="1:11" ht="28.8">
+      <c r="K43" s="34"/>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>775</v>
       </c>
-      <c r="C44" t="s">
-        <v>664</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>705</v>
-      </c>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
+      <c r="C44" s="49" t="s">
+        <v>431</v>
+      </c>
+      <c r="D44" s="48" t="s">
+        <v>545</v>
+      </c>
+      <c r="E44" s="17"/>
       <c r="H44" s="3"/>
-      <c r="K44" s="34"/>
-    </row>
-    <row r="45" spans="1:11" ht="179.4">
-      <c r="A45" s="40" t="s">
-        <v>426</v>
-      </c>
-      <c r="B45" s="37" t="s">
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>775</v>
       </c>
-      <c r="C45" s="38" t="s">
-        <v>802</v>
-      </c>
-      <c r="D45" s="37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E45" s="37" t="s">
-        <v>803</v>
-      </c>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="K45" s="34"/>
+      <c r="C45" s="49" t="s">
+        <v>550</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>551</v>
+      </c>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C46" s="49" t="s">
-        <v>431</v>
-      </c>
-      <c r="D46" s="48" t="s">
-        <v>545</v>
-      </c>
-      <c r="E46" s="17"/>
-      <c r="H46" s="3"/>
+        <v>775</v>
+      </c>
+      <c r="C46" t="s">
+        <v>557</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="47" spans="1:11">
       <c r="A47" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C47" s="49" t="s">
-        <v>550</v>
+        <v>775</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11">
+        <v>350</v>
+      </c>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+    </row>
+    <row r="48" spans="1:11" ht="28.8">
       <c r="A48" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C48" t="s">
-        <v>557</v>
+        <v>775</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>559</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11">
+        <v>558</v>
+      </c>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:10">
       <c r="A49" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>44</v>
+        <v>775</v>
+      </c>
+      <c r="C49" s="49" t="s">
+        <v>42</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>350</v>
+        <v>43</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
-    </row>
-    <row r="50" spans="1:11" ht="28.8">
+      <c r="J49" s="2"/>
+    </row>
+    <row r="50" spans="1:10">
       <c r="A50" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>559</v>
+        <v>31</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>558</v>
+        <v>32</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
-    </row>
-    <row r="51" spans="1:11">
+      <c r="J50" s="2"/>
+    </row>
+    <row r="51" spans="1:10">
       <c r="A51" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C51" s="49" t="s">
-        <v>42</v>
+        <v>775</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>776</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>43</v>
+        <v>567</v>
       </c>
       <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
+      <c r="F51" s="17"/>
       <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
-      <c r="J51" s="2"/>
-    </row>
-    <row r="52" spans="1:11">
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" spans="1:10">
       <c r="A52" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>31</v>
+        <v>777</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
-      <c r="J52" s="2"/>
-    </row>
-    <row r="53" spans="1:11">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
       <c r="A53" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>780</v>
+        <v>775</v>
+      </c>
+      <c r="C53" s="49" t="s">
+        <v>774</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>567</v>
-      </c>
-      <c r="E53" s="3"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="2"/>
-    </row>
-    <row r="54" spans="1:11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
       <c r="A54" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>781</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11">
+        <v>16</v>
+      </c>
+      <c r="D54" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
       <c r="A55" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C55" s="49" t="s">
-        <v>777</v>
+        <v>775</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
       <c r="A56" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D56" t="s">
-        <v>782</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11">
+        <v>775</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="17" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="69">
       <c r="A57" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>775</v>
+      </c>
+      <c r="C57" s="38"/>
       <c r="D57" s="3" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11">
+        <v>383</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="69">
       <c r="A58" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="17" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" ht="69">
+        <v>775</v>
+      </c>
+      <c r="C58" s="38"/>
+      <c r="D58" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="27.6">
       <c r="A59" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="C59" s="38"/>
       <c r="D59" s="3" t="s">
-        <v>383</v>
+        <v>334</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="69">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="82.8">
       <c r="A60" s="2" t="s">
         <v>425</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C60" s="38"/>
-      <c r="D60" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="27.6">
+        <v>775</v>
+      </c>
+      <c r="D60" s="33" t="s">
+        <v>387</v>
+      </c>
+      <c r="E60" s="33" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
       <c r="A61" s="2" t="s">
-        <v>425</v>
+        <v>867</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="C61" s="38"/>
-      <c r="D61" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="82.8">
+        <v>860</v>
+      </c>
+      <c r="C61" t="s">
+        <v>861</v>
+      </c>
+      <c r="D61" s="38" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
       <c r="A62" s="2" t="s">
-        <v>425</v>
+        <v>867</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="D62" s="33" t="s">
-        <v>387</v>
-      </c>
-      <c r="E62" s="33" t="s">
-        <v>787</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11">
+        <v>860</v>
+      </c>
+      <c r="C62" t="s">
+        <v>862</v>
+      </c>
+      <c r="D62" s="38" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
       <c r="A63" s="2" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="B63" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="C63" t="s">
+        <v>863</v>
+      </c>
+      <c r="D63" s="38" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" s="2" t="s">
         <v>867</v>
       </c>
-      <c r="C63" t="s">
-        <v>868</v>
-      </c>
-      <c r="D63" s="38" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11">
-      <c r="A64" s="2" t="s">
-        <v>874</v>
-      </c>
       <c r="B64" s="3" t="s">
-        <v>867</v>
+        <v>860</v>
       </c>
       <c r="C64" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="D64" s="38" t="s">
-        <v>880</v>
+        <v>872</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="2" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>867</v>
+        <v>860</v>
       </c>
       <c r="C65" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="D65" s="38" t="s">
-        <v>878</v>
+        <v>869</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="2" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>867</v>
+        <v>860</v>
       </c>
       <c r="C66" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="D66" s="38" t="s">
-        <v>879</v>
+        <v>870</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="2" t="s">
-        <v>874</v>
+        <v>430</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>867</v>
-      </c>
-      <c r="C67" t="s">
-        <v>872</v>
-      </c>
-      <c r="D67" s="38" t="s">
-        <v>876</v>
+        <v>786</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="2" t="s">
-        <v>874</v>
+        <v>430</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>867</v>
+        <v>786</v>
       </c>
       <c r="C68" t="s">
-        <v>873</v>
-      </c>
-      <c r="D68" s="38" t="s">
-        <v>877</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5">
+        <v>787</v>
+      </c>
+      <c r="D68" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="28.8">
       <c r="A69" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>46</v>
+        <v>560</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="28.8">
       <c r="A70" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C70" t="s">
-        <v>793</v>
-      </c>
-      <c r="D70" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="28.8">
+        <v>786</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="82.8">
       <c r="A71" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>560</v>
+        <v>788</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="28.8">
+        <v>56</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="69">
       <c r="A72" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>48</v>
+        <v>789</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E72" s="5" t="s">
-        <v>783</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="82.8">
+        <v>114</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="55.2">
       <c r="A73" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B73" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E73" s="3" t="s">
         <v>792</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E73" s="3" t="s">
-        <v>796</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="69">
+    </row>
+    <row r="74" spans="1:5" ht="409.6">
       <c r="A74" s="2" t="s">
         <v>430</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>114</v>
+        <v>699</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>797</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="55.2">
-      <c r="A75" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>799</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="E75" s="3" t="s">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" ht="409.6">
-      <c r="A76" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>792</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>800</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>699</v>
-      </c>
-      <c r="E76" s="3" t="s">
         <v>700</v>
       </c>
     </row>
@@ -9059,7 +10296,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
   <dimension ref="A1:N136"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9902,7 +11139,7 @@
         <v>429</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>35</v>
@@ -11153,7 +12390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -11431,301 +12668,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
-  <dimension ref="A1:J51"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="8.88671875" style="5"/>
-    <col min="2" max="2" width="16.88671875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="13" style="5" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="25.109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="44.44140625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="14" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="E3" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="27.6">
-      <c r="A4" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="28.8">
-      <c r="C5" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="E8" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="41.4">
-      <c r="A9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="J9"/>
-    </row>
-    <row r="10" spans="1:10" ht="43.2">
-      <c r="C10" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="J10" s="17"/>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12"/>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
-      <c r="H12"/>
-      <c r="I12"/>
-      <c r="J12"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.6">
-      <c r="A13" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="18"/>
-      <c r="F13"/>
-      <c r="G13"/>
-      <c r="H13"/>
-      <c r="I13"/>
-      <c r="J13"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="J14"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="J15"/>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="B16"/>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-      <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16"/>
-      <c r="I16"/>
-      <c r="J16"/>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="4"/>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="19"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="B28"/>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="B29"/>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="B30"/>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="B31"/>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="B32"/>
-    </row>
-    <row r="33" spans="2:9">
-      <c r="B33"/>
-    </row>
-    <row r="35" spans="2:9">
-      <c r="B35" s="14"/>
-    </row>
-    <row r="37" spans="2:9">
-      <c r="B37"/>
-      <c r="I37"/>
-    </row>
-    <row r="38" spans="2:9">
-      <c r="I38"/>
-    </row>
-    <row r="39" spans="2:9">
-      <c r="I39"/>
-    </row>
-    <row r="41" spans="2:9">
-      <c r="I41"/>
-    </row>
-    <row r="49" spans="2:2">
-      <c r="B49"/>
-    </row>
-    <row r="51" spans="2:2">
-      <c r="B51"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
after partial improvment of new chat
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECB2BEB-B87D-427A-B99B-B58A9271D2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB393DB-9CF3-4554-9EFF-6E5F9F41CC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -3209,9 +3209,6 @@
     <t>אינטואיציה</t>
   </si>
   <si>
-    <t>לחשוב איך מכניסים לסוגי התאמה ולחשוב איך להשתמש בטקסט הכללי</t>
-  </si>
-  <si>
     <t>עמדות</t>
   </si>
   <si>
@@ -3237,9 +3234,6 @@
   </si>
   <si>
     <t>חישוב התאמה</t>
-  </si>
-  <si>
-    <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך</t>
   </si>
   <si>
     <r>
@@ -3755,6 +3749,14 @@
   </si>
   <si>
     <t xml:space="preserve">בחישוב לפי פרופילים שיחקתי קצת עם המשקלים, בגדול כדי להתאים יותר לנוי ורון אז צריך לראות שזה באמת אמין. </t>
+  </si>
+  <si>
+    <t>לחשוב איך מכניסים לסוגי התאמה ולחשוב איך להשתמש בטקסט הכללי (דיל ברייקרס ויתרונות אפשריים)</t>
+  </si>
+  <si>
+    <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
+פרופיל סופר קריטי. להוציא מפה כל מה שקשור לעמדות. להכניס סגנונות אפשריים - צריך לבנות את זה חכם. אולי בתגיות חופשיות (או לא חופשיות). לחשוב על זה. לצורך הבדיקה של זה אצטרך משתמשים מסגנונות שונים באמת, כרגע האוכלוסייה במערכת שלי די הומוגנית.  צריך אולי גם להיות גורם מפלטר לסגנונות לא קשורים.
+סגנונות אפשריים (לחשוב איך לעשות את זה פוליטיקלי קורקט): ערסים, נורמטיבי, עממי, סחי, קיבוצניק/מושבניק, היפי, סובייטי, גיק, תרבות גבוהה, אליטיסטי, קפליניסט. לחשוב מה עוד ואיך לנסח.</t>
   </si>
 </sst>
 </file>
@@ -7272,7 +7274,7 @@
   <sheetData>
     <row r="2" spans="2:20">
       <c r="B2" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="R2" t="s">
         <v>829</v>
@@ -7293,7 +7295,7 @@
     </row>
     <row r="5" spans="2:20">
       <c r="B5" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="R5" t="s">
         <v>836</v>
@@ -7566,16 +7568,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="14" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>880</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>881</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>882</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>883</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="187.2">
@@ -7583,27 +7585,27 @@
         <v>415</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="86.4">
       <c r="A3" s="5" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B3" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="D3" s="61" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="G3" s="14"/>
     </row>
@@ -7612,13 +7614,13 @@
         <v>426</v>
       </c>
       <c r="B4" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8">
@@ -7626,13 +7628,13 @@
         <v>693</v>
       </c>
       <c r="B5" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="C5" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.8">
@@ -7640,41 +7642,41 @@
         <v>429</v>
       </c>
       <c r="B6" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="D6" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2">
       <c r="A7" t="s">
+        <v>877</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>894</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="115.2">
+      <c r="A8" t="s">
         <v>878</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>915</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B8" s="5" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>895</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>896</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>895</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="86.4">
-      <c r="A8" t="s">
-        <v>879</v>
-      </c>
-      <c r="B8" t="s">
-        <v>884</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>897</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>898</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="144">
@@ -7682,27 +7684,27 @@
         <v>867</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="115.2">
       <c r="A10" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B10" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -7710,10 +7712,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>899</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>901</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>903</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -7721,7 +7723,7 @@
         <v>384</v>
       </c>
       <c r="B12" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>260</v>
@@ -7729,16 +7731,16 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B13" t="s">
-        <v>874</v>
+        <v>1022</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="158.4">
@@ -7746,36 +7748,36 @@
         <v>438</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="201.6">
       <c r="A18" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="28.8">
       <c r="B19" s="5" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="B20" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="B21" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -7783,7 +7785,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="14" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -7798,17 +7800,17 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="14" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
     </row>
   </sheetData>
@@ -7829,10 +7831,10 @@
   <sheetData>
     <row r="1" spans="2:16">
       <c r="B1" s="62" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="C1" s="62" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>151</v>
@@ -7841,211 +7843,211 @@
         <v>213</v>
       </c>
       <c r="G1" s="62" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
     </row>
     <row r="2" spans="2:16" ht="28.8">
       <c r="B2" s="63" t="s">
+        <v>916</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>917</v>
+      </c>
+      <c r="D2" s="63" t="s">
         <v>918</v>
-      </c>
-      <c r="C2" s="63" t="s">
-        <v>919</v>
-      </c>
-      <c r="D2" s="63" t="s">
-        <v>920</v>
       </c>
       <c r="E2" s="63">
         <v>4</v>
       </c>
       <c r="G2" s="65" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
     <row r="3" spans="2:16" ht="28.8">
       <c r="B3" s="63" t="s">
+        <v>919</v>
+      </c>
+      <c r="C3" s="63" t="s">
+        <v>920</v>
+      </c>
+      <c r="D3" s="63" t="s">
         <v>921</v>
       </c>
-      <c r="C3" s="63" t="s">
+      <c r="E3" s="63" t="s">
         <v>922</v>
       </c>
-      <c r="D3" s="63" t="s">
-        <v>923</v>
-      </c>
-      <c r="E3" s="63" t="s">
-        <v>924</v>
-      </c>
       <c r="G3" s="63" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
     </row>
     <row r="4" spans="2:16" ht="28.8">
       <c r="B4" s="63" t="s">
+        <v>923</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>924</v>
+      </c>
+      <c r="D4" s="63" t="s">
         <v>925</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="E4" s="63" t="s">
         <v>926</v>
       </c>
-      <c r="D4" s="63" t="s">
-        <v>927</v>
-      </c>
-      <c r="E4" s="63" t="s">
-        <v>928</v>
-      </c>
       <c r="G4" s="63" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="28.8">
       <c r="B5" s="63" t="s">
+        <v>927</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>928</v>
+      </c>
+      <c r="D5" s="63" t="s">
         <v>929</v>
       </c>
-      <c r="C5" s="63" t="s">
-        <v>930</v>
-      </c>
-      <c r="D5" s="63" t="s">
-        <v>931</v>
-      </c>
       <c r="E5" s="63" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="G5" s="63" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="57.6">
       <c r="B6" s="63" t="s">
+        <v>930</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>931</v>
+      </c>
+      <c r="D6" s="63" t="s">
         <v>932</v>
       </c>
-      <c r="C6" s="63" t="s">
+      <c r="E6" s="63" t="s">
         <v>933</v>
       </c>
-      <c r="D6" s="63" t="s">
-        <v>934</v>
-      </c>
-      <c r="E6" s="63" t="s">
-        <v>935</v>
-      </c>
       <c r="G6" s="63" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="28.8">
       <c r="B7" s="63" t="s">
+        <v>934</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>935</v>
+      </c>
+      <c r="D7" s="63" t="s">
         <v>936</v>
       </c>
-      <c r="C7" s="63" t="s">
+      <c r="E7" s="63" t="s">
         <v>937</v>
       </c>
-      <c r="D7" s="63" t="s">
-        <v>938</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>939</v>
-      </c>
       <c r="G7" s="63" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
     </row>
     <row r="8" spans="2:16" ht="43.2">
       <c r="B8" s="63" t="s">
+        <v>938</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>939</v>
+      </c>
+      <c r="D8" s="63" t="s">
         <v>940</v>
       </c>
-      <c r="C8" s="63" t="s">
+      <c r="E8" s="63" t="s">
         <v>941</v>
       </c>
-      <c r="D8" s="63" t="s">
-        <v>942</v>
-      </c>
-      <c r="E8" s="63" t="s">
-        <v>943</v>
-      </c>
       <c r="G8" s="63" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="43.2">
       <c r="B9" s="63" t="s">
+        <v>942</v>
+      </c>
+      <c r="C9" s="63" t="s">
+        <v>943</v>
+      </c>
+      <c r="D9" s="63" t="s">
         <v>944</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="E9" s="63" t="s">
         <v>945</v>
       </c>
-      <c r="D9" s="63" t="s">
-        <v>946</v>
-      </c>
-      <c r="E9" s="63" t="s">
-        <v>947</v>
-      </c>
       <c r="G9" s="63" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="43.2">
       <c r="B10" s="63" t="s">
+        <v>946</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>947</v>
+      </c>
+      <c r="D10" s="63" t="s">
         <v>948</v>
       </c>
-      <c r="C10" s="63" t="s">
+      <c r="E10" s="63" t="s">
         <v>949</v>
       </c>
-      <c r="D10" s="63" t="s">
-        <v>950</v>
-      </c>
-      <c r="E10" s="63" t="s">
-        <v>951</v>
-      </c>
       <c r="G10" s="63" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="28.8">
       <c r="B11" s="63" t="s">
+        <v>950</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>951</v>
+      </c>
+      <c r="D11" s="63" t="s">
         <v>952</v>
       </c>
-      <c r="C11" s="63" t="s">
-        <v>953</v>
-      </c>
-      <c r="D11" s="63" t="s">
-        <v>954</v>
-      </c>
       <c r="E11" s="63" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="28.8">
       <c r="B12" s="63" t="s">
+        <v>953</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>954</v>
+      </c>
+      <c r="D12" s="63" t="s">
         <v>955</v>
       </c>
-      <c r="C12" s="63" t="s">
+      <c r="E12" s="63" t="s">
         <v>956</v>
-      </c>
-      <c r="D12" s="63" t="s">
-        <v>957</v>
-      </c>
-      <c r="E12" s="63" t="s">
-        <v>958</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="F14" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="G14" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="H14" t="s">
         <v>823</v>
       </c>
       <c r="I14" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="J14" t="s">
         <v>822</v>
       </c>
       <c r="K14" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="L14" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="M14" t="s">
         <v>824</v>
@@ -8054,18 +8056,18 @@
         <v>828</v>
       </c>
       <c r="P14" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" s="64" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="D15">
         <v>80</v>
       </c>
       <c r="E15" s="63" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="F15" s="14">
         <v>78</v>
@@ -8103,10 +8105,10 @@
     </row>
     <row r="16" spans="2:16">
       <c r="C16" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="E16" s="63" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="F16">
         <v>92</v>
@@ -8144,13 +8146,13 @@
     </row>
     <row r="17" spans="3:16">
       <c r="C17" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="D17">
         <v>84</v>
       </c>
       <c r="E17" s="63" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="F17" s="14">
         <v>84</v>
@@ -8188,10 +8190,10 @@
     </row>
     <row r="18" spans="3:16">
       <c r="C18" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="E18" s="63" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="F18">
         <v>52</v>
@@ -8229,10 +8231,10 @@
     </row>
     <row r="19" spans="3:16">
       <c r="C19" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="E19" s="63" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="F19">
         <v>88</v>
@@ -8270,13 +8272,13 @@
     </row>
     <row r="20" spans="3:16">
       <c r="C20" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="D20">
         <v>72</v>
       </c>
       <c r="E20" s="63" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="F20" s="14">
         <v>58</v>
@@ -8314,7 +8316,7 @@
     </row>
     <row r="21" spans="3:16">
       <c r="E21" s="63" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="F21">
         <v>64</v>
@@ -8352,7 +8354,7 @@
     </row>
     <row r="22" spans="3:16">
       <c r="E22" s="63" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="F22">
         <v>38</v>
@@ -8384,79 +8386,79 @@
     </row>
     <row r="24" spans="3:16">
       <c r="E24" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="F24" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="25" spans="3:16">
       <c r="E25" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="N25" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="O25" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="26" spans="3:16">
       <c r="E26" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="N26" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
     </row>
     <row r="27" spans="3:16">
       <c r="E27" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="F27" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="N27" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="28" spans="3:16">
       <c r="E28" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="N28" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
     </row>
     <row r="29" spans="3:16">
       <c r="E29" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="N29" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
     </row>
     <row r="30" spans="3:16">
       <c r="E30" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="N30" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
     </row>
     <row r="35" spans="2:2">
       <c r="B35" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="36" spans="2:2">
       <c r="B36" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="37" spans="2:2">
@@ -9262,7 +9264,7 @@
         <v>766</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>765</v>
@@ -9281,10 +9283,10 @@
         <v>766</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -9300,10 +9302,10 @@
         <v>766</v>
       </c>
       <c r="C17" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -9319,10 +9321,10 @@
         <v>766</v>
       </c>
       <c r="C18" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -9357,7 +9359,7 @@
         <v>766</v>
       </c>
       <c r="C20" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
newChat improvments including taste test
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB393DB-9CF3-4554-9EFF-6E5F9F41CC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91FBD22-86B4-4C77-965C-E82FF7E1BC38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="1024">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="1026">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3236,32 +3236,6 @@
     <t>חישוב התאמה</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">מורכב מממוצע התכונות: אינטלגנציה אינטואיטיבית, מודעות עצמית, אינטלגנציה רגשית וערך הפוך לנוירוטיות. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">לוודא.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">לשפר. </t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">ממוצע מרחק אוקלידי. </t>
   </si>
   <si>
@@ -3403,10 +3377,6 @@
 50%- התאמה לפי ציון פרופיל עם התאמה של בהתאם לגבר-אישה. אחרת נשדך גברים שבממוצע יותר רגשיים לנשים שפחות.  תיקון ל4 נקודות לטובת האישה.</t>
   </si>
   <si>
-    <t xml:space="preserve">פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
-להוסיף אולי מידת הסתייגות.. ובכללי לקרוא על הנושא כדי לפתח את זה נכון יותר. </t>
-  </si>
-  <si>
     <t>קטגוריה</t>
   </si>
   <si>
@@ -3757,6 +3727,55 @@
     <t>פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
 פרופיל סופר קריטי. להוציא מפה כל מה שקשור לעמדות. להכניס סגנונות אפשריים - צריך לבנות את זה חכם. אולי בתגיות חופשיות (או לא חופשיות). לחשוב על זה. לצורך הבדיקה של זה אצטרך משתמשים מסגנונות שונים באמת, כרגע האוכלוסייה במערכת שלי די הומוגנית.  צריך אולי גם להיות גורם מפלטר לסגנונות לא קשורים.
 סגנונות אפשריים (לחשוב איך לעשות את זה פוליטיקלי קורקט): ערסים, נורמטיבי, עממי, סחי, קיבוצניק/מושבניק, היפי, סובייטי, גיק, תרבות גבוהה, אליטיסטי, קפליניסט. לחשוב מה עוד ואיך לנסח.</t>
+  </si>
+  <si>
+    <t>אימון על זוגות אמיתיים</t>
+  </si>
+  <si>
+    <t>ייעוץ משפטי וconsents על השירות</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">מורכב מממוצע התכונות: אינטלגנציה אינטואיטיבית, מודעות עצמית, אינטלגנציה רגשית וערך הפוך לנוירוטיות. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">לוודא.   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">לשפר.  לא בטוחה שנוירוטיות קשור כאן. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">פרומפט נפרד לכל התכונות הקשורות.   לשפר בהתאם לצורך.
+להוסיף אולי מידת הסתייגות.. ובכללי לקרוא על הנושא כדי לפתח את זה נכון יותר.   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>לעדכן למה שעשיתי</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4628,7 +4647,7 @@
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="A17" s="14" t="s">
         <v>406</v>
       </c>
       <c r="B17" t="s">
@@ -4671,12 +4690,12 @@
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="A22" s="14" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="A23" s="14" t="s">
         <v>465</v>
       </c>
       <c r="D23" t="s">
@@ -4692,18 +4711,28 @@
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="A25" s="14" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" t="s">
+      <c r="A26" s="14" t="s">
         <v>688</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" t="s">
+      <c r="A27" s="14" t="s">
         <v>689</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="14" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="14" t="s">
+        <v>1023</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -7274,7 +7303,7 @@
   <sheetData>
     <row r="2" spans="2:20">
       <c r="B2" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="R2" t="s">
         <v>829</v>
@@ -7295,7 +7324,7 @@
     </row>
     <row r="5" spans="2:20">
       <c r="B5" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="R5" t="s">
         <v>836</v>
@@ -7585,13 +7614,13 @@
         <v>415</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="86.4">
@@ -7599,13 +7628,13 @@
         <v>876</v>
       </c>
       <c r="B3" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>883</v>
+        <v>1024</v>
       </c>
       <c r="D3" s="61" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="G3" s="14"/>
     </row>
@@ -7614,13 +7643,13 @@
         <v>426</v>
       </c>
       <c r="B4" t="s">
+        <v>889</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>890</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>891</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8">
@@ -7628,13 +7657,13 @@
         <v>693</v>
       </c>
       <c r="B5" t="s">
+        <v>884</v>
+      </c>
+      <c r="C5" t="s">
         <v>885</v>
       </c>
-      <c r="C5" t="s">
-        <v>886</v>
-      </c>
       <c r="D5" s="5" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.8">
@@ -7642,13 +7671,13 @@
         <v>429</v>
       </c>
       <c r="B6" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="D6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2">
@@ -7656,13 +7685,13 @@
         <v>877</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>913</v>
+        <v>1025</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="115.2">
@@ -7670,13 +7699,13 @@
         <v>878</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>894</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>895</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>896</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="144">
@@ -7684,13 +7713,13 @@
         <v>867</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>906</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>907</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>908</v>
-      </c>
       <c r="D9" s="5" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="115.2">
@@ -7698,13 +7727,13 @@
         <v>874</v>
       </c>
       <c r="B10" t="s">
+        <v>898</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>899</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>900</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -7712,10 +7741,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -7723,7 +7752,7 @@
         <v>384</v>
       </c>
       <c r="B12" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>260</v>
@@ -7734,13 +7763,13 @@
         <v>879</v>
       </c>
       <c r="B13" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="158.4">
@@ -7748,36 +7777,36 @@
         <v>438</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="201.6">
       <c r="A18" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="28.8">
       <c r="B19" s="5" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="B20" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="B21" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -7785,7 +7814,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="14" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -7800,17 +7829,17 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="14" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
   </sheetData>
@@ -7831,10 +7860,10 @@
   <sheetData>
     <row r="1" spans="2:16">
       <c r="B1" s="62" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="C1" s="62" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>151</v>
@@ -7843,211 +7872,211 @@
         <v>213</v>
       </c>
       <c r="G1" s="62" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
     </row>
     <row r="2" spans="2:16" ht="28.8">
       <c r="B2" s="63" t="s">
+        <v>914</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>915</v>
+      </c>
+      <c r="D2" s="63" t="s">
         <v>916</v>
-      </c>
-      <c r="C2" s="63" t="s">
-        <v>917</v>
-      </c>
-      <c r="D2" s="63" t="s">
-        <v>918</v>
       </c>
       <c r="E2" s="63">
         <v>4</v>
       </c>
       <c r="G2" s="65" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="3" spans="2:16" ht="28.8">
       <c r="B3" s="63" t="s">
+        <v>917</v>
+      </c>
+      <c r="C3" s="63" t="s">
+        <v>918</v>
+      </c>
+      <c r="D3" s="63" t="s">
         <v>919</v>
       </c>
-      <c r="C3" s="63" t="s">
+      <c r="E3" s="63" t="s">
         <v>920</v>
       </c>
-      <c r="D3" s="63" t="s">
-        <v>921</v>
-      </c>
-      <c r="E3" s="63" t="s">
-        <v>922</v>
-      </c>
       <c r="G3" s="63" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
     </row>
     <row r="4" spans="2:16" ht="28.8">
       <c r="B4" s="63" t="s">
+        <v>921</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>922</v>
+      </c>
+      <c r="D4" s="63" t="s">
         <v>923</v>
       </c>
-      <c r="C4" s="63" t="s">
+      <c r="E4" s="63" t="s">
         <v>924</v>
       </c>
-      <c r="D4" s="63" t="s">
-        <v>925</v>
-      </c>
-      <c r="E4" s="63" t="s">
-        <v>926</v>
-      </c>
       <c r="G4" s="63" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
     <row r="5" spans="2:16" ht="28.8">
       <c r="B5" s="63" t="s">
+        <v>925</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>926</v>
+      </c>
+      <c r="D5" s="63" t="s">
         <v>927</v>
       </c>
-      <c r="C5" s="63" t="s">
-        <v>928</v>
-      </c>
-      <c r="D5" s="63" t="s">
-        <v>929</v>
-      </c>
       <c r="E5" s="63" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="G5" s="63" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
     <row r="6" spans="2:16" ht="57.6">
       <c r="B6" s="63" t="s">
+        <v>928</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>929</v>
+      </c>
+      <c r="D6" s="63" t="s">
         <v>930</v>
       </c>
-      <c r="C6" s="63" t="s">
+      <c r="E6" s="63" t="s">
         <v>931</v>
       </c>
-      <c r="D6" s="63" t="s">
-        <v>932</v>
-      </c>
-      <c r="E6" s="63" t="s">
-        <v>933</v>
-      </c>
       <c r="G6" s="63" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="28.8">
       <c r="B7" s="63" t="s">
+        <v>932</v>
+      </c>
+      <c r="C7" s="63" t="s">
+        <v>933</v>
+      </c>
+      <c r="D7" s="63" t="s">
         <v>934</v>
       </c>
-      <c r="C7" s="63" t="s">
+      <c r="E7" s="63" t="s">
         <v>935</v>
       </c>
-      <c r="D7" s="63" t="s">
-        <v>936</v>
-      </c>
-      <c r="E7" s="63" t="s">
-        <v>937</v>
-      </c>
       <c r="G7" s="63" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="8" spans="2:16" ht="43.2">
       <c r="B8" s="63" t="s">
+        <v>936</v>
+      </c>
+      <c r="C8" s="63" t="s">
+        <v>937</v>
+      </c>
+      <c r="D8" s="63" t="s">
         <v>938</v>
       </c>
-      <c r="C8" s="63" t="s">
+      <c r="E8" s="63" t="s">
         <v>939</v>
       </c>
-      <c r="D8" s="63" t="s">
-        <v>940</v>
-      </c>
-      <c r="E8" s="63" t="s">
-        <v>941</v>
-      </c>
       <c r="G8" s="63" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="43.2">
       <c r="B9" s="63" t="s">
+        <v>940</v>
+      </c>
+      <c r="C9" s="63" t="s">
+        <v>941</v>
+      </c>
+      <c r="D9" s="63" t="s">
         <v>942</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="E9" s="63" t="s">
         <v>943</v>
       </c>
-      <c r="D9" s="63" t="s">
-        <v>944</v>
-      </c>
-      <c r="E9" s="63" t="s">
-        <v>945</v>
-      </c>
       <c r="G9" s="63" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="43.2">
       <c r="B10" s="63" t="s">
+        <v>944</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>945</v>
+      </c>
+      <c r="D10" s="63" t="s">
         <v>946</v>
       </c>
-      <c r="C10" s="63" t="s">
+      <c r="E10" s="63" t="s">
         <v>947</v>
       </c>
-      <c r="D10" s="63" t="s">
-        <v>948</v>
-      </c>
-      <c r="E10" s="63" t="s">
-        <v>949</v>
-      </c>
       <c r="G10" s="63" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="28.8">
       <c r="B11" s="63" t="s">
+        <v>948</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>949</v>
+      </c>
+      <c r="D11" s="63" t="s">
         <v>950</v>
       </c>
-      <c r="C11" s="63" t="s">
-        <v>951</v>
-      </c>
-      <c r="D11" s="63" t="s">
-        <v>952</v>
-      </c>
       <c r="E11" s="63" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="28.8">
       <c r="B12" s="63" t="s">
+        <v>951</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>952</v>
+      </c>
+      <c r="D12" s="63" t="s">
         <v>953</v>
       </c>
-      <c r="C12" s="63" t="s">
+      <c r="E12" s="63" t="s">
         <v>954</v>
-      </c>
-      <c r="D12" s="63" t="s">
-        <v>955</v>
-      </c>
-      <c r="E12" s="63" t="s">
-        <v>956</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="F14" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="G14" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="H14" t="s">
         <v>823</v>
       </c>
       <c r="I14" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="J14" t="s">
         <v>822</v>
       </c>
       <c r="K14" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="L14" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="M14" t="s">
         <v>824</v>
@@ -8056,18 +8085,18 @@
         <v>828</v>
       </c>
       <c r="P14" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" s="64" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="D15">
         <v>80</v>
       </c>
       <c r="E15" s="63" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="F15" s="14">
         <v>78</v>
@@ -8105,10 +8134,10 @@
     </row>
     <row r="16" spans="2:16">
       <c r="C16" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="E16" s="63" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="F16">
         <v>92</v>
@@ -8146,13 +8175,13 @@
     </row>
     <row r="17" spans="3:16">
       <c r="C17" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="D17">
         <v>84</v>
       </c>
       <c r="E17" s="63" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="F17" s="14">
         <v>84</v>
@@ -8190,10 +8219,10 @@
     </row>
     <row r="18" spans="3:16">
       <c r="C18" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="E18" s="63" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="F18">
         <v>52</v>
@@ -8231,10 +8260,10 @@
     </row>
     <row r="19" spans="3:16">
       <c r="C19" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="E19" s="63" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="F19">
         <v>88</v>
@@ -8272,13 +8301,13 @@
     </row>
     <row r="20" spans="3:16">
       <c r="C20" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="D20">
         <v>72</v>
       </c>
       <c r="E20" s="63" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="F20" s="14">
         <v>58</v>
@@ -8316,7 +8345,7 @@
     </row>
     <row r="21" spans="3:16">
       <c r="E21" s="63" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="F21">
         <v>64</v>
@@ -8354,7 +8383,7 @@
     </row>
     <row r="22" spans="3:16">
       <c r="E22" s="63" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="F22">
         <v>38</v>
@@ -8386,79 +8415,79 @@
     </row>
     <row r="24" spans="3:16">
       <c r="E24" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="F24" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25" spans="3:16">
       <c r="E25" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="N25" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="O25" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
     </row>
     <row r="26" spans="3:16">
       <c r="E26" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="N26" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
     </row>
     <row r="27" spans="3:16">
       <c r="E27" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="F27" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="N27" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="28" spans="3:16">
       <c r="E28" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="N28" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
     </row>
     <row r="29" spans="3:16">
       <c r="E29" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="N29" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="30" spans="3:16">
       <c r="E30" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="N30" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
     </row>
     <row r="34" spans="2:2">
       <c r="B34" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="35" spans="2:2">
       <c r="B35" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="36" spans="2:2">
       <c r="B36" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
     </row>
     <row r="37" spans="2:2">
@@ -9264,7 +9293,7 @@
         <v>766</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>765</v>
@@ -9283,10 +9312,10 @@
         <v>766</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -9302,10 +9331,10 @@
         <v>766</v>
       </c>
       <c r="C17" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -9321,10 +9350,10 @@
         <v>766</v>
       </c>
       <c r="C18" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -9359,7 +9388,7 @@
         <v>766</v>
       </c>
       <c r="C20" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
Add Supabase OAuth auth, Tailwind, profile setup, taste test profiles v2
- Auth: Google + Apple OAuth via Supabase (AuthScreen, AuthCallback, ProfileSetup)
- Backend: JWT middleware (auth.ts), /auth/sync endpoint, schema columns
- Frontend: Tailwind CSS setup, Supabase client + API wrapper
- Docs: taste test profiles v2, updated notes
- Cleanup: removed old topic prompt files

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/MatchMe DB.xlsx
+++ b/Docs/MatchMe DB.xlsx
@@ -8,32 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPFX\MatchMe\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91FBD22-86B4-4C77-965C-E82FF7E1BC38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C56084-E553-4CC3-A2F7-05F2B3563458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tasks Guidline" sheetId="12" r:id="rId1"/>
-    <sheet name="Current Tasks" sheetId="16" r:id="rId2"/>
-    <sheet name="Analyzer Tasks" sheetId="17" r:id="rId3"/>
-    <sheet name="פירוט מודל מנתח" sheetId="18" r:id="rId4"/>
-    <sheet name="external traits analyze" sheetId="19" r:id="rId5"/>
-    <sheet name="פרטי משתמש" sheetId="3" r:id="rId6"/>
-    <sheet name="Internal Traits" sheetId="1" r:id="rId7"/>
-    <sheet name="internal traits - Old" sheetId="14" r:id="rId8"/>
-    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId9"/>
-    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId10"/>
-    <sheet name="בניית ציונים" sheetId="9" r:id="rId11"/>
-    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId12"/>
-    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId13"/>
-    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId14"/>
-    <sheet name="טופס הזנה" sheetId="8" r:id="rId15"/>
-    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId16"/>
-    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId17"/>
-    <sheet name="בדיקות" sheetId="13" r:id="rId18"/>
-    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId19"/>
+    <sheet name="MVP Guidline" sheetId="20" r:id="rId1"/>
+    <sheet name="Tasks Guidline" sheetId="12" r:id="rId2"/>
+    <sheet name="Current Tasks" sheetId="16" r:id="rId3"/>
+    <sheet name="Analyzer Tasks" sheetId="17" r:id="rId4"/>
+    <sheet name="פירוט מודל מנתח" sheetId="18" r:id="rId5"/>
+    <sheet name="external traits analyze" sheetId="19" r:id="rId6"/>
+    <sheet name="פרטי משתמש" sheetId="3" r:id="rId7"/>
+    <sheet name="Internal Traits" sheetId="1" r:id="rId8"/>
+    <sheet name="internal traits - Old" sheetId="14" r:id="rId9"/>
+    <sheet name="מאפיינים חיצוניים - כללי" sheetId="5" r:id="rId10"/>
+    <sheet name="משתמש - מאפיינים" sheetId="2" r:id="rId11"/>
+    <sheet name="בניית ציונים" sheetId="9" r:id="rId12"/>
+    <sheet name="אלגוריתם ציון פנימי" sheetId="4" r:id="rId13"/>
+    <sheet name="אלגוריתם ציון חיצוני" sheetId="6" r:id="rId14"/>
+    <sheet name="אלגוריתם שידוכים" sheetId="7" r:id="rId15"/>
+    <sheet name="טופס הזנה" sheetId="8" r:id="rId16"/>
+    <sheet name="טבלאות דאטה" sheetId="11" r:id="rId17"/>
+    <sheet name="שאלות עבור הAI" sheetId="10" r:id="rId18"/>
+    <sheet name="בדיקות" sheetId="13" r:id="rId19"/>
+    <sheet name="שאלות לפי מלווה" sheetId="15" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="1026">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="1065">
   <si>
     <t>סוג חישוב</t>
   </si>
@@ -3776,6 +3778,136 @@
       </rPr>
       <t>לעדכן למה שעשיתי</t>
     </r>
+  </si>
+  <si>
+    <t>כניסה עם אוטנטיקציה</t>
+  </si>
+  <si>
+    <t>צעדים לMVP</t>
+  </si>
+  <si>
+    <t>לעשות יוזר אוטנטיקיישן</t>
+  </si>
+  <si>
+    <t>לאפשר לעצמי לשנות נתוני משתמשים - גם תכונות וגם ציוני התאמה</t>
+  </si>
+  <si>
+    <t>להכניס קונסנט וייעוץ בסיסי עם הילה</t>
+  </si>
+  <si>
+    <t>לאפשר לעצמי לאשר התאמות (ברמת הפוטנציאל הראשוני)</t>
+  </si>
+  <si>
+    <t>לסיים את חווית ההתאמה - שליחת של נוטיפיקציה, אפשרות לדירוג, כרטיס התאמה.</t>
+  </si>
+  <si>
+    <t>לסדר את הצ'אט כך שידע לדבר על ההתאמה ועל מה שקורה אחרי</t>
+  </si>
+  <si>
+    <t>בקאפס והפרדת טסט פרוד</t>
+  </si>
+  <si>
+    <t>דרך הריילווי</t>
+  </si>
+  <si>
+    <t>אוטומציה של הוספה כאפליקציה</t>
+  </si>
+  <si>
+    <t>לעשות UI מוצלח</t>
+  </si>
+  <si>
+    <t>אבטחת מידע - סגירת פינות</t>
+  </si>
+  <si>
+    <t>אפשרות לשיחה אחרי קבלת כרטיס ההתאמה</t>
+  </si>
+  <si>
+    <t>דרך ווטסאפ/הודעות/גם וגם</t>
+  </si>
+  <si>
+    <t>לחשוב על עניין העלויות - אולי לחסום צ'אט בשלב מסוים</t>
+  </si>
+  <si>
+    <t>לחשוב מה אני עושה עם זה שלא יחרוג מדי כל עוד אני לא גובה תשלום</t>
+  </si>
+  <si>
+    <t>האם להישאר עם GPT4o?</t>
+  </si>
+  <si>
+    <t>אולי כדאי לשקול מעבר לג'מיני/גרוק כדי לא להסתבך עם החסימות</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בדיקות </t>
+  </si>
+  <si>
+    <t>צעדי הפצה</t>
+  </si>
+  <si>
+    <t>להתחיל פשוט - 10 משתמשים שאני מכירה שיכולים להגיד לי אם הכול תקין</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ואז - להפיץ אצל חברים וכו'.  </t>
+  </si>
+  <si>
+    <t>אחרי ותוך כדי הMVP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">לשפר את חווית הצ'אט קודם כל </t>
+  </si>
+  <si>
+    <t>לשפר את הניתוח והאלגוריתם שיהיה אוטומטי</t>
+  </si>
+  <si>
+    <t>העלאת תמונות מסודרת כולל קונסנט על ניתוח התמונה</t>
+  </si>
+  <si>
+    <t>עם הסבר שהם לא חייבים אבל..</t>
+  </si>
+  <si>
+    <t>במסך הcandidate matches אני אוכל לשחק עם ציוני ההתאמות. וגם כפתור שבלחיצה יוצר כרטיס התאמה ומחזיר ציון התאמה מהAI שמשתלב בציון הכולל. במסך של הmatched - יהיה לי כפתור שליחה ש: 1. יציג את ההתאמה עם כרטיס ההתאמה במסך של שני המשתמשים. 2. ישלח להם ווטסאפ שאומר שיש להם התאמה.  3. בכרטיס ההתאמה יהיה כפתור "החל בשיחה" שיאפשר שליחת הודעה.  אולי עם אופציה של עבור לשיחה בווטסאפ. (צריך לוודא שיש אישור לזה. אולי אם המשתמש יבקש שיחה בווטסאפ זה בעצם ישלח מהמערכת הודעה לצד השני אם הוא רוצה להתחיל בשיחה ומשם השיחה האמיתית תתחיל)</t>
+  </si>
+  <si>
+    <t>הגבלת קצב בקשות (Rate Limiting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">מסך אדמין - שיהיה פתוח רק למשתמשים שמוגדרים כאדמין. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">או רק לי. אולי לעשות מסך מסודר להרשאות. ושיעבוד שונה בלוקל ובפרוד. אפשר אולי שבכלל לא יעבוד בפרוד.  בלוקאל זה יכול להישאר עם הלינק בלבד. </t>
+  </si>
+  <si>
+    <t>חסימת "זליגת מידע" דרך ה-ID (הגנת ID enumeration).  לבדוק מה עוד צריך ואפשרי כבר עכשיו</t>
+  </si>
+  <si>
+    <t>לוודא שרואים את התפריט, שקל לנווט, לעשות לוג אאוט וכו'. לבדוק באייפון ובאנדרואיד.  אולי לעשות גם לוגו טוב</t>
+  </si>
+  <si>
+    <t>כרגע להכניס קונסנט והסבר במסך הראשי של ההסבר + כשמעלים תמונות.</t>
+  </si>
+  <si>
+    <t>תוך כדי הכול</t>
+  </si>
+  <si>
+    <t>לשלוח לזוגות בסיסיים - עדן וגל, הינדי ואלי, אלכס, דני. אולי גם ללחוץ קצת על הבנות דודות. ולשלוח לזוגות אחרים לצורך הבדיקות</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">בביצוע. להשלים את המשימות שלי. לבדוק אחר כך גם מה קורה עם משתמשים שלא רוצים להתחבר דרך גוגל/אפל ומה קורה עם משתמשים שכבר רשומים (בשתי הוריאציות). לבדוק גם באפל וגם בגלקסי.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">לפני שאני חוזרת לזה - להעתיק לקלוד את הפלט של מה שעשינו. </t>
+    </r>
+  </si>
+  <si>
+    <t>בוצע - לא עובד באנדרואיד</t>
   </si>
 </sst>
 </file>
@@ -3996,7 +4128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4171,6 +4303,7 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4450,299 +4583,178 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38DFD5D3-52D3-4B85-A770-31E2BD7FCBB7}">
-  <dimension ref="A1:D32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECF54B88-E3B9-441A-8257-9C1C5A3ED25F}">
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="4" max="4" width="50.44140625" customWidth="1"/>
+    <col min="1" max="1" width="55.109375" customWidth="1"/>
+    <col min="2" max="2" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="35" t="s">
-        <v>389</v>
-      </c>
-      <c r="B1" s="35" t="s">
-        <v>390</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="35" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+    <row r="1" spans="1:2">
+      <c r="A1" s="14" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="43.2">
       <c r="A2" t="s">
-        <v>392</v>
-      </c>
-      <c r="B2" t="s">
-        <v>393</v>
-      </c>
-      <c r="C2" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>1028</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>392</v>
+        <v>1036</v>
       </c>
       <c r="B3" t="s">
-        <v>395</v>
-      </c>
-      <c r="C3" t="s">
-        <v>402</v>
-      </c>
-      <c r="D3" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>392</v>
+        <v>1034</v>
       </c>
       <c r="B4" t="s">
-        <v>394</v>
-      </c>
-      <c r="C4" t="s">
-        <v>405</v>
-      </c>
-      <c r="D4" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>468</v>
+        <v>1030</v>
       </c>
       <c r="B5" t="s">
-        <v>469</v>
-      </c>
-      <c r="C5" t="s">
-        <v>402</v>
-      </c>
-      <c r="D5" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="28.8">
       <c r="A6" t="s">
-        <v>399</v>
-      </c>
-      <c r="C6" t="s">
-        <v>396</v>
-      </c>
-      <c r="D6" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>1056</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>400</v>
+        <v>1038</v>
       </c>
       <c r="B7" t="s">
-        <v>401</v>
-      </c>
-      <c r="C7" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>400</v>
-      </c>
-      <c r="B8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C8" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>400</v>
-      </c>
-      <c r="B9" t="s">
-        <v>404</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>409</v>
-      </c>
-      <c r="C10" t="s">
-        <v>396</v>
-      </c>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11" spans="1:4">
+        <v>1037</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>406</v>
+        <v>1052</v>
       </c>
       <c r="B11" t="s">
-        <v>407</v>
-      </c>
-      <c r="C11" t="s">
-        <v>402</v>
-      </c>
-      <c r="D11" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>412</v>
-      </c>
-      <c r="B12" t="s">
-        <v>614</v>
-      </c>
-      <c r="C12" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="100.8">
+      <c r="A12" s="5" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>615</v>
+        <v>1039</v>
       </c>
       <c r="B13" t="s">
-        <v>616</v>
-      </c>
-      <c r="C13" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>406</v>
-      </c>
-      <c r="B15" t="s">
-        <v>454</v>
-      </c>
-      <c r="C15" t="s">
-        <v>402</v>
-      </c>
-      <c r="D15" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>406</v>
+        <v>1041</v>
       </c>
       <c r="B16" t="s">
-        <v>456</v>
-      </c>
-      <c r="C16" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="14" t="s">
-        <v>406</v>
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>1043</v>
       </c>
       <c r="B17" t="s">
-        <v>463</v>
-      </c>
-      <c r="D17" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>617</v>
-      </c>
-      <c r="B18" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>406</v>
-      </c>
-      <c r="B19" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>406</v>
-      </c>
-      <c r="B20" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>461</v>
-      </c>
-      <c r="B21" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="14" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
       <c r="A23" s="14" t="s">
-        <v>465</v>
-      </c>
-      <c r="D23" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>466</v>
-      </c>
-      <c r="D24" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="14" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="14" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
       <c r="A27" s="14" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="14" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="14" t="s">
-        <v>1023</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="14" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>620</v>
+        <v>1062</v>
       </c>
     </row>
   </sheetData>
@@ -4751,6 +4763,286 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="23.88671875" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" customWidth="1"/>
+    <col min="9" max="9" width="11.77734375" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" customWidth="1"/>
+    <col min="11" max="11" width="23.5546875" customWidth="1"/>
+    <col min="12" max="12" width="42.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="16" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="41.4">
+      <c r="A2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" t="s">
+        <v>423</v>
+      </c>
+      <c r="F3">
+        <v>90</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s">
+        <v>352</v>
+      </c>
+      <c r="I3" s="19"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" t="s">
+        <v>423</v>
+      </c>
+      <c r="F4">
+        <v>80</v>
+      </c>
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" t="s">
+        <v>351</v>
+      </c>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" ht="28.8">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E5">
+        <v>0.5</v>
+      </c>
+      <c r="F5">
+        <v>90</v>
+      </c>
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" t="s">
+        <v>290</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C6" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" t="s">
+        <v>298</v>
+      </c>
+      <c r="C8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K8" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>289</v>
+      </c>
+      <c r="C9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9">
+        <v>0.3</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>9</v>
+      </c>
+      <c r="K9" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>299</v>
+      </c>
+      <c r="B10" t="s">
+        <v>301</v>
+      </c>
+      <c r="C10" t="s">
+        <v>154</v>
+      </c>
+      <c r="E10">
+        <v>0.4</v>
+      </c>
+      <c r="F10">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>8</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="28.8">
+      <c r="A11" t="s">
+        <v>341</v>
+      </c>
+      <c r="B11" t="s">
+        <v>342</v>
+      </c>
+      <c r="C11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D11" t="s">
+        <v>424</v>
+      </c>
+      <c r="E11">
+        <v>0.5</v>
+      </c>
+      <c r="F11">
+        <v>80</v>
+      </c>
+      <c r="G11" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="L11" t="s">
+        <v>354</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E0B4537-96F8-4545-983B-184D65EBDB8F}">
   <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5047,7 +5339,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31382F6D-1248-4EE3-8D30-0A86E7B5E4BF}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5397,7 +5689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2D5149E-0B86-4D57-8B9A-686514500CE9}">
   <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6012,7 +6304,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487A18-0B10-40C8-BA24-F0DC1678FA48}">
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6297,7 +6589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{032081D0-9A99-4BF0-86DD-30C10F371A76}">
   <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6519,7 +6811,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233E8F68-8BA3-48DC-98C9-B07384CDF822}">
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6681,7 +6973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E73849-9796-44C6-80F8-1CA54A2F64E9}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6831,7 +7123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D465AB7-D7AD-4770-A1DB-A227111CD595}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6876,7 +7168,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC47FA1-3DB6-4F73-94E7-2B8A7BD334E9}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6955,7 +7247,313 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38DFD5D3-52D3-4B85-A770-31E2BD7FCBB7}">
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+    <col min="4" max="4" width="50.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="35" t="s">
+        <v>389</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>390</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>392</v>
+      </c>
+      <c r="B3" t="s">
+        <v>395</v>
+      </c>
+      <c r="C3" t="s">
+        <v>402</v>
+      </c>
+      <c r="D3" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>392</v>
+      </c>
+      <c r="B4" t="s">
+        <v>394</v>
+      </c>
+      <c r="C4" t="s">
+        <v>405</v>
+      </c>
+      <c r="D4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>468</v>
+      </c>
+      <c r="B5" t="s">
+        <v>469</v>
+      </c>
+      <c r="C5" t="s">
+        <v>402</v>
+      </c>
+      <c r="D5" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>399</v>
+      </c>
+      <c r="C6" t="s">
+        <v>396</v>
+      </c>
+      <c r="D6" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>400</v>
+      </c>
+      <c r="B7" t="s">
+        <v>401</v>
+      </c>
+      <c r="C7" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>400</v>
+      </c>
+      <c r="B8" t="s">
+        <v>403</v>
+      </c>
+      <c r="C8" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>400</v>
+      </c>
+      <c r="B9" t="s">
+        <v>404</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>409</v>
+      </c>
+      <c r="C10" t="s">
+        <v>396</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>406</v>
+      </c>
+      <c r="B11" t="s">
+        <v>407</v>
+      </c>
+      <c r="C11" t="s">
+        <v>402</v>
+      </c>
+      <c r="D11" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>412</v>
+      </c>
+      <c r="B12" t="s">
+        <v>614</v>
+      </c>
+      <c r="C12" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>615</v>
+      </c>
+      <c r="B13" t="s">
+        <v>616</v>
+      </c>
+      <c r="C13" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>406</v>
+      </c>
+      <c r="B15" t="s">
+        <v>454</v>
+      </c>
+      <c r="C15" t="s">
+        <v>402</v>
+      </c>
+      <c r="D15" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>406</v>
+      </c>
+      <c r="B16" t="s">
+        <v>456</v>
+      </c>
+      <c r="C16" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="B17" t="s">
+        <v>463</v>
+      </c>
+      <c r="D17" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>617</v>
+      </c>
+      <c r="B18" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>406</v>
+      </c>
+      <c r="B19" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>406</v>
+      </c>
+      <c r="B20" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>461</v>
+      </c>
+      <c r="B21" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="14" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="D23" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>466</v>
+      </c>
+      <c r="D24" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="14" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="14" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="14" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="66" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="14" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="14" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>620</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC7838B-7DDE-48A8-A573-BCAB05D487CE}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7110,7 +7708,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C1EE30-A7E2-4C7A-8C61-FDFDE8F0687C}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7291,7 +7889,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50151C83-D621-46FF-871C-82BDAD5480FD}">
   <dimension ref="B2:T31"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7584,7 +8182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E890832A-DBF2-45FA-8E41-3FB9FF4AFB94}">
   <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -7847,7 +8445,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6DB26E2-2FEB-428C-8A2B-44341C3C4297}">
   <dimension ref="B1:P37"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -8500,7 +9098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1C79E50-A761-4208-AC1F-7EE61CFDD025}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -9021,7 +9619,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N74"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -10327,7 +10925,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE069491-4F9B-48D9-B01E-4A4E77F5C60E}">
   <dimension ref="A1:N136"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -12419,284 +13017,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6089DD-60E7-435A-A2E0-E6886B132143}">
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" customWidth="1"/>
-    <col min="4" max="4" width="23.88671875" customWidth="1"/>
-    <col min="7" max="7" width="10.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" customWidth="1"/>
-    <col min="11" max="11" width="23.5546875" customWidth="1"/>
-    <col min="12" max="12" width="42.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" s="16" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="41.4">
-      <c r="A2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" t="s">
-        <v>303</v>
-      </c>
-      <c r="C3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D3" t="s">
-        <v>423</v>
-      </c>
-      <c r="F3">
-        <v>90</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" t="s">
-        <v>352</v>
-      </c>
-      <c r="I3" s="19"/>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D4" t="s">
-        <v>423</v>
-      </c>
-      <c r="F4">
-        <v>80</v>
-      </c>
-      <c r="G4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" t="s">
-        <v>351</v>
-      </c>
-      <c r="L4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" ht="28.8">
-      <c r="A5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B5" t="s">
-        <v>295</v>
-      </c>
-      <c r="C5" t="s">
-        <v>154</v>
-      </c>
-      <c r="E5">
-        <v>0.5</v>
-      </c>
-      <c r="F5">
-        <v>90</v>
-      </c>
-      <c r="G5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" t="s">
-        <v>290</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" t="s">
-        <v>296</v>
-      </c>
-      <c r="C6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>10</v>
-      </c>
-      <c r="G6" t="s">
-        <v>8</v>
-      </c>
-      <c r="K6" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" t="s">
-        <v>297</v>
-      </c>
-      <c r="C7" t="s">
-        <v>154</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7" t="s">
-        <v>8</v>
-      </c>
-      <c r="K7" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>135</v>
-      </c>
-      <c r="B8" t="s">
-        <v>298</v>
-      </c>
-      <c r="C8" t="s">
-        <v>154</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K8" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>289</v>
-      </c>
-      <c r="C9" t="s">
-        <v>154</v>
-      </c>
-      <c r="E9">
-        <v>0.3</v>
-      </c>
-      <c r="F9">
-        <v>50</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-      <c r="K9" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
-        <v>299</v>
-      </c>
-      <c r="B10" t="s">
-        <v>301</v>
-      </c>
-      <c r="C10" t="s">
-        <v>154</v>
-      </c>
-      <c r="E10">
-        <v>0.4</v>
-      </c>
-      <c r="F10">
-        <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>8</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="28.8">
-      <c r="A11" t="s">
-        <v>341</v>
-      </c>
-      <c r="B11" t="s">
-        <v>342</v>
-      </c>
-      <c r="C11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D11" t="s">
-        <v>424</v>
-      </c>
-      <c r="E11">
-        <v>0.5</v>
-      </c>
-      <c r="F11">
-        <v>80</v>
-      </c>
-      <c r="G11" t="s">
-        <v>9</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="L11" t="s">
-        <v>354</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>